<commit_message>
Module 1 seems to be working
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BDA0AED-B903-44F0-8FB4-FAD2F6570C32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{955041BD-FC14-4984-8036-CC3A335DD234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Проект" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="479">
   <si>
     <t>Параметр</t>
   </si>
@@ -962,15 +962,6 @@
     <t>liq_gamma</t>
   </si>
   <si>
-    <t>pressure_present</t>
-  </si>
-  <si>
-    <t>pres_z_surf</t>
-  </si>
-  <si>
-    <t>pres_z_bot</t>
-  </si>
-  <si>
     <t>pres_gamma</t>
   </si>
   <si>
@@ -1035,10 +1026,6 @@
 тс/м³</t>
   </si>
   <si>
-    <t>Давление
-(да/нет)</t>
-  </si>
-  <si>
     <t>Z поверхн.
 грунта, м</t>
   </si>
@@ -1115,14 +1102,6 @@
     <t>elem_offset_piles</t>
   </si>
   <si>
-    <t>Узлы
-свай 1</t>
-  </si>
-  <si>
-    <t>Эл-ты
-свай 1</t>
-  </si>
-  <si>
     <t>Sochi_PK12</t>
   </si>
   <si>
@@ -1467,6 +1446,104 @@
   </si>
   <si>
     <t>да / нет</t>
+  </si>
+  <si>
+    <t>mct</t>
+  </si>
+  <si>
+    <t>не выдает ошибку, если нет пути</t>
+  </si>
+  <si>
+    <t>o4.mct</t>
+  </si>
+  <si>
+    <t>o4_6.mct</t>
+  </si>
+  <si>
+    <t>не сделан случай, когда по mct считается?</t>
+  </si>
+  <si>
+    <t>Перенос и поворот</t>
+  </si>
+  <si>
+    <t>shift_x</t>
+  </si>
+  <si>
+    <t>shift_y</t>
+  </si>
+  <si>
+    <t>shift_z</t>
+  </si>
+  <si>
+    <t>rotation_angle</t>
+  </si>
+  <si>
+    <t>Перенос по x, м</t>
+  </si>
+  <si>
+    <t>Перенос по y, м</t>
+  </si>
+  <si>
+    <t>Перенос по z, м</t>
+  </si>
+  <si>
+    <t>Угол поворота (положительное направление против часовой стрелки, если смотрим сверху), град</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Узлы
+свай </t>
+  </si>
+  <si>
+    <t>Эл-ты
+свай</t>
+  </si>
+  <si>
+    <t>y_pressure_present</t>
+  </si>
+  <si>
+    <t>y_pres_z_surf</t>
+  </si>
+  <si>
+    <t>y_pres_z_bot</t>
+  </si>
+  <si>
+    <t>z_pressure_present</t>
+  </si>
+  <si>
+    <t>z_pres_z_surf</t>
+  </si>
+  <si>
+    <t>z_pres_z_bot</t>
+  </si>
+  <si>
+    <t>Давление по локальной оси y
+(да/нет)</t>
+  </si>
+  <si>
+    <t>Давление по локальной оси z
+(да/нет)</t>
+  </si>
+  <si>
+    <t>Ширина сечений элементов, м
+для бокового давления грунта</t>
+  </si>
+  <si>
+    <t>Ширина ростверка, м</t>
+  </si>
+  <si>
+    <t>cap_width</t>
+  </si>
+  <si>
+    <t>col_width</t>
+  </si>
+  <si>
+    <t>Ширина стойки, м</t>
+  </si>
+  <si>
+    <t>pile_width</t>
+  </si>
+  <si>
+    <t>Ширина сваи, м</t>
   </si>
 </sst>
 </file>
@@ -1581,7 +1658,7 @@
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1671,6 +1748,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1770,7 +1853,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1843,17 +1926,33 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1861,6 +1960,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1887,6 +1991,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1923,25 +2031,13 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2285,7 +2381,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2321,7 +2417,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="D6" s="22"/>
     </row>
@@ -2363,59 +2459,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="34" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="28" t="s">
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
     </row>
     <row r="2" spans="1:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="28" t="s">
-        <v>332</v>
-      </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="34" t="s">
+      <c r="B2" s="38" t="s">
+        <v>328</v>
+      </c>
+      <c r="C2" s="39"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="29"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="35" t="s">
+      <c r="F2" s="39"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="30"/>
+      <c r="I2" s="40"/>
       <c r="J2" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="28" t="s">
+      <c r="K2" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="L2" s="29"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="35" t="s">
+      <c r="L2" s="39"/>
+      <c r="M2" s="40"/>
+      <c r="N2" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="O2" s="30"/>
+      <c r="O2" s="40"/>
       <c r="P2" s="8" t="s">
         <v>23</v>
       </c>
@@ -2425,13 +2521,13 @@
         <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>25</v>
@@ -2521,24 +2617,24 @@
       </c>
     </row>
     <row r="5" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="33"/>
-      <c r="K5" s="33"/>
-      <c r="L5" s="33"/>
-      <c r="M5" s="33"/>
-      <c r="N5" s="33"/>
-      <c r="O5" s="33"/>
-      <c r="P5" s="33"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
     </row>
     <row r="6" spans="1:16" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
@@ -2697,24 +2793,24 @@
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="26" t="s">
-        <v>329</v>
-      </c>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="27"/>
-      <c r="L9" s="27"/>
-      <c r="M9" s="27"/>
-      <c r="N9" s="27"/>
-      <c r="O9" s="27"/>
-      <c r="P9" s="27"/>
+      <c r="A9" s="33" t="s">
+        <v>325</v>
+      </c>
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="34"/>
+      <c r="K9" s="34"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="34"/>
+      <c r="N9" s="34"/>
+      <c r="O9" s="34"/>
+      <c r="P9" s="34"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
@@ -2822,7 +2918,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B12" s="21">
         <v>49.19</v>
@@ -2877,7 +2973,7 @@
         <v>53</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="132" x14ac:dyDescent="0.25">
@@ -2885,7 +2981,7 @@
         <v>54</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="56.25" x14ac:dyDescent="0.25">
@@ -2951,132 +3047,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:42" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="34" t="s">
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="42" t="s">
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="43"/>
-      <c r="U1" s="43"/>
-      <c r="V1" s="43"/>
-      <c r="W1" s="44"/>
-      <c r="X1" s="28" t="s">
+      <c r="P1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
+      <c r="S1" s="50"/>
+      <c r="T1" s="50"/>
+      <c r="U1" s="50"/>
+      <c r="V1" s="50"/>
+      <c r="W1" s="51"/>
+      <c r="X1" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="29"/>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="29"/>
-      <c r="AC1" s="29"/>
-      <c r="AD1" s="29"/>
-      <c r="AE1" s="29"/>
-      <c r="AF1" s="29"/>
-      <c r="AG1" s="30"/>
-      <c r="AH1" s="39" t="s">
+      <c r="Y1" s="39"/>
+      <c r="Z1" s="39"/>
+      <c r="AA1" s="39"/>
+      <c r="AB1" s="39"/>
+      <c r="AC1" s="39"/>
+      <c r="AD1" s="39"/>
+      <c r="AE1" s="39"/>
+      <c r="AF1" s="39"/>
+      <c r="AG1" s="40"/>
+      <c r="AH1" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="AI1" s="40"/>
-      <c r="AJ1" s="40"/>
-      <c r="AK1" s="40"/>
-      <c r="AL1" s="40"/>
-      <c r="AM1" s="40"/>
-      <c r="AN1" s="40"/>
-      <c r="AO1" s="40"/>
-      <c r="AP1" s="41"/>
+      <c r="AI1" s="47"/>
+      <c r="AJ1" s="47"/>
+      <c r="AK1" s="47"/>
+      <c r="AL1" s="47"/>
+      <c r="AM1" s="47"/>
+      <c r="AN1" s="47"/>
+      <c r="AO1" s="47"/>
+      <c r="AP1" s="48"/>
     </row>
     <row r="2" spans="1:42" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="30"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="40"/>
       <c r="E2" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F2" s="45" t="s">
+      <c r="F2" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="G2" s="46"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="35" t="s">
+      <c r="G2" s="53"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="J2" s="29"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="36" t="s">
+      <c r="J2" s="39"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="M2" s="37"/>
-      <c r="N2" s="38"/>
-      <c r="O2" s="45" t="s">
+      <c r="M2" s="44"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="47"/>
-      <c r="R2" s="35" t="s">
+      <c r="P2" s="53"/>
+      <c r="Q2" s="54"/>
+      <c r="R2" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="S2" s="29"/>
-      <c r="T2" s="30"/>
-      <c r="U2" s="36" t="s">
+      <c r="S2" s="39"/>
+      <c r="T2" s="40"/>
+      <c r="U2" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="V2" s="37"/>
-      <c r="W2" s="38"/>
+      <c r="V2" s="44"/>
+      <c r="W2" s="45"/>
       <c r="X2" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="Y2" s="45" t="s">
+      <c r="Y2" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="Z2" s="46"/>
-      <c r="AA2" s="47"/>
-      <c r="AB2" s="35" t="s">
+      <c r="Z2" s="53"/>
+      <c r="AA2" s="54"/>
+      <c r="AB2" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="AC2" s="29"/>
-      <c r="AD2" s="30"/>
-      <c r="AE2" s="36" t="s">
+      <c r="AC2" s="39"/>
+      <c r="AD2" s="40"/>
+      <c r="AE2" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="AF2" s="37"/>
-      <c r="AG2" s="38"/>
-      <c r="AH2" s="45" t="s">
+      <c r="AF2" s="44"/>
+      <c r="AG2" s="45"/>
+      <c r="AH2" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="AI2" s="46"/>
-      <c r="AJ2" s="47"/>
-      <c r="AK2" s="35" t="s">
+      <c r="AI2" s="53"/>
+      <c r="AJ2" s="54"/>
+      <c r="AK2" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="AL2" s="29"/>
-      <c r="AM2" s="30"/>
-      <c r="AN2" s="36" t="s">
+      <c r="AL2" s="39"/>
+      <c r="AM2" s="40"/>
+      <c r="AN2" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="AO2" s="37"/>
-      <c r="AP2" s="38"/>
+      <c r="AO2" s="44"/>
+      <c r="AP2" s="45"/>
     </row>
     <row r="3" spans="1:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -3836,48 +3932,48 @@
       </c>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="A8" s="61"/>
-      <c r="B8" s="63"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="64"/>
-      <c r="G8" s="65"/>
-      <c r="H8" s="64"/>
-      <c r="I8" s="64"/>
-      <c r="J8" s="65"/>
-      <c r="K8" s="64"/>
-      <c r="L8" s="64"/>
-      <c r="M8" s="65"/>
-      <c r="N8" s="64"/>
-      <c r="O8" s="64"/>
-      <c r="P8" s="65"/>
-      <c r="Q8" s="64"/>
-      <c r="R8" s="64"/>
-      <c r="S8" s="65"/>
-      <c r="T8" s="64"/>
-      <c r="U8" s="64"/>
-      <c r="V8" s="65"/>
-      <c r="W8" s="64"/>
-      <c r="X8" s="62"/>
-      <c r="Y8" s="64"/>
-      <c r="Z8" s="65"/>
-      <c r="AA8" s="64"/>
-      <c r="AB8" s="64"/>
-      <c r="AC8" s="65"/>
-      <c r="AD8" s="64"/>
-      <c r="AE8" s="64"/>
-      <c r="AF8" s="65"/>
-      <c r="AG8" s="64"/>
-      <c r="AH8" s="64"/>
-      <c r="AI8" s="65"/>
-      <c r="AJ8" s="64"/>
-      <c r="AK8" s="64"/>
-      <c r="AL8" s="65"/>
-      <c r="AM8" s="64"/>
-      <c r="AN8" s="64"/>
-      <c r="AO8" s="65"/>
-      <c r="AP8" s="64"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="31"/>
+      <c r="N8" s="30"/>
+      <c r="O8" s="30"/>
+      <c r="P8" s="31"/>
+      <c r="Q8" s="30"/>
+      <c r="R8" s="30"/>
+      <c r="S8" s="31"/>
+      <c r="T8" s="30"/>
+      <c r="U8" s="30"/>
+      <c r="V8" s="31"/>
+      <c r="W8" s="30"/>
+      <c r="X8" s="28"/>
+      <c r="Y8" s="30"/>
+      <c r="Z8" s="31"/>
+      <c r="AA8" s="30"/>
+      <c r="AB8" s="30"/>
+      <c r="AC8" s="31"/>
+      <c r="AD8" s="30"/>
+      <c r="AE8" s="30"/>
+      <c r="AF8" s="31"/>
+      <c r="AG8" s="30"/>
+      <c r="AH8" s="30"/>
+      <c r="AI8" s="31"/>
+      <c r="AJ8" s="30"/>
+      <c r="AK8" s="30"/>
+      <c r="AL8" s="31"/>
+      <c r="AM8" s="30"/>
+      <c r="AN8" s="30"/>
+      <c r="AO8" s="31"/>
+      <c r="AP8" s="30"/>
     </row>
     <row r="9" spans="1:42" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
@@ -3931,120 +4027,126 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:CI14"/>
+  <dimension ref="A1:CM14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="87" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:87" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:91" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>451</v>
-      </c>
-      <c r="B1" s="34" t="s">
+        <v>445</v>
+      </c>
+      <c r="B1" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="51" t="s">
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="60" t="s">
         <v>129</v>
       </c>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
-      <c r="L1" s="52"/>
-      <c r="M1" s="52"/>
-      <c r="N1" s="52"/>
-      <c r="O1" s="52"/>
-      <c r="P1" s="52"/>
-      <c r="Q1" s="52"/>
-      <c r="R1" s="52"/>
-      <c r="S1" s="53"/>
-      <c r="T1" s="35" t="s">
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="61"/>
+      <c r="R1" s="61"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="42" t="s">
         <v>130</v>
       </c>
-      <c r="U1" s="29"/>
-      <c r="V1" s="29"/>
-      <c r="W1" s="29"/>
-      <c r="X1" s="29"/>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="29"/>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="29"/>
-      <c r="AC1" s="30"/>
-      <c r="AD1" s="28" t="s">
+      <c r="U1" s="39"/>
+      <c r="V1" s="39"/>
+      <c r="W1" s="39"/>
+      <c r="X1" s="39"/>
+      <c r="Y1" s="39"/>
+      <c r="Z1" s="39"/>
+      <c r="AA1" s="39"/>
+      <c r="AB1" s="39"/>
+      <c r="AC1" s="40"/>
+      <c r="AD1" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="AE1" s="29"/>
-      <c r="AF1" s="29"/>
-      <c r="AG1" s="29"/>
-      <c r="AH1" s="29"/>
-      <c r="AI1" s="29"/>
-      <c r="AJ1" s="29"/>
-      <c r="AK1" s="29"/>
-      <c r="AL1" s="29"/>
-      <c r="AM1" s="29"/>
-      <c r="AN1" s="29"/>
-      <c r="AO1" s="29"/>
-      <c r="AP1" s="29"/>
-      <c r="AQ1" s="30"/>
-      <c r="AR1" s="48" t="s">
+      <c r="AE1" s="39"/>
+      <c r="AF1" s="39"/>
+      <c r="AG1" s="39"/>
+      <c r="AH1" s="39"/>
+      <c r="AI1" s="39"/>
+      <c r="AJ1" s="39"/>
+      <c r="AK1" s="39"/>
+      <c r="AL1" s="39"/>
+      <c r="AM1" s="39"/>
+      <c r="AN1" s="39"/>
+      <c r="AO1" s="39"/>
+      <c r="AP1" s="39"/>
+      <c r="AQ1" s="40"/>
+      <c r="AR1" s="57" t="s">
         <v>132</v>
       </c>
-      <c r="AS1" s="49"/>
-      <c r="AT1" s="49"/>
-      <c r="AU1" s="49"/>
-      <c r="AV1" s="49"/>
-      <c r="AW1" s="49"/>
-      <c r="AX1" s="49"/>
-      <c r="AY1" s="49"/>
-      <c r="AZ1" s="49"/>
-      <c r="BA1" s="49"/>
-      <c r="BB1" s="49"/>
-      <c r="BC1" s="49"/>
-      <c r="BD1" s="49"/>
-      <c r="BE1" s="49"/>
-      <c r="BF1" s="49"/>
-      <c r="BG1" s="49"/>
-      <c r="BH1" s="49"/>
-      <c r="BI1" s="50"/>
-      <c r="BJ1" s="35" t="s">
+      <c r="AS1" s="58"/>
+      <c r="AT1" s="58"/>
+      <c r="AU1" s="58"/>
+      <c r="AV1" s="58"/>
+      <c r="AW1" s="58"/>
+      <c r="AX1" s="58"/>
+      <c r="AY1" s="58"/>
+      <c r="AZ1" s="58"/>
+      <c r="BA1" s="58"/>
+      <c r="BB1" s="58"/>
+      <c r="BC1" s="58"/>
+      <c r="BD1" s="58"/>
+      <c r="BE1" s="58"/>
+      <c r="BF1" s="58"/>
+      <c r="BG1" s="58"/>
+      <c r="BH1" s="58"/>
+      <c r="BI1" s="59"/>
+      <c r="BJ1" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="BK1" s="29"/>
-      <c r="BL1" s="29"/>
-      <c r="BM1" s="29"/>
-      <c r="BN1" s="29"/>
-      <c r="BO1" s="29"/>
-      <c r="BP1" s="29"/>
-      <c r="BQ1" s="29"/>
-      <c r="BR1" s="29"/>
-      <c r="BS1" s="29"/>
-      <c r="BT1" s="29"/>
-      <c r="BU1" s="29"/>
-      <c r="BV1" s="30"/>
-      <c r="BW1" s="34" t="s">
+      <c r="BK1" s="39"/>
+      <c r="BL1" s="39"/>
+      <c r="BM1" s="39"/>
+      <c r="BN1" s="39"/>
+      <c r="BO1" s="39"/>
+      <c r="BP1" s="39"/>
+      <c r="BQ1" s="39"/>
+      <c r="BR1" s="39"/>
+      <c r="BS1" s="39"/>
+      <c r="BT1" s="39"/>
+      <c r="BU1" s="39"/>
+      <c r="BV1" s="40"/>
+      <c r="BW1" s="41" t="s">
         <v>128</v>
       </c>
-      <c r="BX1" s="29"/>
-      <c r="BY1" s="29"/>
-      <c r="BZ1" s="29"/>
-      <c r="CA1" s="29"/>
-      <c r="CB1" s="29"/>
-      <c r="CC1" s="29"/>
-      <c r="CD1" s="29"/>
-      <c r="CE1" s="29"/>
-      <c r="CF1" s="29"/>
-      <c r="CG1" s="29"/>
-      <c r="CH1" s="29"/>
-      <c r="CI1" s="30"/>
-    </row>
-    <row r="2" spans="1:87" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BX1" s="39"/>
+      <c r="BY1" s="39"/>
+      <c r="BZ1" s="39"/>
+      <c r="CA1" s="39"/>
+      <c r="CB1" s="39"/>
+      <c r="CC1" s="39"/>
+      <c r="CD1" s="39"/>
+      <c r="CE1" s="39"/>
+      <c r="CF1" s="39"/>
+      <c r="CG1" s="39"/>
+      <c r="CH1" s="39"/>
+      <c r="CI1" s="40"/>
+      <c r="CJ1" s="55" t="s">
+        <v>453</v>
+      </c>
+      <c r="CK1" s="56"/>
+      <c r="CL1" s="56"/>
+      <c r="CM1" s="56"/>
+    </row>
+    <row r="2" spans="1:91" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>24</v>
@@ -4095,10 +4197,10 @@
         <v>146</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>147</v>
@@ -4304,10 +4406,22 @@
       <c r="CI2" s="3" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="3" spans="1:87" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CJ2" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="CK2" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="CL2" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="CM2" s="3" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="3" spans="1:91" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>37</v>
@@ -4358,10 +4472,10 @@
         <v>227</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>337</v>
+        <v>462</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>338</v>
+        <v>463</v>
       </c>
       <c r="T3" s="9" t="s">
         <v>228</v>
@@ -4567,16 +4681,28 @@
       <c r="CI3" s="9" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="4" spans="1:87" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CJ3" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="CK3" s="9" t="s">
+        <v>459</v>
+      </c>
+      <c r="CL3" s="9" t="s">
+        <v>460</v>
+      </c>
+      <c r="CM3" s="9" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="4" spans="1:91" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>122</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>266</v>
+        <v>448</v>
       </c>
       <c r="D4" s="21">
         <v>10</v>
@@ -4584,8 +4710,12 @@
       <c r="E4" s="21">
         <v>12</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
+      <c r="F4" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>451</v>
+      </c>
       <c r="H4" s="21">
         <v>1</v>
       </c>
@@ -4766,10 +4896,22 @@
       <c r="CG4" s="10"/>
       <c r="CH4" s="10"/>
       <c r="CI4" s="10"/>
-    </row>
-    <row r="5" spans="1:87" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CJ4" s="21">
+        <v>0</v>
+      </c>
+      <c r="CK4" s="21">
+        <v>0</v>
+      </c>
+      <c r="CL4" s="21">
+        <v>0</v>
+      </c>
+      <c r="CM4" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:91" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>453</v>
+        <v>268</v>
       </c>
       <c r="B5" s="21" t="s">
         <v>52</v>
@@ -4993,63 +5135,82 @@
       <c r="CI5" s="21" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="6" spans="1:87" x14ac:dyDescent="0.25">
+      <c r="CJ5" s="21">
+        <v>0</v>
+      </c>
+      <c r="CK5" s="21">
+        <v>0</v>
+      </c>
+      <c r="CL5" s="21">
+        <v>0</v>
+      </c>
+      <c r="CM5" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:91" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>449</v>
+      </c>
       <c r="AE6" s="19" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="AS6" s="19" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BW6" s="19" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="7" spans="1:87" ht="101.25" x14ac:dyDescent="0.25">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="7" spans="1:91" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="AE7" s="19" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="8" spans="1:87" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>452</v>
+      </c>
+      <c r="BW7" s="19" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="8" spans="1:91" ht="112.5" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="9" spans="1:87" ht="101.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:91" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="10" spans="1:87" ht="90" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:91" ht="90" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="11" spans="1:87" ht="123.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:91" ht="123.75" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="12" spans="1:87" ht="90" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:91" ht="90" x14ac:dyDescent="0.25">
       <c r="B12" s="6" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="13" spans="1:87" ht="101.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:91" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="14" spans="1:87" ht="90" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:91" ht="90" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
         <v>276</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="CJ1:CM1"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="BJ1:BV1"/>
     <mergeCell ref="T1:AC1"/>
@@ -5064,61 +5225,69 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="5" width="14" customWidth="1"/>
-    <col min="6" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="10" width="14" customWidth="1"/>
-    <col min="11" max="12" width="12" customWidth="1"/>
-    <col min="13" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="12" customWidth="1"/>
-    <col min="16" max="16" width="10" customWidth="1"/>
-    <col min="17" max="17" width="12.5703125" customWidth="1"/>
-    <col min="18" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="16" customWidth="1"/>
-    <col min="21" max="21" width="12" customWidth="1"/>
-    <col min="22" max="22" width="14" customWidth="1"/>
+    <col min="6" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="13" width="14" customWidth="1"/>
+    <col min="14" max="15" width="12" customWidth="1"/>
+    <col min="16" max="17" width="14" customWidth="1"/>
+    <col min="18" max="18" width="12" customWidth="1"/>
+    <col min="19" max="22" width="10" customWidth="1"/>
+    <col min="23" max="23" width="12.5703125" customWidth="1"/>
+    <col min="24" max="25" width="14" customWidth="1"/>
+    <col min="26" max="26" width="16" customWidth="1"/>
+    <col min="27" max="27" width="12" customWidth="1"/>
+    <col min="28" max="28" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="66" t="s">
         <v>277</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="35" t="s">
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="49" t="s">
+        <v>472</v>
+      </c>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="42" t="s">
         <v>278</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="34" t="s">
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="69" t="s">
         <v>279</v>
       </c>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="54" t="s">
+      <c r="P1" s="70"/>
+      <c r="Q1" s="70"/>
+      <c r="R1" s="70"/>
+      <c r="S1" s="70"/>
+      <c r="T1" s="70"/>
+      <c r="U1" s="70"/>
+      <c r="V1" s="71"/>
+      <c r="W1" s="63" t="s">
         <v>280</v>
       </c>
-      <c r="R1" s="55"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="58" t="s">
+      <c r="X1" s="64"/>
+      <c r="Y1" s="65"/>
+      <c r="Z1" s="67" t="s">
         <v>281</v>
       </c>
-      <c r="U1" s="59"/>
-      <c r="V1" s="59"/>
-    </row>
-    <row r="2" spans="1:22" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AA1" s="68"/>
+      <c r="AB1" s="68"/>
+    </row>
+    <row r="2" spans="1:28" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>24</v>
       </c>
@@ -5141,273 +5310,346 @@
         <v>287</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="O2" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="V2" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="W2" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="X2" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Y2" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="AA2" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="AB2" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="T2" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="3" spans="1:22" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:28" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>37</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="H3" s="9" t="s">
+        <v>473</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>478</v>
+      </c>
+      <c r="K3" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>308</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="N3" s="9" t="s">
         <v>309</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="O3" s="9" t="s">
+        <v>470</v>
+      </c>
+      <c r="P3" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="Q3" s="9" t="s">
         <v>311</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="R3" s="9" t="s">
+        <v>471</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>310</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="U3" s="9" t="s">
         <v>312</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="V3" s="9" t="s">
         <v>313</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="W3" s="9" t="s">
         <v>314</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="X3" s="9" t="s">
         <v>315</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="Y3" s="9" t="s">
         <v>316</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="Z3" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="AA3" s="9" t="s">
+        <v>312</v>
+      </c>
+      <c r="AB3" s="9" t="s">
         <v>317</v>
       </c>
-      <c r="Q3" s="9" t="s">
-        <v>318</v>
-      </c>
-      <c r="R3" s="9" t="s">
-        <v>319</v>
-      </c>
-      <c r="S3" s="9" t="s">
-        <v>320</v>
-      </c>
-      <c r="T3" s="25" t="s">
-        <v>342</v>
-      </c>
-      <c r="U3" s="9" t="s">
-        <v>316</v>
-      </c>
-      <c r="V3" s="9" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:28" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="66">
+      <c r="B4" s="32">
         <v>1</v>
       </c>
-      <c r="C4" s="66">
+      <c r="C4" s="32">
         <v>1</v>
       </c>
-      <c r="D4" s="66">
+      <c r="D4" s="32">
         <v>1</v>
       </c>
-      <c r="E4" s="66">
+      <c r="E4" s="32">
         <v>1</v>
       </c>
-      <c r="F4" s="66">
+      <c r="F4" s="32">
         <v>1</v>
       </c>
-      <c r="G4" s="66">
+      <c r="G4" s="32">
         <v>1</v>
       </c>
-      <c r="H4" s="66" t="s">
+      <c r="H4" s="32">
+        <v>1</v>
+      </c>
+      <c r="I4" s="32">
+        <v>1</v>
+      </c>
+      <c r="J4" s="32">
+        <v>1</v>
+      </c>
+      <c r="K4" s="32" t="s">
         <v>267</v>
       </c>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
-      <c r="L4" s="66" t="s">
+      <c r="L4" s="32"/>
+      <c r="M4" s="32"/>
+      <c r="N4" s="32"/>
+      <c r="O4" s="32" t="s">
         <v>267</v>
       </c>
-      <c r="M4" s="66">
+      <c r="P4" s="32">
         <v>5</v>
       </c>
-      <c r="N4" s="66">
+      <c r="Q4" s="32">
         <v>0</v>
       </c>
-      <c r="O4" s="66">
+      <c r="R4" s="32" t="s">
+        <v>267</v>
+      </c>
+      <c r="S4" s="32">
+        <v>5</v>
+      </c>
+      <c r="T4" s="32">
+        <v>0</v>
+      </c>
+      <c r="U4" s="32">
         <v>1.8</v>
       </c>
-      <c r="P4" s="66">
+      <c r="V4" s="32">
         <v>30</v>
       </c>
-      <c r="Q4" s="66" t="s">
+      <c r="W4" s="32" t="s">
         <v>267</v>
       </c>
-      <c r="R4" s="66"/>
-      <c r="S4" s="66"/>
-      <c r="T4" s="66" t="s">
+      <c r="X4" s="32"/>
+      <c r="Y4" s="32"/>
+      <c r="Z4" s="32" t="s">
         <v>267</v>
       </c>
-      <c r="U4" s="66"/>
-      <c r="V4" s="66"/>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA4" s="32"/>
+      <c r="AB4" s="32"/>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="66">
+      <c r="B5" s="32">
         <v>1</v>
       </c>
-      <c r="C5" s="66">
+      <c r="C5" s="32">
         <v>1</v>
       </c>
-      <c r="D5" s="66">
+      <c r="D5" s="32">
         <v>1</v>
       </c>
-      <c r="E5" s="66">
+      <c r="E5" s="32">
         <v>1</v>
       </c>
-      <c r="F5" s="66">
+      <c r="F5" s="32">
         <v>1</v>
       </c>
-      <c r="G5" s="66">
+      <c r="G5" s="32">
         <v>1</v>
       </c>
-      <c r="H5" s="66" t="s">
+      <c r="H5" s="32">
+        <v>1</v>
+      </c>
+      <c r="I5" s="32">
+        <v>1</v>
+      </c>
+      <c r="J5" s="32">
+        <v>1</v>
+      </c>
+      <c r="K5" s="32" t="s">
         <v>268</v>
       </c>
-      <c r="I5" s="66">
+      <c r="L5" s="32">
         <v>4</v>
       </c>
-      <c r="J5" s="66">
+      <c r="M5" s="32">
         <v>0</v>
       </c>
-      <c r="K5" s="66">
+      <c r="N5" s="32">
         <v>2</v>
       </c>
-      <c r="L5" s="66" t="s">
+      <c r="O5" s="32" t="s">
         <v>268</v>
       </c>
-      <c r="M5" s="66">
+      <c r="P5" s="32">
         <v>5</v>
       </c>
-      <c r="N5" s="66">
+      <c r="Q5" s="32">
         <v>0</v>
       </c>
-      <c r="O5" s="66">
+      <c r="R5" s="32" t="s">
+        <v>268</v>
+      </c>
+      <c r="S5" s="32">
+        <v>5</v>
+      </c>
+      <c r="T5" s="32">
+        <v>0</v>
+      </c>
+      <c r="U5" s="32">
         <v>1.8</v>
       </c>
-      <c r="P5" s="66">
+      <c r="V5" s="32">
         <v>30</v>
       </c>
-      <c r="Q5" s="66" t="s">
+      <c r="W5" s="32" t="s">
         <v>268</v>
       </c>
-      <c r="R5" s="66">
+      <c r="X5" s="32">
         <v>5</v>
       </c>
-      <c r="S5" s="66">
+      <c r="Y5" s="32">
         <v>4</v>
       </c>
-      <c r="T5" s="66" t="s">
+      <c r="Z5" s="32" t="s">
         <v>268</v>
       </c>
-      <c r="U5" s="66">
+      <c r="AA5" s="32">
         <v>2</v>
       </c>
-      <c r="V5" s="66">
+      <c r="AB5" s="32">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="112.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" ht="123.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="7" spans="1:22" ht="112.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22" ht="123.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22" ht="90" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" ht="112.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>326</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="Q1:S1"/>
+  <mergeCells count="6">
+    <mergeCell ref="W1:Y1"/>
     <mergeCell ref="B1:G1"/>
-    <mergeCell ref="H1:K1"/>
-    <mergeCell ref="L1:P1"/>
-    <mergeCell ref="T1:V1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="Z1:AB1"/>
+    <mergeCell ref="O1:V1"/>
+    <mergeCell ref="H1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5423,7 +5665,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5431,32 +5673,32 @@
     </row>
     <row r="3" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5464,22 +5706,22 @@
     </row>
     <row r="10" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5487,27 +5729,27 @@
     </row>
     <row r="15" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5515,52 +5757,52 @@
     </row>
     <row r="21" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="60" t="s">
-        <v>362</v>
+      <c r="A26" s="26" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>365</v>
+        <v>359</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
@@ -5568,92 +5810,92 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
@@ -5661,92 +5903,92 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
@@ -5754,112 +5996,112 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="14" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="14" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="14" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="14" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="14" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="14" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="14" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="14" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="14" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="14" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="14" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="14" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="14" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
@@ -5867,87 +6109,87 @@
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="14" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="14" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="14" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="14" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="14" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="14" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="14" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="14" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="14" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="14" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="14" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
@@ -5955,27 +6197,27 @@
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="15" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Module 2 part 1
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E762FA-CF66-4525-85EB-F2F2D711248C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C5AD42-245A-4D83-9475-541BB99E6369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="479">
   <si>
     <t>Параметр</t>
   </si>
@@ -1452,6 +1452,9 @@
   </si>
   <si>
     <t>не выдает ошибку, если нет пути</t>
+  </si>
+  <si>
+    <t>o4.mct</t>
   </si>
   <si>
     <t>o4_6.mct</t>
@@ -4135,7 +4138,7 @@
       <c r="CH1" s="39"/>
       <c r="CI1" s="40"/>
       <c r="CJ1" s="55" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="CK1" s="56"/>
       <c r="CL1" s="56"/>
@@ -4404,16 +4407,16 @@
         <v>214</v>
       </c>
       <c r="CJ2" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="CK2" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="CL2" s="3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="CM2" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="3" spans="1:91" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -4469,10 +4472,10 @@
         <v>227</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="T3" s="9" t="s">
         <v>228</v>
@@ -4679,21 +4682,21 @@
         <v>265</v>
       </c>
       <c r="CJ3" s="9" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="CK3" s="9" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="CL3" s="9" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="CM3" s="9" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="4" spans="1:91" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>122</v>
@@ -4707,9 +4710,11 @@
       <c r="E4" s="21">
         <v>12</v>
       </c>
-      <c r="F4" s="10"/>
+      <c r="F4" s="10" t="s">
+        <v>450</v>
+      </c>
       <c r="G4" s="10" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H4" s="21">
         <v>1</v>
@@ -4768,7 +4773,7 @@
       </c>
       <c r="AC4" s="24"/>
       <c r="AD4" s="21">
-        <v>10.41</v>
+        <v>15.41</v>
       </c>
       <c r="AE4" s="21">
         <v>0.5</v>
@@ -4796,7 +4801,7 @@
       </c>
       <c r="AQ4" s="24"/>
       <c r="AR4" s="21">
-        <v>11.51</v>
+        <v>16.510000000000002</v>
       </c>
       <c r="AS4" s="21">
         <v>0.4</v>
@@ -4812,7 +4817,7 @@
       </c>
       <c r="AW4" s="24"/>
       <c r="AX4" s="24">
-        <v>10.81</v>
+        <v>15.81</v>
       </c>
       <c r="AY4" s="24">
         <v>3</v>
@@ -4822,7 +4827,7 @@
       </c>
       <c r="BA4" s="24"/>
       <c r="BB4" s="24">
-        <v>11.21</v>
+        <v>16.21</v>
       </c>
       <c r="BC4" s="24">
         <v>5</v>
@@ -4845,7 +4850,7 @@
       </c>
       <c r="BL4" s="5">
         <f>AR4</f>
-        <v>11.51</v>
+        <v>16.510000000000002</v>
       </c>
       <c r="BM4" s="21">
         <v>11.88</v>
@@ -4979,7 +4984,7 @@
       </c>
       <c r="AC5" s="24"/>
       <c r="AD5" s="21">
-        <v>10.41</v>
+        <v>15.41</v>
       </c>
       <c r="AE5" s="21">
         <v>0.5</v>
@@ -5007,7 +5012,7 @@
       </c>
       <c r="AQ5" s="24"/>
       <c r="AR5" s="21">
-        <v>11.51</v>
+        <v>16.510000000000002</v>
       </c>
       <c r="AS5" s="21">
         <v>0.4</v>
@@ -5023,7 +5028,7 @@
       </c>
       <c r="AW5" s="24"/>
       <c r="AX5" s="24">
-        <v>10.81</v>
+        <v>15.81</v>
       </c>
       <c r="AY5" s="24">
         <v>3</v>
@@ -5033,7 +5038,7 @@
       </c>
       <c r="BA5" s="24"/>
       <c r="BB5" s="24">
-        <v>11.21</v>
+        <v>16.21</v>
       </c>
       <c r="BC5" s="24">
         <v>5</v>
@@ -5056,7 +5061,7 @@
       </c>
       <c r="BL5" s="5">
         <f>AR5</f>
-        <v>11.51</v>
+        <v>16.510000000000002</v>
       </c>
       <c r="BM5" s="21">
         <v>11.88</v>
@@ -5097,7 +5102,7 @@
       </c>
       <c r="BY5" s="5">
         <f>AR5</f>
-        <v>11.51</v>
+        <v>16.510000000000002</v>
       </c>
       <c r="BZ5" s="21">
         <v>11.88</v>
@@ -5162,7 +5167,7 @@
         <v>269</v>
       </c>
       <c r="F7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="BW7" s="19" t="s">
         <v>441</v>
@@ -5251,7 +5256,7 @@
       <c r="F1" s="39"/>
       <c r="G1" s="39"/>
       <c r="H1" s="52" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="I1" s="53"/>
       <c r="J1" s="53"/>
@@ -5305,13 +5310,13 @@
         <v>287</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>288</v>
@@ -5326,22 +5331,22 @@
         <v>291</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="U2" s="3" t="s">
         <v>292</v>
@@ -5391,13 +5396,13 @@
         <v>305</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K3" s="9" t="s">
         <v>306</v>
@@ -5412,7 +5417,7 @@
         <v>309</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="P3" s="9" t="s">
         <v>310</v>
@@ -5421,7 +5426,7 @@
         <v>311</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="S3" s="9" t="s">
         <v>310</v>

</xml_diff>

<commit_message>
Module 2 part 2 (frames)
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C5AD42-245A-4D83-9475-541BB99E6369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D2C800-725C-4260-950B-ABB62932491B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Проект" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="482">
   <si>
     <t>Параметр</t>
   </si>
@@ -616,9 +616,6 @@
     <t>f1_x</t>
   </si>
   <si>
-    <t>f1_pad_y</t>
-  </si>
-  <si>
     <t>f1_pad_z_bot</t>
   </si>
   <si>
@@ -653,9 +650,6 @@
   </si>
   <si>
     <t>f2_x</t>
-  </si>
-  <si>
-    <t>f2_pad_y</t>
   </si>
   <si>
     <t>f2_pad_z_bot</t>
@@ -818,10 +812,6 @@
     <t>X рамки 1, м</t>
   </si>
   <si>
-    <t>Y подф.
-(одна сторона), м</t>
-  </si>
-  <si>
     <t>Z низа подф.
 (= верх ригеля)</t>
   </si>
@@ -1084,9 +1074,6 @@
     <t>O5</t>
   </si>
   <si>
-    <t>Подумать, как сделать, чтобы адекватно разбивал</t>
-  </si>
-  <si>
     <t>Отметки Z ОЧ СПРАВА по ходу возрастания пикетажа, м</t>
   </si>
   <si>
@@ -1544,6 +1531,27 @@
   </si>
   <si>
     <t>Ширина сваи, м</t>
+  </si>
+  <si>
+    <t>Может быть не симметрично</t>
+  </si>
+  <si>
+    <t>f1_r_pad_y</t>
+  </si>
+  <si>
+    <t>f1_l_pad_y</t>
+  </si>
+  <si>
+    <t>Y левого подф., м</t>
+  </si>
+  <si>
+    <t>Y правого подф., м</t>
+  </si>
+  <si>
+    <t>f2_r_pad_y</t>
+  </si>
+  <si>
+    <t>f2_l_pad_y</t>
   </si>
 </sst>
 </file>
@@ -1553,7 +1561,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1656,6 +1664,13 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="19">
@@ -1853,7 +1868,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1971,11 +1986,6 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1991,6 +2001,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2040,6 +2055,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -2381,7 +2397,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2417,7 +2433,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="D6" s="22"/>
     </row>
@@ -2487,7 +2503,7 @@
         <v>20</v>
       </c>
       <c r="B2" s="38" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="C2" s="39"/>
       <c r="D2" s="40"/>
@@ -2521,13 +2537,13 @@
         <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>25</v>
@@ -2776,7 +2792,7 @@
         <v>2</v>
       </c>
       <c r="L8" s="21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M8" s="21" t="s">
         <v>49</v>
@@ -2794,7 +2810,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B9" s="34"/>
       <c r="C9" s="34"/>
@@ -2817,13 +2833,13 @@
         <v>52</v>
       </c>
       <c r="B10" s="21">
-        <v>49.19</v>
+        <v>12.18</v>
       </c>
       <c r="C10" s="21">
-        <v>51.45</v>
+        <v>14.23</v>
       </c>
       <c r="D10" s="21">
-        <v>53.45</v>
+        <v>15.5</v>
       </c>
       <c r="E10" s="21">
         <v>3</v>
@@ -2918,7 +2934,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="B12" s="21">
         <v>49.19</v>
@@ -2973,7 +2989,7 @@
         <v>53</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="132" x14ac:dyDescent="0.25">
@@ -2981,7 +2997,7 @@
         <v>54</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="56.25" x14ac:dyDescent="0.25">
@@ -3065,17 +3081,17 @@
       <c r="L1" s="39"/>
       <c r="M1" s="39"/>
       <c r="N1" s="40"/>
-      <c r="O1" s="52" t="s">
+      <c r="O1" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="P1" s="53"/>
-      <c r="Q1" s="53"/>
-      <c r="R1" s="53"/>
-      <c r="S1" s="53"/>
-      <c r="T1" s="53"/>
-      <c r="U1" s="53"/>
-      <c r="V1" s="53"/>
-      <c r="W1" s="54"/>
+      <c r="P1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
+      <c r="S1" s="50"/>
+      <c r="T1" s="50"/>
+      <c r="U1" s="50"/>
+      <c r="V1" s="50"/>
+      <c r="W1" s="51"/>
       <c r="X1" s="38" t="s">
         <v>58</v>
       </c>
@@ -3088,17 +3104,17 @@
       <c r="AE1" s="39"/>
       <c r="AF1" s="39"/>
       <c r="AG1" s="40"/>
-      <c r="AH1" s="49" t="s">
+      <c r="AH1" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="AI1" s="50"/>
-      <c r="AJ1" s="50"/>
-      <c r="AK1" s="50"/>
-      <c r="AL1" s="50"/>
-      <c r="AM1" s="50"/>
-      <c r="AN1" s="50"/>
-      <c r="AO1" s="50"/>
-      <c r="AP1" s="51"/>
+      <c r="AI1" s="47"/>
+      <c r="AJ1" s="47"/>
+      <c r="AK1" s="47"/>
+      <c r="AL1" s="47"/>
+      <c r="AM1" s="47"/>
+      <c r="AN1" s="47"/>
+      <c r="AO1" s="47"/>
+      <c r="AP1" s="48"/>
     </row>
     <row r="2" spans="1:42" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
@@ -3110,69 +3126,69 @@
       <c r="E2" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F2" s="43" t="s">
+      <c r="F2" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="G2" s="44"/>
-      <c r="H2" s="45"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="54"/>
       <c r="I2" s="42" t="s">
         <v>63</v>
       </c>
       <c r="J2" s="39"/>
       <c r="K2" s="40"/>
-      <c r="L2" s="46" t="s">
+      <c r="L2" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="M2" s="47"/>
-      <c r="N2" s="48"/>
-      <c r="O2" s="43" t="s">
+      <c r="M2" s="44"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="P2" s="44"/>
-      <c r="Q2" s="45"/>
+      <c r="P2" s="53"/>
+      <c r="Q2" s="54"/>
       <c r="R2" s="42" t="s">
         <v>66</v>
       </c>
       <c r="S2" s="39"/>
       <c r="T2" s="40"/>
-      <c r="U2" s="46" t="s">
+      <c r="U2" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="V2" s="47"/>
-      <c r="W2" s="48"/>
+      <c r="V2" s="44"/>
+      <c r="W2" s="45"/>
       <c r="X2" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="Y2" s="43" t="s">
+      <c r="Y2" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="Z2" s="44"/>
-      <c r="AA2" s="45"/>
+      <c r="Z2" s="53"/>
+      <c r="AA2" s="54"/>
       <c r="AB2" s="42" t="s">
         <v>63</v>
       </c>
       <c r="AC2" s="39"/>
       <c r="AD2" s="40"/>
-      <c r="AE2" s="46" t="s">
+      <c r="AE2" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="AF2" s="47"/>
-      <c r="AG2" s="48"/>
-      <c r="AH2" s="43" t="s">
+      <c r="AF2" s="44"/>
+      <c r="AG2" s="45"/>
+      <c r="AH2" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="AI2" s="44"/>
-      <c r="AJ2" s="45"/>
+      <c r="AI2" s="53"/>
+      <c r="AJ2" s="54"/>
       <c r="AK2" s="42" t="s">
         <v>66</v>
       </c>
       <c r="AL2" s="39"/>
       <c r="AM2" s="40"/>
-      <c r="AN2" s="46" t="s">
+      <c r="AN2" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="AO2" s="47"/>
-      <c r="AP2" s="48"/>
+      <c r="AO2" s="44"/>
+      <c r="AP2" s="45"/>
     </row>
     <row r="3" spans="1:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -3693,11 +3709,11 @@
       </c>
       <c r="Y6" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!l"&amp;$C6&amp;":l"&amp;$D6),"fixed",INDIRECT("Плеть!A"&amp;$C6&amp;":A"&amp;$D6),$A6)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C6&amp;":A"&amp;$D6),"&lt;&gt;",INDIRECT("Плеть!n"&amp;$C6&amp;":n"&amp;$D6)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C6&amp;":A"&amp;$D6)=$A6)*INDIRECT("Плеть!n"&amp;$C6&amp;":n"&amp;$D6)*INDIRECT("Плеть!p"&amp;$C6&amp;":p"&amp;$D6)))</f>
-        <v>69.600000000000009</v>
+        <v>2387</v>
       </c>
       <c r="Z6" s="17">
         <f ca="1">Y6/B6</f>
-        <v>7.0976952885988185</v>
+        <v>243.42239445237612</v>
       </c>
       <c r="AA6" s="12">
         <f ca="1">H6</f>
@@ -3729,11 +3745,11 @@
       </c>
       <c r="AH6" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!l"&amp;$C6&amp;":l"&amp;$D6),"fixed",INDIRECT("Плеть!A"&amp;$C6&amp;":A"&amp;$D6),$A6)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C6&amp;":A"&amp;$D6),"&lt;&gt;",INDIRECT("Плеть!o"&amp;$C6&amp;":o"&amp;$D6)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C6&amp;":A"&amp;$D6)=$A6)*INDIRECT("Плеть!o"&amp;$C6&amp;":o"&amp;$D6)*INDIRECT("Плеть!p"&amp;$C6&amp;":p"&amp;$D6)))</f>
-        <v>10.4</v>
+        <v>355</v>
       </c>
       <c r="AI6" s="17">
         <f ca="1">AH6/B6</f>
-        <v>1.0605751580664899</v>
+        <v>36.2023251070773</v>
       </c>
       <c r="AJ6" s="12">
         <f ca="1">Q6</f>
@@ -3792,7 +3808,7 @@
       </c>
       <c r="H7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!b"&amp;$C7&amp;":b"&amp;$D7))</f>
-        <v>49.19</v>
+        <v>12.18</v>
       </c>
       <c r="I7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!h"&amp;$C7&amp;":h"&amp;$D7))</f>
@@ -3804,7 +3820,7 @@
       </c>
       <c r="K7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!c"&amp;$C7&amp;":c"&amp;$D7))</f>
-        <v>51.45</v>
+        <v>14.23</v>
       </c>
       <c r="L7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!h"&amp;$C7&amp;":h"&amp;$D7))</f>
@@ -3816,7 +3832,7 @@
       </c>
       <c r="N7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!c"&amp;$C7&amp;":c"&amp;$D7))</f>
-        <v>51.45</v>
+        <v>14.23</v>
       </c>
       <c r="O7" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!f"&amp;$C7&amp;":f"&amp;$D7),"fixed",INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),$A7)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),"&lt;&gt;",INDIRECT("Плеть!i"&amp;$C7&amp;":i"&amp;$D7)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!i"&amp;$C7&amp;":i"&amp;$D7)*INDIRECT("Плеть!j"&amp;$C7&amp;":j"&amp;$D7)))</f>
@@ -3828,7 +3844,7 @@
       </c>
       <c r="Q7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!b"&amp;$C7&amp;":b"&amp;$D7))</f>
-        <v>49.19</v>
+        <v>12.18</v>
       </c>
       <c r="R7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!i"&amp;$C7&amp;":i"&amp;$D7))</f>
@@ -3840,7 +3856,7 @@
       </c>
       <c r="T7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!d"&amp;$C7&amp;":d"&amp;$D7))</f>
-        <v>53.45</v>
+        <v>15.5</v>
       </c>
       <c r="U7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!i"&amp;$C7&amp;":i"&amp;$D7))</f>
@@ -3852,7 +3868,7 @@
       </c>
       <c r="W7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!d"&amp;$C7&amp;":d"&amp;$D7))</f>
-        <v>53.45</v>
+        <v>15.5</v>
       </c>
       <c r="X7" s="5">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!k"&amp;$C7&amp;":k"&amp;$D7))</f>
@@ -3868,7 +3884,7 @@
       </c>
       <c r="AA7" s="12">
         <f ca="1">H7</f>
-        <v>49.19</v>
+        <v>12.18</v>
       </c>
       <c r="AB7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!n"&amp;$C7&amp;":n"&amp;$D7))</f>
@@ -3880,7 +3896,7 @@
       </c>
       <c r="AD7" s="12">
         <f ca="1">K7</f>
-        <v>51.45</v>
+        <v>14.23</v>
       </c>
       <c r="AE7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!n"&amp;$C7&amp;":n"&amp;$D7))</f>
@@ -3892,7 +3908,7 @@
       </c>
       <c r="AG7" s="12">
         <f ca="1">N7</f>
-        <v>51.45</v>
+        <v>14.23</v>
       </c>
       <c r="AH7" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!l"&amp;$C7&amp;":l"&amp;$D7),"fixed",INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),$A7)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),"&lt;&gt;",INDIRECT("Плеть!o"&amp;$C7&amp;":o"&amp;$D7)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!o"&amp;$C7&amp;":o"&amp;$D7)*INDIRECT("Плеть!p"&amp;$C7&amp;":p"&amp;$D7)))</f>
@@ -3904,7 +3920,7 @@
       </c>
       <c r="AJ7" s="12">
         <f ca="1">Q7</f>
-        <v>49.19</v>
+        <v>12.18</v>
       </c>
       <c r="AK7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!o"&amp;$C7&amp;":o"&amp;$D7))</f>
@@ -3916,7 +3932,7 @@
       </c>
       <c r="AM7" s="12">
         <f ca="1">T7</f>
-        <v>53.45</v>
+        <v>15.5</v>
       </c>
       <c r="AN7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!o"&amp;$C7&amp;":o"&amp;$D7))</f>
@@ -3928,7 +3944,7 @@
       </c>
       <c r="AP7" s="12">
         <f ca="1">W7</f>
-        <v>53.45</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.25">
@@ -4002,6 +4018,14 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="AB2:AD2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="Y2:AA2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="E1:N1"/>
     <mergeCell ref="AE2:AG2"/>
     <mergeCell ref="AH1:AP1"/>
     <mergeCell ref="R2:T2"/>
@@ -4012,14 +4036,6 @@
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="AH2:AJ2"/>
     <mergeCell ref="U2:W2"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="AB2:AD2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="Y2:AA2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="E1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4027,15 +4043,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:CM14"/>
+  <dimension ref="A1:CO14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="87" width="12" customWidth="1"/>
+    <col min="2" max="89" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:91" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:93" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="B1" s="41" t="s">
         <v>20</v>
@@ -4121,11 +4137,11 @@
       <c r="BS1" s="39"/>
       <c r="BT1" s="39"/>
       <c r="BU1" s="39"/>
-      <c r="BV1" s="40"/>
-      <c r="BW1" s="41" t="s">
+      <c r="BV1" s="39"/>
+      <c r="BW1" s="40"/>
+      <c r="BX1" s="41" t="s">
         <v>128</v>
       </c>
-      <c r="BX1" s="39"/>
       <c r="BY1" s="39"/>
       <c r="BZ1" s="39"/>
       <c r="CA1" s="39"/>
@@ -4136,17 +4152,19 @@
       <c r="CF1" s="39"/>
       <c r="CG1" s="39"/>
       <c r="CH1" s="39"/>
-      <c r="CI1" s="40"/>
-      <c r="CJ1" s="55" t="s">
-        <v>453</v>
-      </c>
-      <c r="CK1" s="56"/>
-      <c r="CL1" s="56"/>
+      <c r="CI1" s="39"/>
+      <c r="CJ1" s="39"/>
+      <c r="CK1" s="40"/>
+      <c r="CL1" s="55" t="s">
+        <v>449</v>
+      </c>
       <c r="CM1" s="56"/>
-    </row>
-    <row r="2" spans="1:91" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CN1" s="56"/>
+      <c r="CO1" s="56"/>
+    </row>
+    <row r="2" spans="1:93" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>24</v>
@@ -4197,10 +4215,10 @@
         <v>146</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>147</v>
@@ -4332,102 +4350,108 @@
         <v>189</v>
       </c>
       <c r="BK2" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="BL2" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="BM2" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="BL2" s="3" t="s">
+      <c r="BN2" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="BM2" s="3" t="s">
+      <c r="BO2" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="BN2" s="3" t="s">
+      <c r="BP2" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="BO2" s="3" t="s">
+      <c r="BQ2" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="BP2" s="3" t="s">
+      <c r="BR2" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="BQ2" s="3" t="s">
+      <c r="BS2" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="BR2" s="3" t="s">
+      <c r="BT2" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="BS2" s="3" t="s">
+      <c r="BU2" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="BT2" s="3" t="s">
+      <c r="BV2" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="BU2" s="3" t="s">
+      <c r="BW2" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="BV2" s="3" t="s">
+      <c r="BX2" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="BW2" s="3" t="s">
+      <c r="BY2" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="BZ2" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="CA2" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="BX2" s="3" t="s">
+      <c r="CB2" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="BY2" s="3" t="s">
+      <c r="CC2" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="BZ2" s="3" t="s">
+      <c r="CD2" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="CA2" s="3" t="s">
+      <c r="CE2" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="CB2" s="3" t="s">
+      <c r="CF2" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="CC2" s="3" t="s">
+      <c r="CG2" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="CD2" s="3" t="s">
+      <c r="CH2" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="CE2" s="3" t="s">
+      <c r="CI2" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="CF2" s="3" t="s">
+      <c r="CJ2" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="CG2" s="3" t="s">
+      <c r="CK2" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="CH2" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="CI2" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="CJ2" s="3" t="s">
-        <v>454</v>
-      </c>
-      <c r="CK2" s="3" t="s">
-        <v>455</v>
-      </c>
       <c r="CL2" s="3" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="CM2" s="3" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="3" spans="1:91" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+        <v>451</v>
+      </c>
+      <c r="CN2" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="CO2" s="3" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="3" spans="1:93" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>37</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>107</v>
@@ -4436,273 +4460,279 @@
         <v>108</v>
       </c>
       <c r="F3" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="H3" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="J3" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="N3" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="P3" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="Q3" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="R3" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>459</v>
+      </c>
+      <c r="T3" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="U3" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="R3" s="9" t="s">
-        <v>462</v>
-      </c>
-      <c r="S3" s="9" t="s">
-        <v>463</v>
-      </c>
-      <c r="T3" s="9" t="s">
+      <c r="V3" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="U3" s="9" t="s">
+      <c r="W3" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="V3" s="9" t="s">
+      <c r="X3" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="W3" s="9" t="s">
+      <c r="Y3" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="X3" s="9" t="s">
+      <c r="Z3" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="Y3" s="9" t="s">
+      <c r="AA3" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="Z3" s="9" t="s">
+      <c r="AB3" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="AA3" s="9" t="s">
+      <c r="AC3" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="AB3" s="9" t="s">
+      <c r="AD3" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="AC3" s="9" t="s">
+      <c r="AE3" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="AF3" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="AG3" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="AH3" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="AI3" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="AJ3" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="AK3" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="AL3" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="AM3" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="AN3" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="AD3" s="9" t="s">
+      <c r="AO3" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="AE3" s="9" t="s">
+      <c r="AP3" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="AQ3" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="AR3" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="AS3" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="AT3" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="AU3" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="AF3" s="9" t="s">
+      <c r="AV3" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="AG3" s="9" t="s">
+      <c r="AW3" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="AH3" s="9" t="s">
+      <c r="AX3" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="AI3" s="9" t="s">
+      <c r="AY3" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="AJ3" s="9" t="s">
+      <c r="AZ3" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="AK3" s="9" t="s">
+      <c r="BA3" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="AL3" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="AM3" s="9" t="s">
+      <c r="BB3" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="AN3" s="9" t="s">
+      <c r="BC3" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="BD3" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="AO3" s="9" t="s">
+      <c r="BE3" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="AP3" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="AQ3" s="9" t="s">
+      <c r="BF3" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="AR3" s="9" t="s">
+      <c r="BG3" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="AS3" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="AT3" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="AU3" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="AV3" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="AW3" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="AX3" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="AY3" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="AZ3" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="BA3" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="BB3" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="BC3" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="BD3" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="BE3" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="BF3" s="9" t="s">
+      <c r="BH3" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="BG3" s="9" t="s">
+      <c r="BI3" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="BH3" s="9" t="s">
+      <c r="BJ3" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="BI3" s="9" t="s">
+      <c r="BK3" s="9" t="s">
+        <v>479</v>
+      </c>
+      <c r="BL3" s="9" t="s">
+        <v>478</v>
+      </c>
+      <c r="BM3" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="BJ3" s="9" t="s">
+      <c r="BN3" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="BK3" s="9" t="s">
+      <c r="BO3" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="BL3" s="9" t="s">
+      <c r="BP3" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="BM3" s="9" t="s">
+      <c r="BQ3" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="BN3" s="9" t="s">
+      <c r="BR3" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="BO3" s="9" t="s">
+      <c r="BS3" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="BP3" s="9" t="s">
+      <c r="BT3" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="BQ3" s="9" t="s">
+      <c r="BU3" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="BR3" s="9" t="s">
+      <c r="BV3" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="BS3" s="9" t="s">
+      <c r="BW3" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="BT3" s="9" t="s">
+      <c r="BX3" s="9" t="s">
         <v>258</v>
       </c>
-      <c r="BU3" s="9" t="s">
+      <c r="BY3" s="9" t="s">
+        <v>479</v>
+      </c>
+      <c r="BZ3" s="9" t="s">
+        <v>478</v>
+      </c>
+      <c r="CA3" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="BV3" s="9" t="s">
+      <c r="CB3" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="BW3" s="9" t="s">
+      <c r="CC3" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="CD3" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="CE3" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="BX3" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="BY3" s="9" t="s">
+      <c r="CF3" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="CG3" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="CH3" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="CI3" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="CJ3" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="CK3" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="BZ3" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="CA3" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="CB3" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="CC3" s="9" t="s">
+      <c r="CL3" s="9" t="s">
+        <v>454</v>
+      </c>
+      <c r="CM3" s="9" t="s">
+        <v>455</v>
+      </c>
+      <c r="CN3" s="9" t="s">
+        <v>456</v>
+      </c>
+      <c r="CO3" s="9" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="4" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>264</v>
-      </c>
-      <c r="CD3" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="CE3" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="CF3" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="CG3" s="9" t="s">
-        <v>258</v>
-      </c>
-      <c r="CH3" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="CI3" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="CJ3" s="9" t="s">
-        <v>458</v>
-      </c>
-      <c r="CK3" s="9" t="s">
-        <v>459</v>
-      </c>
-      <c r="CL3" s="9" t="s">
-        <v>460</v>
-      </c>
-      <c r="CM3" s="9" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="4" spans="1:91" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>267</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>122</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="D4" s="21">
         <v>10</v>
@@ -4711,10 +4741,10 @@
         <v>12</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="H4" s="21">
         <v>1</v>
@@ -4761,7 +4791,7 @@
         <v>6</v>
       </c>
       <c r="X4" s="24" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="Y4" s="24">
         <v>1</v>
@@ -4769,11 +4799,11 @@
       <c r="Z4" s="24"/>
       <c r="AA4" s="24"/>
       <c r="AB4" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AC4" s="24"/>
       <c r="AD4" s="21">
-        <v>15.41</v>
+        <v>10.01</v>
       </c>
       <c r="AE4" s="21">
         <v>0.5</v>
@@ -4785,23 +4815,23 @@
         <v>1</v>
       </c>
       <c r="AH4" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AI4" s="24"/>
       <c r="AJ4" s="24"/>
       <c r="AK4" s="24"/>
       <c r="AL4" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AM4" s="24"/>
       <c r="AN4" s="24"/>
       <c r="AO4" s="24"/>
       <c r="AP4" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AQ4" s="24"/>
       <c r="AR4" s="21">
-        <v>16.510000000000002</v>
+        <v>11.51</v>
       </c>
       <c r="AS4" s="21">
         <v>0.4</v>
@@ -4813,33 +4843,33 @@
         <v>4</v>
       </c>
       <c r="AV4" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AW4" s="24"/>
       <c r="AX4" s="24">
-        <v>15.81</v>
+        <v>10.81</v>
       </c>
       <c r="AY4" s="24">
         <v>3</v>
       </c>
       <c r="AZ4" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="BA4" s="24"/>
       <c r="BB4" s="24">
-        <v>16.21</v>
+        <v>11.21</v>
       </c>
       <c r="BC4" s="24">
         <v>5</v>
       </c>
       <c r="BD4" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="BE4" s="24"/>
       <c r="BF4" s="24"/>
       <c r="BG4" s="24"/>
       <c r="BH4" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="BI4" s="24"/>
       <c r="BJ4" s="21">
@@ -4848,45 +4878,51 @@
       <c r="BK4" s="21">
         <v>1.9</v>
       </c>
-      <c r="BL4" s="5">
+      <c r="BL4" s="21">
+        <v>2</v>
+      </c>
+      <c r="BM4" s="5">
         <f>AR4</f>
-        <v>16.510000000000002</v>
-      </c>
-      <c r="BM4" s="21">
+        <v>11.51</v>
+      </c>
+      <c r="BN4" s="21">
         <v>11.88</v>
       </c>
-      <c r="BN4" s="21">
+      <c r="BO4" s="21">
         <v>7</v>
       </c>
-      <c r="BO4" s="21">
+      <c r="BP4" s="21">
         <v>1</v>
       </c>
-      <c r="BP4" s="21">
-        <f>BM4</f>
+      <c r="BQ4" s="21">
+        <f>BN4</f>
         <v>11.88</v>
       </c>
-      <c r="BQ4" s="21">
+      <c r="BR4" s="21">
         <v>8</v>
       </c>
-      <c r="BR4" s="21">
+      <c r="BS4" s="21">
         <v>4</v>
       </c>
-      <c r="BS4" s="21">
+      <c r="BT4" s="21">
         <v>11</v>
       </c>
-      <c r="BT4" s="21">
+      <c r="BU4" s="21">
         <v>4</v>
       </c>
-      <c r="BU4" s="21">
+      <c r="BV4" s="21">
         <v>1</v>
       </c>
-      <c r="BV4" s="21" t="s">
-        <v>267</v>
-      </c>
-      <c r="BW4" s="10"/>
+      <c r="BW4" s="21" t="s">
+        <v>264</v>
+      </c>
       <c r="BX4" s="10"/>
-      <c r="BY4" s="10"/>
-      <c r="BZ4" s="10"/>
+      <c r="BY4" s="21">
+        <v>1.9</v>
+      </c>
+      <c r="BZ4" s="21">
+        <v>2</v>
+      </c>
       <c r="CA4" s="10"/>
       <c r="CB4" s="10"/>
       <c r="CC4" s="10"/>
@@ -4896,28 +4932,30 @@
       <c r="CG4" s="10"/>
       <c r="CH4" s="10"/>
       <c r="CI4" s="10"/>
-      <c r="CJ4" s="21">
-        <v>0</v>
-      </c>
-      <c r="CK4" s="21">
-        <v>0</v>
-      </c>
+      <c r="CJ4" s="10"/>
+      <c r="CK4" s="10"/>
       <c r="CL4" s="21">
         <v>0</v>
       </c>
       <c r="CM4" s="21">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:91" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CN4" s="21">
+        <v>0</v>
+      </c>
+      <c r="CO4" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B5" s="21" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D5" s="21">
         <v>10</v>
@@ -4972,7 +5010,7 @@
         <v>6</v>
       </c>
       <c r="X5" s="24" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="Y5" s="24">
         <v>1</v>
@@ -4980,11 +5018,11 @@
       <c r="Z5" s="24"/>
       <c r="AA5" s="24"/>
       <c r="AB5" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AC5" s="24"/>
       <c r="AD5" s="21">
-        <v>15.41</v>
+        <v>10.09</v>
       </c>
       <c r="AE5" s="21">
         <v>0.5</v>
@@ -4996,23 +5034,23 @@
         <v>1</v>
       </c>
       <c r="AH5" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AI5" s="24"/>
       <c r="AJ5" s="24"/>
       <c r="AK5" s="24"/>
       <c r="AL5" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AM5" s="24"/>
       <c r="AN5" s="24"/>
       <c r="AO5" s="24"/>
       <c r="AP5" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AQ5" s="24"/>
       <c r="AR5" s="21">
-        <v>16.510000000000002</v>
+        <v>11.51</v>
       </c>
       <c r="AS5" s="21">
         <v>0.4</v>
@@ -5024,202 +5062,209 @@
         <v>4</v>
       </c>
       <c r="AV5" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AW5" s="24"/>
       <c r="AX5" s="24">
-        <v>15.81</v>
+        <v>10.81</v>
       </c>
       <c r="AY5" s="24">
         <v>3</v>
       </c>
       <c r="AZ5" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="BA5" s="24"/>
       <c r="BB5" s="24">
-        <v>16.21</v>
+        <v>11.21</v>
       </c>
       <c r="BC5" s="24">
         <v>5</v>
       </c>
       <c r="BD5" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="BE5" s="24"/>
       <c r="BF5" s="24"/>
       <c r="BG5" s="24"/>
       <c r="BH5" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="BI5" s="24"/>
       <c r="BJ5" s="21">
         <v>1</v>
       </c>
       <c r="BK5" s="21">
-        <v>1.9</v>
-      </c>
-      <c r="BL5" s="5">
+        <v>1</v>
+      </c>
+      <c r="BL5" s="21">
+        <v>-1.5</v>
+      </c>
+      <c r="BM5" s="5">
         <f>AR5</f>
-        <v>16.510000000000002</v>
-      </c>
-      <c r="BM5" s="21">
+        <v>11.51</v>
+      </c>
+      <c r="BN5" s="21">
         <v>11.88</v>
       </c>
-      <c r="BN5" s="21">
+      <c r="BO5" s="21">
         <v>7</v>
       </c>
-      <c r="BO5" s="21">
+      <c r="BP5" s="21">
         <v>1</v>
       </c>
-      <c r="BP5" s="21">
-        <f>BM5</f>
+      <c r="BQ5" s="21">
+        <f>BN5</f>
         <v>11.88</v>
       </c>
-      <c r="BQ5" s="21">
+      <c r="BR5" s="21">
         <v>8</v>
       </c>
-      <c r="BR5" s="21">
+      <c r="BS5" s="21">
         <v>4</v>
       </c>
-      <c r="BS5" s="21">
+      <c r="BT5" s="21">
         <v>11</v>
       </c>
-      <c r="BT5" s="21">
+      <c r="BU5" s="21">
         <v>4</v>
       </c>
-      <c r="BU5" s="21">
+      <c r="BV5" s="21">
         <v>1</v>
       </c>
-      <c r="BV5" s="21" t="s">
-        <v>267</v>
-      </c>
-      <c r="BW5" s="21">
+      <c r="BW5" s="21" t="s">
+        <v>264</v>
+      </c>
+      <c r="BX5" s="21">
         <v>-1</v>
       </c>
-      <c r="BX5" s="21">
-        <v>1.9</v>
-      </c>
-      <c r="BY5" s="5">
+      <c r="BY5" s="21">
+        <v>2</v>
+      </c>
+      <c r="BZ5" s="21">
+        <v>-2.5</v>
+      </c>
+      <c r="CA5" s="5">
         <f>AR5</f>
-        <v>16.510000000000002</v>
-      </c>
-      <c r="BZ5" s="21">
+        <v>11.51</v>
+      </c>
+      <c r="CB5" s="21">
         <v>11.88</v>
       </c>
-      <c r="CA5" s="21">
-        <v>7</v>
-      </c>
-      <c r="CB5" s="21">
-        <v>1</v>
-      </c>
       <c r="CC5" s="21">
-        <f>BZ5</f>
+        <v>10</v>
+      </c>
+      <c r="CD5" s="21">
+        <v>2</v>
+      </c>
+      <c r="CE5" s="21">
+        <f>CB5</f>
         <v>11.88</v>
       </c>
-      <c r="CD5" s="21">
+      <c r="CF5" s="21">
         <v>8</v>
-      </c>
-      <c r="CE5" s="21">
-        <v>4</v>
-      </c>
-      <c r="CF5" s="21">
-        <v>11</v>
       </c>
       <c r="CG5" s="21">
         <v>4</v>
       </c>
       <c r="CH5" s="21">
-        <v>1</v>
-      </c>
-      <c r="CI5" s="21" t="s">
-        <v>267</v>
+        <v>11</v>
+      </c>
+      <c r="CI5" s="21">
+        <v>4</v>
       </c>
       <c r="CJ5" s="21">
         <v>1</v>
       </c>
-      <c r="CK5" s="21">
+      <c r="CK5" s="21" t="s">
+        <v>264</v>
+      </c>
+      <c r="CL5" s="21">
+        <v>1</v>
+      </c>
+      <c r="CM5" s="21">
         <v>2</v>
       </c>
-      <c r="CL5" s="21">
+      <c r="CN5" s="21">
         <v>0</v>
       </c>
-      <c r="CM5" s="21">
+      <c r="CO5" s="21">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:91" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:93" x14ac:dyDescent="0.25">
       <c r="F6" t="s">
-        <v>449</v>
-      </c>
-      <c r="AE6" s="19" t="s">
-        <v>327</v>
-      </c>
-      <c r="AS6" s="19" t="s">
-        <v>327</v>
-      </c>
-      <c r="BW6" s="19" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="7" spans="1:91" ht="101.25" x14ac:dyDescent="0.25">
+        <v>445</v>
+      </c>
+      <c r="AE6" s="19"/>
+      <c r="AS6" s="19"/>
+      <c r="BX6" s="19" t="s">
+        <v>331</v>
+      </c>
+      <c r="BY6" s="72" t="s">
+        <v>475</v>
+      </c>
+      <c r="BZ6" s="72"/>
+    </row>
+    <row r="7" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="F7" t="s">
+        <v>448</v>
+      </c>
+      <c r="BX7" s="19" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="8" spans="1:93" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="9" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="10" spans="1:93" ht="90" x14ac:dyDescent="0.25">
+      <c r="B10" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="F7" t="s">
-        <v>452</v>
-      </c>
-      <c r="BW7" s="19" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="8" spans="1:91" ht="112.5" x14ac:dyDescent="0.25">
-      <c r="B8" s="6" t="s">
+    </row>
+    <row r="11" spans="1:93" ht="123.75" x14ac:dyDescent="0.25">
+      <c r="B11" s="6" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="9" spans="1:91" ht="101.25" x14ac:dyDescent="0.25">
-      <c r="B9" s="6" t="s">
+    <row r="12" spans="1:93" ht="90" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="10" spans="1:91" ht="90" x14ac:dyDescent="0.25">
-      <c r="B10" s="6" t="s">
+    <row r="13" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
+      <c r="B13" s="6" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="11" spans="1:91" ht="123.75" x14ac:dyDescent="0.25">
-      <c r="B11" s="6" t="s">
+    <row r="14" spans="1:93" ht="90" x14ac:dyDescent="0.25">
+      <c r="B14" s="6" t="s">
         <v>273</v>
-      </c>
-    </row>
-    <row r="12" spans="1:91" ht="90" x14ac:dyDescent="0.25">
-      <c r="B12" s="6" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="13" spans="1:91" ht="101.25" x14ac:dyDescent="0.25">
-      <c r="B13" s="6" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="14" spans="1:91" ht="90" x14ac:dyDescent="0.25">
-      <c r="B14" s="6" t="s">
-        <v>276</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="CJ1:CM1"/>
+    <mergeCell ref="CL1:CO1"/>
     <mergeCell ref="B1:G1"/>
-    <mergeCell ref="BJ1:BV1"/>
+    <mergeCell ref="BJ1:BW1"/>
     <mergeCell ref="T1:AC1"/>
-    <mergeCell ref="BW1:CI1"/>
+    <mergeCell ref="BX1:CK1"/>
     <mergeCell ref="AD1:AQ1"/>
     <mergeCell ref="AR1:BI1"/>
     <mergeCell ref="H1:S1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5248,26 +5293,26 @@
         <v>20</v>
       </c>
       <c r="B1" s="66" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C1" s="39"/>
       <c r="D1" s="39"/>
       <c r="E1" s="39"/>
       <c r="F1" s="39"/>
       <c r="G1" s="39"/>
-      <c r="H1" s="52" t="s">
-        <v>472</v>
-      </c>
-      <c r="I1" s="53"/>
-      <c r="J1" s="53"/>
+      <c r="H1" s="49" t="s">
+        <v>468</v>
+      </c>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
       <c r="K1" s="42" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="L1" s="39"/>
       <c r="M1" s="39"/>
       <c r="N1" s="40"/>
       <c r="O1" s="69" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="P1" s="70"/>
       <c r="Q1" s="70"/>
@@ -5277,12 +5322,12 @@
       <c r="U1" s="70"/>
       <c r="V1" s="71"/>
       <c r="W1" s="63" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="X1" s="64"/>
       <c r="Y1" s="65"/>
       <c r="Z1" s="67" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="AA1" s="68"/>
       <c r="AB1" s="68"/>
@@ -5292,85 +5337,85 @@
         <v>24</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="H2" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>474</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>477</v>
-      </c>
-      <c r="K2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="O2" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="V2" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="W2" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="O2" s="3" t="s">
-        <v>464</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>466</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>467</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>468</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>469</v>
-      </c>
-      <c r="U2" s="3" t="s">
+      <c r="X2" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="V2" s="3" t="s">
+      <c r="Y2" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="W2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="AA2" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="Y2" s="3" t="s">
+      <c r="AB2" s="3" t="s">
         <v>296</v>
-      </c>
-      <c r="Z2" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="AB2" s="3" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="3" spans="1:28" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -5378,85 +5423,85 @@
         <v>37</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>301</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>302</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="H3" s="9" t="s">
+        <v>469</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>472</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="K3" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>473</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>476</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>478</v>
-      </c>
-      <c r="K3" s="9" t="s">
+      <c r="N3" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="O3" s="9" t="s">
+        <v>466</v>
+      </c>
+      <c r="P3" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="Q3" s="9" t="s">
         <v>308</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="R3" s="9" t="s">
+        <v>467</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>308</v>
+      </c>
+      <c r="U3" s="9" t="s">
         <v>309</v>
       </c>
-      <c r="O3" s="9" t="s">
-        <v>470</v>
-      </c>
-      <c r="P3" s="9" t="s">
+      <c r="V3" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="W3" s="9" t="s">
         <v>311</v>
       </c>
-      <c r="R3" s="9" t="s">
-        <v>471</v>
-      </c>
-      <c r="S3" s="9" t="s">
-        <v>310</v>
-      </c>
-      <c r="T3" s="9" t="s">
-        <v>311</v>
-      </c>
-      <c r="U3" s="9" t="s">
+      <c r="X3" s="9" t="s">
         <v>312</v>
       </c>
-      <c r="V3" s="9" t="s">
+      <c r="Y3" s="9" t="s">
         <v>313</v>
       </c>
-      <c r="W3" s="9" t="s">
+      <c r="Z3" s="25" t="s">
+        <v>332</v>
+      </c>
+      <c r="AA3" s="9" t="s">
+        <v>309</v>
+      </c>
+      <c r="AB3" s="9" t="s">
         <v>314</v>
-      </c>
-      <c r="X3" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="Y3" s="9" t="s">
-        <v>316</v>
-      </c>
-      <c r="Z3" s="25" t="s">
-        <v>336</v>
-      </c>
-      <c r="AA3" s="9" t="s">
-        <v>312</v>
-      </c>
-      <c r="AB3" s="9" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="4" spans="1:28" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -5491,13 +5536,13 @@
         <v>1</v>
       </c>
       <c r="K4" s="32" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="L4" s="32"/>
       <c r="M4" s="32"/>
       <c r="N4" s="32"/>
       <c r="O4" s="32" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="P4" s="32">
         <v>5</v>
@@ -5506,7 +5551,7 @@
         <v>0</v>
       </c>
       <c r="R4" s="32" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="S4" s="32">
         <v>5</v>
@@ -5521,12 +5566,12 @@
         <v>30</v>
       </c>
       <c r="W4" s="32" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="X4" s="32"/>
       <c r="Y4" s="32"/>
       <c r="Z4" s="32" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AA4" s="32"/>
       <c r="AB4" s="32"/>
@@ -5563,7 +5608,7 @@
         <v>1</v>
       </c>
       <c r="K5" s="32" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="L5" s="32">
         <v>4</v>
@@ -5575,7 +5620,7 @@
         <v>2</v>
       </c>
       <c r="O5" s="32" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="P5" s="32">
         <v>5</v>
@@ -5584,7 +5629,7 @@
         <v>0</v>
       </c>
       <c r="R5" s="32" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="S5" s="32">
         <v>5</v>
@@ -5599,7 +5644,7 @@
         <v>30</v>
       </c>
       <c r="W5" s="32" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="X5" s="32">
         <v>5</v>
@@ -5608,7 +5653,7 @@
         <v>4</v>
       </c>
       <c r="Z5" s="32" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="AA5" s="32">
         <v>2</v>
@@ -5619,27 +5664,27 @@
     </row>
     <row r="6" spans="1:28" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="7" spans="1:28" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8" spans="1:28" ht="123.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="10" spans="1:28" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>
@@ -5665,7 +5710,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5673,32 +5718,32 @@
     </row>
     <row r="3" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5706,22 +5751,22 @@
     </row>
     <row r="10" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5729,27 +5774,27 @@
     </row>
     <row r="15" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5757,52 +5802,52 @@
     </row>
     <row r="21" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
@@ -5810,92 +5855,92 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
@@ -5903,92 +5948,92 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
@@ -5996,112 +6041,112 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="14" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="14" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="14" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="14" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="14" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="14" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="14" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="14" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="14" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="14" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="14" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="14" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="14" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
@@ -6109,87 +6154,87 @@
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="14" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="14" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="14" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="14" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="14" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="14" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="14" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="14" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="14" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="14" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="14" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
@@ -6197,27 +6242,27 @@
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="15" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Module 2 part 3 (piles anf pier from .mct)
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D2C800-725C-4260-950B-ABB62932491B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89468595-D5BC-4B0D-81E7-A1798F896E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Проект" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="482">
   <si>
     <t>Параметр</t>
   </si>
@@ -1962,6 +1962,7 @@
     <xf numFmtId="0" fontId="8" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1986,6 +1987,11 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2001,11 +2007,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2055,7 +2056,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -2475,59 +2475,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="41" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="38" t="s">
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
-      <c r="P1" s="39"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+      <c r="P1" s="40"/>
     </row>
     <row r="2" spans="1:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="39" t="s">
         <v>324</v>
       </c>
-      <c r="C2" s="39"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="41" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="42" t="s">
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="40"/>
+      <c r="I2" s="41"/>
       <c r="J2" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="38" t="s">
+      <c r="K2" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="L2" s="39"/>
-      <c r="M2" s="40"/>
-      <c r="N2" s="42" t="s">
+      <c r="L2" s="40"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="O2" s="40"/>
+      <c r="O2" s="41"/>
       <c r="P2" s="8" t="s">
         <v>23</v>
       </c>
@@ -2633,24 +2633,24 @@
       </c>
     </row>
     <row r="5" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="37"/>
-      <c r="L5" s="37"/>
-      <c r="M5" s="37"/>
-      <c r="N5" s="37"/>
-      <c r="O5" s="37"/>
-      <c r="P5" s="37"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38"/>
+      <c r="L5" s="38"/>
+      <c r="M5" s="38"/>
+      <c r="N5" s="38"/>
+      <c r="O5" s="38"/>
+      <c r="P5" s="38"/>
     </row>
     <row r="6" spans="1:16" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
@@ -2809,24 +2809,24 @@
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="34" t="s">
         <v>322</v>
       </c>
-      <c r="B9" s="34"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
-      <c r="M9" s="34"/>
-      <c r="N9" s="34"/>
-      <c r="O9" s="34"/>
-      <c r="P9" s="34"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="35"/>
+      <c r="K9" s="35"/>
+      <c r="L9" s="35"/>
+      <c r="M9" s="35"/>
+      <c r="N9" s="35"/>
+      <c r="O9" s="35"/>
+      <c r="P9" s="35"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
@@ -3063,132 +3063,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:42" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="41" t="s">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="49" t="s">
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="P1" s="50"/>
-      <c r="Q1" s="50"/>
-      <c r="R1" s="50"/>
-      <c r="S1" s="50"/>
-      <c r="T1" s="50"/>
-      <c r="U1" s="50"/>
-      <c r="V1" s="50"/>
-      <c r="W1" s="51"/>
-      <c r="X1" s="38" t="s">
+      <c r="P1" s="54"/>
+      <c r="Q1" s="54"/>
+      <c r="R1" s="54"/>
+      <c r="S1" s="54"/>
+      <c r="T1" s="54"/>
+      <c r="U1" s="54"/>
+      <c r="V1" s="54"/>
+      <c r="W1" s="55"/>
+      <c r="X1" s="39" t="s">
         <v>58</v>
       </c>
-      <c r="Y1" s="39"/>
-      <c r="Z1" s="39"/>
-      <c r="AA1" s="39"/>
-      <c r="AB1" s="39"/>
-      <c r="AC1" s="39"/>
-      <c r="AD1" s="39"/>
-      <c r="AE1" s="39"/>
-      <c r="AF1" s="39"/>
-      <c r="AG1" s="40"/>
-      <c r="AH1" s="46" t="s">
+      <c r="Y1" s="40"/>
+      <c r="Z1" s="40"/>
+      <c r="AA1" s="40"/>
+      <c r="AB1" s="40"/>
+      <c r="AC1" s="40"/>
+      <c r="AD1" s="40"/>
+      <c r="AE1" s="40"/>
+      <c r="AF1" s="40"/>
+      <c r="AG1" s="41"/>
+      <c r="AH1" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="AI1" s="47"/>
-      <c r="AJ1" s="47"/>
-      <c r="AK1" s="47"/>
-      <c r="AL1" s="47"/>
-      <c r="AM1" s="47"/>
-      <c r="AN1" s="47"/>
-      <c r="AO1" s="47"/>
-      <c r="AP1" s="48"/>
+      <c r="AI1" s="51"/>
+      <c r="AJ1" s="51"/>
+      <c r="AK1" s="51"/>
+      <c r="AL1" s="51"/>
+      <c r="AM1" s="51"/>
+      <c r="AN1" s="51"/>
+      <c r="AO1" s="51"/>
+      <c r="AP1" s="52"/>
     </row>
     <row r="2" spans="1:42" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="40"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="41"/>
       <c r="E2" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="G2" s="53"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="42" t="s">
+      <c r="G2" s="45"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="J2" s="39"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="43" t="s">
+      <c r="J2" s="40"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="M2" s="44"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="52" t="s">
+      <c r="M2" s="48"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="P2" s="53"/>
-      <c r="Q2" s="54"/>
-      <c r="R2" s="42" t="s">
+      <c r="P2" s="45"/>
+      <c r="Q2" s="46"/>
+      <c r="R2" s="43" t="s">
         <v>66</v>
       </c>
-      <c r="S2" s="39"/>
-      <c r="T2" s="40"/>
-      <c r="U2" s="43" t="s">
+      <c r="S2" s="40"/>
+      <c r="T2" s="41"/>
+      <c r="U2" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="V2" s="44"/>
-      <c r="W2" s="45"/>
+      <c r="V2" s="48"/>
+      <c r="W2" s="49"/>
       <c r="X2" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="Y2" s="52" t="s">
+      <c r="Y2" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="Z2" s="53"/>
-      <c r="AA2" s="54"/>
-      <c r="AB2" s="42" t="s">
+      <c r="Z2" s="45"/>
+      <c r="AA2" s="46"/>
+      <c r="AB2" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="AC2" s="39"/>
-      <c r="AD2" s="40"/>
-      <c r="AE2" s="43" t="s">
+      <c r="AC2" s="40"/>
+      <c r="AD2" s="41"/>
+      <c r="AE2" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="AF2" s="44"/>
-      <c r="AG2" s="45"/>
-      <c r="AH2" s="52" t="s">
+      <c r="AF2" s="48"/>
+      <c r="AG2" s="49"/>
+      <c r="AH2" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="AI2" s="53"/>
-      <c r="AJ2" s="54"/>
-      <c r="AK2" s="42" t="s">
+      <c r="AI2" s="45"/>
+      <c r="AJ2" s="46"/>
+      <c r="AK2" s="43" t="s">
         <v>66</v>
       </c>
-      <c r="AL2" s="39"/>
-      <c r="AM2" s="40"/>
-      <c r="AN2" s="43" t="s">
+      <c r="AL2" s="40"/>
+      <c r="AM2" s="41"/>
+      <c r="AN2" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="AO2" s="44"/>
-      <c r="AP2" s="45"/>
+      <c r="AO2" s="48"/>
+      <c r="AP2" s="49"/>
     </row>
     <row r="3" spans="1:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -4018,14 +4018,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="AB2:AD2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="Y2:AA2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="E1:N1"/>
     <mergeCell ref="AE2:AG2"/>
     <mergeCell ref="AH1:AP1"/>
     <mergeCell ref="R2:T2"/>
@@ -4036,6 +4028,14 @@
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="AH2:AJ2"/>
     <mergeCell ref="U2:W2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="AB2:AD2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="Y2:AA2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="E1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4053,114 +4053,114 @@
       <c r="A1" s="16" t="s">
         <v>441</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="60" t="s">
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="61" t="s">
         <v>129</v>
       </c>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="61"/>
-      <c r="Q1" s="61"/>
-      <c r="R1" s="61"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="42" t="s">
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="63"/>
+      <c r="T1" s="43" t="s">
         <v>130</v>
       </c>
-      <c r="U1" s="39"/>
-      <c r="V1" s="39"/>
-      <c r="W1" s="39"/>
-      <c r="X1" s="39"/>
-      <c r="Y1" s="39"/>
-      <c r="Z1" s="39"/>
-      <c r="AA1" s="39"/>
-      <c r="AB1" s="39"/>
-      <c r="AC1" s="40"/>
-      <c r="AD1" s="38" t="s">
+      <c r="U1" s="40"/>
+      <c r="V1" s="40"/>
+      <c r="W1" s="40"/>
+      <c r="X1" s="40"/>
+      <c r="Y1" s="40"/>
+      <c r="Z1" s="40"/>
+      <c r="AA1" s="40"/>
+      <c r="AB1" s="40"/>
+      <c r="AC1" s="41"/>
+      <c r="AD1" s="39" t="s">
         <v>131</v>
       </c>
-      <c r="AE1" s="39"/>
-      <c r="AF1" s="39"/>
-      <c r="AG1" s="39"/>
-      <c r="AH1" s="39"/>
-      <c r="AI1" s="39"/>
-      <c r="AJ1" s="39"/>
-      <c r="AK1" s="39"/>
-      <c r="AL1" s="39"/>
-      <c r="AM1" s="39"/>
-      <c r="AN1" s="39"/>
-      <c r="AO1" s="39"/>
-      <c r="AP1" s="39"/>
-      <c r="AQ1" s="40"/>
-      <c r="AR1" s="57" t="s">
+      <c r="AE1" s="40"/>
+      <c r="AF1" s="40"/>
+      <c r="AG1" s="40"/>
+      <c r="AH1" s="40"/>
+      <c r="AI1" s="40"/>
+      <c r="AJ1" s="40"/>
+      <c r="AK1" s="40"/>
+      <c r="AL1" s="40"/>
+      <c r="AM1" s="40"/>
+      <c r="AN1" s="40"/>
+      <c r="AO1" s="40"/>
+      <c r="AP1" s="40"/>
+      <c r="AQ1" s="41"/>
+      <c r="AR1" s="58" t="s">
         <v>132</v>
       </c>
-      <c r="AS1" s="58"/>
-      <c r="AT1" s="58"/>
-      <c r="AU1" s="58"/>
-      <c r="AV1" s="58"/>
-      <c r="AW1" s="58"/>
-      <c r="AX1" s="58"/>
-      <c r="AY1" s="58"/>
-      <c r="AZ1" s="58"/>
-      <c r="BA1" s="58"/>
-      <c r="BB1" s="58"/>
-      <c r="BC1" s="58"/>
-      <c r="BD1" s="58"/>
-      <c r="BE1" s="58"/>
-      <c r="BF1" s="58"/>
-      <c r="BG1" s="58"/>
-      <c r="BH1" s="58"/>
-      <c r="BI1" s="59"/>
-      <c r="BJ1" s="42" t="s">
+      <c r="AS1" s="59"/>
+      <c r="AT1" s="59"/>
+      <c r="AU1" s="59"/>
+      <c r="AV1" s="59"/>
+      <c r="AW1" s="59"/>
+      <c r="AX1" s="59"/>
+      <c r="AY1" s="59"/>
+      <c r="AZ1" s="59"/>
+      <c r="BA1" s="59"/>
+      <c r="BB1" s="59"/>
+      <c r="BC1" s="59"/>
+      <c r="BD1" s="59"/>
+      <c r="BE1" s="59"/>
+      <c r="BF1" s="59"/>
+      <c r="BG1" s="59"/>
+      <c r="BH1" s="59"/>
+      <c r="BI1" s="60"/>
+      <c r="BJ1" s="43" t="s">
         <v>133</v>
       </c>
-      <c r="BK1" s="39"/>
-      <c r="BL1" s="39"/>
-      <c r="BM1" s="39"/>
-      <c r="BN1" s="39"/>
-      <c r="BO1" s="39"/>
-      <c r="BP1" s="39"/>
-      <c r="BQ1" s="39"/>
-      <c r="BR1" s="39"/>
-      <c r="BS1" s="39"/>
-      <c r="BT1" s="39"/>
-      <c r="BU1" s="39"/>
-      <c r="BV1" s="39"/>
-      <c r="BW1" s="40"/>
-      <c r="BX1" s="41" t="s">
+      <c r="BK1" s="40"/>
+      <c r="BL1" s="40"/>
+      <c r="BM1" s="40"/>
+      <c r="BN1" s="40"/>
+      <c r="BO1" s="40"/>
+      <c r="BP1" s="40"/>
+      <c r="BQ1" s="40"/>
+      <c r="BR1" s="40"/>
+      <c r="BS1" s="40"/>
+      <c r="BT1" s="40"/>
+      <c r="BU1" s="40"/>
+      <c r="BV1" s="40"/>
+      <c r="BW1" s="41"/>
+      <c r="BX1" s="42" t="s">
         <v>128</v>
       </c>
-      <c r="BY1" s="39"/>
-      <c r="BZ1" s="39"/>
-      <c r="CA1" s="39"/>
-      <c r="CB1" s="39"/>
-      <c r="CC1" s="39"/>
-      <c r="CD1" s="39"/>
-      <c r="CE1" s="39"/>
-      <c r="CF1" s="39"/>
-      <c r="CG1" s="39"/>
-      <c r="CH1" s="39"/>
-      <c r="CI1" s="39"/>
-      <c r="CJ1" s="39"/>
-      <c r="CK1" s="40"/>
-      <c r="CL1" s="55" t="s">
+      <c r="BY1" s="40"/>
+      <c r="BZ1" s="40"/>
+      <c r="CA1" s="40"/>
+      <c r="CB1" s="40"/>
+      <c r="CC1" s="40"/>
+      <c r="CD1" s="40"/>
+      <c r="CE1" s="40"/>
+      <c r="CF1" s="40"/>
+      <c r="CG1" s="40"/>
+      <c r="CH1" s="40"/>
+      <c r="CI1" s="40"/>
+      <c r="CJ1" s="40"/>
+      <c r="CK1" s="41"/>
+      <c r="CL1" s="56" t="s">
         <v>449</v>
       </c>
-      <c r="CM1" s="56"/>
-      <c r="CN1" s="56"/>
-      <c r="CO1" s="56"/>
+      <c r="CM1" s="57"/>
+      <c r="CN1" s="57"/>
+      <c r="CO1" s="57"/>
     </row>
     <row r="2" spans="1:93" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -4894,7 +4894,7 @@
       <c r="BP4" s="21">
         <v>1</v>
       </c>
-      <c r="BQ4" s="21">
+      <c r="BQ4" s="5">
         <f>BN4</f>
         <v>11.88</v>
       </c>
@@ -4964,7 +4964,9 @@
         <v>12</v>
       </c>
       <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
+      <c r="G5" s="10" t="s">
+        <v>447</v>
+      </c>
       <c r="H5" s="21">
         <v>1</v>
       </c>
@@ -4989,8 +4991,12 @@
       <c r="O5" s="21">
         <v>301</v>
       </c>
-      <c r="P5" s="24"/>
-      <c r="Q5" s="24"/>
+      <c r="P5" s="24">
+        <v>401</v>
+      </c>
+      <c r="Q5" s="24">
+        <v>401</v>
+      </c>
       <c r="R5" s="21">
         <v>1001</v>
       </c>
@@ -5113,7 +5119,7 @@
       <c r="BP5" s="21">
         <v>1</v>
       </c>
-      <c r="BQ5" s="21">
+      <c r="BQ5" s="5">
         <f>BN5</f>
         <v>11.88</v>
       </c>
@@ -5201,10 +5207,10 @@
       <c r="BX6" s="19" t="s">
         <v>331</v>
       </c>
-      <c r="BY6" s="72" t="s">
+      <c r="BY6" s="33" t="s">
         <v>475</v>
       </c>
-      <c r="BZ6" s="72"/>
+      <c r="BZ6" s="33"/>
     </row>
     <row r="7" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
@@ -5292,45 +5298,45 @@
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="66" t="s">
+      <c r="B1" s="67" t="s">
         <v>274</v>
       </c>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="49" t="s">
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="53" t="s">
         <v>468</v>
       </c>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="42" t="s">
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="43" t="s">
         <v>275</v>
       </c>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="69" t="s">
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="70" t="s">
         <v>276</v>
       </c>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="R1" s="70"/>
-      <c r="S1" s="70"/>
-      <c r="T1" s="70"/>
-      <c r="U1" s="70"/>
-      <c r="V1" s="71"/>
-      <c r="W1" s="63" t="s">
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="71"/>
+      <c r="U1" s="71"/>
+      <c r="V1" s="72"/>
+      <c r="W1" s="64" t="s">
         <v>277</v>
       </c>
-      <c r="X1" s="64"/>
-      <c r="Y1" s="65"/>
-      <c r="Z1" s="67" t="s">
+      <c r="X1" s="65"/>
+      <c r="Y1" s="66"/>
+      <c r="Z1" s="68" t="s">
         <v>278</v>
       </c>
-      <c r="AA1" s="68"/>
-      <c r="AB1" s="68"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
     </row>
     <row r="2" spans="1:28" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">

</xml_diff>

<commit_message>
Module 4 doesn't work
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0228F3-C564-44AC-9A8B-777C97C0ADBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{303B6709-5801-45C4-920D-474DA76B2707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Проект" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="498">
   <si>
     <t>Параметр</t>
   </si>
@@ -149,10 +149,6 @@
 пролёта, м</t>
   </si>
   <si>
-    <t>Z верха пр.
-части, м</t>
-  </si>
-  <si>
     <t>№ ОЧ
 (1–4)</t>
   </si>
@@ -753,9 +749,6 @@
 зоны 1</t>
   </si>
   <si>
-    <t>№ гр.'ы 1</t>
-  </si>
-  <si>
     <t>Z верха
 зоны 1</t>
   </si>
@@ -768,9 +761,6 @@
 зоны 2</t>
   </si>
   <si>
-    <t>№ гр.'ы 2</t>
-  </si>
-  <si>
     <t>Z верха
 стойки, м</t>
   </si>
@@ -787,9 +777,6 @@
 зоны 3</t>
   </si>
   <si>
-    <t>№ гр.'ы 3</t>
-  </si>
-  <si>
     <t>Z верха
 ригеля, м</t>
   </si>
@@ -806,9 +793,6 @@
 зоны 4</t>
   </si>
   <si>
-    <t>№ гр.'ы 4</t>
-  </si>
-  <si>
     <t>X рамки 1, м</t>
   </si>
   <si>
@@ -922,18 +906,6 @@
 на ростверк</t>
   </si>
   <si>
-    <t>cap_area_top</t>
-  </si>
-  <si>
-    <t>cap_area_bot</t>
-  </si>
-  <si>
-    <t>col_area_top</t>
-  </si>
-  <si>
-    <t>col_area_bot</t>
-  </si>
-  <si>
     <t>pile_area_top</t>
   </si>
   <si>
@@ -974,22 +946,6 @@
   </si>
   <si>
     <t>soil_on_cap_h</t>
-  </si>
-  <si>
-    <t>S ростверка
-вверху, м²</t>
-  </si>
-  <si>
-    <t>S ростверка
-внизу, м²</t>
-  </si>
-  <si>
-    <t>S стойки
-вверху, м²</t>
-  </si>
-  <si>
-    <t>S стойки
-внизу, м²</t>
   </si>
   <si>
     <t>S сваи
@@ -1515,18 +1471,6 @@
 для бокового давления грунта</t>
   </si>
   <si>
-    <t>Ширина ростверка, м</t>
-  </si>
-  <si>
-    <t>cap_width</t>
-  </si>
-  <si>
-    <t>col_width</t>
-  </si>
-  <si>
-    <t>Ширина стойки, м</t>
-  </si>
-  <si>
     <t>pile_width</t>
   </si>
   <si>
@@ -1552,6 +1496,131 @@
   </si>
   <si>
     <t>f2_l_pad_y</t>
+  </si>
+  <si>
+    <t>Z верха проезжей.
+части, м</t>
+  </si>
+  <si>
+    <t>S стойки
+вверху
+(1 зона), м²</t>
+  </si>
+  <si>
+    <t>S стойки
+внизу
+(1 зона), м²</t>
+  </si>
+  <si>
+    <t>cap_area_sec_1_top</t>
+  </si>
+  <si>
+    <t>cap_area_sec_1_bot</t>
+  </si>
+  <si>
+    <t>S ростверка
+вверху
+(1 зона), м²</t>
+  </si>
+  <si>
+    <t>S ростверка
+внизу
+(1 зона), м²</t>
+  </si>
+  <si>
+    <t>cap_area_sec_2_top</t>
+  </si>
+  <si>
+    <t>cap_area_sec_2_bot</t>
+  </si>
+  <si>
+    <t>S ростверка
+внизу
+(2 зона), м²</t>
+  </si>
+  <si>
+    <t>S ростверка
+вверху
+(2 зона), м²</t>
+  </si>
+  <si>
+    <t>S стойки
+вверху
+(3 зона), м²</t>
+  </si>
+  <si>
+    <t>col_area_sec_1_top</t>
+  </si>
+  <si>
+    <t>col_area_sec_1_bot</t>
+  </si>
+  <si>
+    <t>col_area_sec_2_top</t>
+  </si>
+  <si>
+    <t>col_area_sec_2_bot</t>
+  </si>
+  <si>
+    <t>S стойки
+вверху
+(2 зона), м²</t>
+  </si>
+  <si>
+    <t>S стойки
+внизу
+(2 зона), м²</t>
+  </si>
+  <si>
+    <t>S стойки
+внизу
+(3 зона), м²</t>
+  </si>
+  <si>
+    <t>№ группы 1</t>
+  </si>
+  <si>
+    <t>№ группы 2</t>
+  </si>
+  <si>
+    <t>№ группы 3</t>
+  </si>
+  <si>
+    <t>№ группы 4</t>
+  </si>
+  <si>
+    <t>cap_sec_1_width</t>
+  </si>
+  <si>
+    <t>col_sec_1_width</t>
+  </si>
+  <si>
+    <t>col_sec_2_width</t>
+  </si>
+  <si>
+    <t>col_sec_3_width</t>
+  </si>
+  <si>
+    <t>Ширина ростверка
+(1 зона), м</t>
+  </si>
+  <si>
+    <t>Ширина ростверка
+(2 зона), м</t>
+  </si>
+  <si>
+    <t>Ширина стойки
+(1 зона), м</t>
+  </si>
+  <si>
+    <t>Ширина стойки
+(2 зона), м</t>
+  </si>
+  <si>
+    <t>Ширина стойки
+(3 зона), м</t>
+  </si>
+  <si>
+    <t>cap_sec_2_width</t>
   </si>
 </sst>
 </file>
@@ -1868,7 +1937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2054,6 +2123,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2397,7 +2469,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>329</v>
+        <v>316</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2433,7 +2505,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>330</v>
+        <v>317</v>
       </c>
       <c r="D6" s="22"/>
     </row>
@@ -2503,7 +2575,7 @@
         <v>20</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>324</v>
+        <v>311</v>
       </c>
       <c r="C2" s="40"/>
       <c r="D2" s="41"/>
@@ -2537,13 +2609,13 @@
         <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>438</v>
+        <v>425</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>439</v>
+        <v>426</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>440</v>
+        <v>427</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>25</v>
@@ -2593,48 +2665,48 @@
         <v>39</v>
       </c>
       <c r="D4" s="9" t="s">
+        <v>465</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="J4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="J4" s="9" t="s">
-        <v>46</v>
-      </c>
       <c r="K4" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="M4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="N4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="N4" s="9" t="s">
+      <c r="O4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="P4" s="9" t="s">
         <v>45</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="34" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" s="38"/>
       <c r="C5" s="38"/>
@@ -2654,7 +2726,7 @@
     </row>
     <row r="6" spans="1:16" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="21">
         <v>49.19</v>
@@ -2669,10 +2741,10 @@
         <v>1</v>
       </c>
       <c r="F6" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="21" t="s">
         <v>49</v>
-      </c>
-      <c r="G6" s="21" t="s">
-        <v>50</v>
       </c>
       <c r="H6" s="21">
         <v>950</v>
@@ -2688,10 +2760,10 @@
         <v>2</v>
       </c>
       <c r="L6" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M6" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N6" s="21">
         <v>870</v>
@@ -2706,7 +2778,7 @@
     </row>
     <row r="7" spans="1:16" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B7" s="21">
         <v>12.18</v>
@@ -2721,10 +2793,10 @@
         <v>1</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H7" s="21">
         <v>820</v>
@@ -2740,10 +2812,10 @@
         <v>2</v>
       </c>
       <c r="L7" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M7" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N7" s="21">
         <v>647</v>
@@ -2758,7 +2830,7 @@
     </row>
     <row r="8" spans="1:16" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B8" s="21">
         <v>49.19</v>
@@ -2773,10 +2845,10 @@
         <v>1</v>
       </c>
       <c r="F8" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="21" t="s">
         <v>49</v>
-      </c>
-      <c r="G8" s="21" t="s">
-        <v>50</v>
       </c>
       <c r="H8" s="21">
         <v>950</v>
@@ -2792,10 +2864,10 @@
         <v>2</v>
       </c>
       <c r="L8" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M8" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N8" s="21">
         <v>870</v>
@@ -2810,7 +2882,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="34" t="s">
-        <v>322</v>
+        <v>309</v>
       </c>
       <c r="B9" s="35"/>
       <c r="C9" s="35"/>
@@ -2830,7 +2902,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B10" s="21">
         <v>12.18</v>
@@ -2845,16 +2917,16 @@
         <v>3</v>
       </c>
       <c r="F10" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="G10" s="21" t="s">
-        <v>50</v>
-      </c>
       <c r="H10" s="21">
-        <v>950</v>
+        <v>920</v>
       </c>
       <c r="I10" s="21">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="J10" s="10">
         <f>IF($F10="fixed",1,Проект!$D$4)</f>
@@ -2864,16 +2936,16 @@
         <v>4</v>
       </c>
       <c r="L10" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M10" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N10" s="21">
-        <v>870</v>
+        <v>880</v>
       </c>
       <c r="O10" s="21">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="P10" s="10">
         <f>IF($F10="fixed",1,Проект!$D$4)</f>
@@ -2882,7 +2954,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B11" s="21">
         <v>12.18</v>
@@ -2897,10 +2969,10 @@
         <v>1</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H11" s="21">
         <v>820</v>
@@ -2916,10 +2988,10 @@
         <v>2</v>
       </c>
       <c r="L11" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M11" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N11" s="21">
         <v>647</v>
@@ -2934,7 +3006,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>323</v>
+        <v>310</v>
       </c>
       <c r="B12" s="21">
         <v>49.19</v>
@@ -2949,10 +3021,10 @@
         <v>1</v>
       </c>
       <c r="F12" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="21" t="s">
         <v>49</v>
-      </c>
-      <c r="G12" s="21" t="s">
-        <v>50</v>
       </c>
       <c r="H12" s="21">
         <v>950</v>
@@ -2968,10 +3040,10 @@
         <v>2</v>
       </c>
       <c r="L12" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M12" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N12" s="21">
         <v>870</v>
@@ -2986,23 +3058,23 @@
     </row>
     <row r="15" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>325</v>
+        <v>312</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="132" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>326</v>
+        <v>313</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -3070,7 +3142,7 @@
       <c r="C1" s="40"/>
       <c r="D1" s="41"/>
       <c r="E1" s="42" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F1" s="40"/>
       <c r="G1" s="40"/>
@@ -3082,7 +3154,7 @@
       <c r="M1" s="40"/>
       <c r="N1" s="41"/>
       <c r="O1" s="53" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P1" s="54"/>
       <c r="Q1" s="54"/>
@@ -3093,7 +3165,7 @@
       <c r="V1" s="54"/>
       <c r="W1" s="55"/>
       <c r="X1" s="39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Y1" s="40"/>
       <c r="Z1" s="40"/>
@@ -3105,7 +3177,7 @@
       <c r="AF1" s="40"/>
       <c r="AG1" s="41"/>
       <c r="AH1" s="50" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="AI1" s="51"/>
       <c r="AJ1" s="51"/>
@@ -3118,74 +3190,74 @@
     </row>
     <row r="2" spans="1:42" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B2" s="40"/>
       <c r="C2" s="40"/>
       <c r="D2" s="41"/>
       <c r="E2" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" s="44" t="s">
         <v>61</v>
-      </c>
-      <c r="F2" s="44" t="s">
-        <v>62</v>
       </c>
       <c r="G2" s="45"/>
       <c r="H2" s="46"/>
       <c r="I2" s="43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J2" s="40"/>
       <c r="K2" s="41"/>
       <c r="L2" s="47" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M2" s="48"/>
       <c r="N2" s="49"/>
       <c r="O2" s="44" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P2" s="45"/>
       <c r="Q2" s="46"/>
       <c r="R2" s="43" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="S2" s="40"/>
       <c r="T2" s="41"/>
       <c r="U2" s="47" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="V2" s="48"/>
       <c r="W2" s="49"/>
       <c r="X2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y2" s="44" t="s">
         <v>61</v>
-      </c>
-      <c r="Y2" s="44" t="s">
-        <v>62</v>
       </c>
       <c r="Z2" s="45"/>
       <c r="AA2" s="46"/>
       <c r="AB2" s="43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AC2" s="40"/>
       <c r="AD2" s="41"/>
       <c r="AE2" s="47" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AF2" s="48"/>
       <c r="AG2" s="49"/>
       <c r="AH2" s="44" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AI2" s="45"/>
       <c r="AJ2" s="46"/>
       <c r="AK2" s="43" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AL2" s="40"/>
       <c r="AM2" s="41"/>
       <c r="AN2" s="47" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AO2" s="48"/>
       <c r="AP2" s="49"/>
@@ -3195,127 +3267,127 @@
         <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>25</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="P3" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="P3" s="3" t="s">
+      <c r="Q3" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="R3" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="S3" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="T3" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="U3" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="V3" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="V3" s="3" t="s">
+      <c r="W3" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="W3" s="3" t="s">
-        <v>88</v>
       </c>
       <c r="X3" s="3" t="s">
         <v>31</v>
       </c>
       <c r="Y3" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z3" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="Z3" s="3" t="s">
+      <c r="AA3" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="AA3" s="3" t="s">
+      <c r="AB3" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="AB3" s="3" t="s">
+      <c r="AC3" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="AC3" s="3" t="s">
+      <c r="AD3" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="AD3" s="3" t="s">
+      <c r="AE3" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="AE3" s="3" t="s">
+      <c r="AF3" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="AF3" s="3" t="s">
+      <c r="AG3" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AG3" s="3" t="s">
+      <c r="AH3" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="AH3" s="3" t="s">
+      <c r="AI3" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="AI3" s="3" t="s">
+      <c r="AJ3" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="AJ3" s="3" t="s">
+      <c r="AK3" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="AK3" s="3" t="s">
+      <c r="AL3" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="AL3" s="3" t="s">
+      <c r="AM3" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="AM3" s="3" t="s">
+      <c r="AN3" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="AN3" s="3" t="s">
+      <c r="AO3" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="AO3" s="3" t="s">
+      <c r="AP3" s="3" t="s">
         <v>105</v>
-      </c>
-      <c r="AP3" s="3" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:42" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3326,129 +3398,129 @@
         <v>7</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="J4" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="K4" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="L4" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="M4" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="N4" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="O4" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="N4" s="9" t="s">
+      <c r="P4" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q4" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="R4" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="S4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="T4" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="U4" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="V4" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="W4" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="X4" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="Y4" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="Z4" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="AA4" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AB4" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="AC4" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="AD4" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="AE4" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="AF4" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG4" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="AH4" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="AI4" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="AJ4" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AK4" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="P4" s="9" t="s">
+      <c r="AL4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="Q4" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="R4" s="9" t="s">
+      <c r="AM4" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="S4" s="9" t="s">
+      <c r="AN4" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="AO4" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="T4" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="U4" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="V4" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="W4" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="X4" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="Y4" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="Z4" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AA4" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB4" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="AC4" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AD4" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="AE4" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="AF4" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="AG4" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="AH4" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="AI4" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="AJ4" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="AK4" s="9" t="s">
+      <c r="AP4" s="9" t="s">
         <v>119</v>
-      </c>
-      <c r="AL4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="AM4" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="AN4" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="AO4" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP4" s="9" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:42" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B5" s="11">
         <f>Проект!$D$3</f>
@@ -3466,11 +3538,11 @@
       </c>
       <c r="F5" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!f"&amp;$C5&amp;":f"&amp;$D5),"fixed",INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5),$A5)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5),"&lt;&gt;",INDIRECT("Плеть!h"&amp;$C5&amp;":h"&amp;$D5)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5)=$A5)*INDIRECT("Плеть!h"&amp;$C5&amp;":h"&amp;$D5)*INDIRECT("Плеть!j"&amp;$C5&amp;":j"&amp;$D5)))</f>
-        <v>2720</v>
+        <v>2690</v>
       </c>
       <c r="G5" s="17">
         <f ca="1">F5/B5</f>
-        <v>277.38119518662046</v>
+        <v>274.32184376912096</v>
       </c>
       <c r="H5" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5)=$A5)*INDIRECT("Плеть!b"&amp;$C5&amp;":b"&amp;$D5))</f>
@@ -3502,11 +3574,11 @@
       </c>
       <c r="O5" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!f"&amp;$C5&amp;":f"&amp;$D5),"fixed",INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5),$A5)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5),"&lt;&gt;",INDIRECT("Плеть!i"&amp;$C5&amp;":i"&amp;$D5)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5)=$A5)*INDIRECT("Плеть!i"&amp;$C5&amp;":i"&amp;$D5)*INDIRECT("Плеть!j"&amp;$C5&amp;":j"&amp;$D5)))</f>
-        <v>390</v>
+        <v>400</v>
       </c>
       <c r="P5" s="17">
         <f ca="1">O5/B5</f>
-        <v>39.771568427493378</v>
+        <v>40.791352233326535</v>
       </c>
       <c r="Q5" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5)=$A5)*INDIRECT("Плеть!b"&amp;$C5&amp;":b"&amp;$D5))</f>
@@ -3542,11 +3614,11 @@
       </c>
       <c r="Y5" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!l"&amp;$C5&amp;":l"&amp;$D5),"fixed",INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5),$A5)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5),"&lt;&gt;",INDIRECT("Плеть!n"&amp;$C5&amp;":n"&amp;$D5)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5)=$A5)*INDIRECT("Плеть!n"&amp;$C5&amp;":n"&amp;$D5)*INDIRECT("Плеть!p"&amp;$C5&amp;":p"&amp;$D5)))</f>
-        <v>2387</v>
+        <v>2397</v>
       </c>
       <c r="Z5" s="17">
         <f ca="1">Y5/B5</f>
-        <v>243.42239445237612</v>
+        <v>244.44217825820928</v>
       </c>
       <c r="AA5" s="12">
         <f ca="1">H5</f>
@@ -3578,11 +3650,11 @@
       </c>
       <c r="AH5" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!l"&amp;$C5&amp;":l"&amp;$D5),"fixed",INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5),$A5)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5),"&lt;&gt;",INDIRECT("Плеть!o"&amp;$C5&amp;":o"&amp;$D5)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C5&amp;":A"&amp;$D5)=$A5)*INDIRECT("Плеть!o"&amp;$C5&amp;":o"&amp;$D5)*INDIRECT("Плеть!p"&amp;$C5&amp;":p"&amp;$D5)))</f>
-        <v>355</v>
+        <v>345</v>
       </c>
       <c r="AI5" s="17">
         <f ca="1">AH5/B5</f>
-        <v>36.2023251070773</v>
+        <v>35.182541301244136</v>
       </c>
       <c r="AJ5" s="12">
         <f ca="1">Q5</f>
@@ -3615,7 +3687,7 @@
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B6" s="11">
         <f>Проект!$D$3</f>
@@ -3782,7 +3854,7 @@
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" s="11">
         <f>Проект!$D$3</f>
@@ -3800,11 +3872,11 @@
       </c>
       <c r="F7" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!f"&amp;$C7&amp;":f"&amp;$D7),"fixed",INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),$A7)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),"&lt;&gt;",INDIRECT("Плеть!h"&amp;$C7&amp;":h"&amp;$D7)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!h"&amp;$C7&amp;":h"&amp;$D7)*INDIRECT("Плеть!j"&amp;$C7&amp;":j"&amp;$D7)))</f>
-        <v>76</v>
+        <v>73.600000000000009</v>
       </c>
       <c r="G7" s="17">
         <f ca="1">F7/B7</f>
-        <v>7.750356924332042</v>
+        <v>7.5056088109320838</v>
       </c>
       <c r="H7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!b"&amp;$C7&amp;":b"&amp;$D7))</f>
@@ -3812,11 +3884,11 @@
       </c>
       <c r="I7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!h"&amp;$C7&amp;":h"&amp;$D7))</f>
-        <v>950</v>
+        <v>920</v>
       </c>
       <c r="J7" s="17">
         <f ca="1">I7/B7</f>
-        <v>96.879461554150524</v>
+        <v>93.820110136651039</v>
       </c>
       <c r="K7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!c"&amp;$C7&amp;":c"&amp;$D7))</f>
@@ -3824,11 +3896,11 @@
       </c>
       <c r="L7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!h"&amp;$C7&amp;":h"&amp;$D7))</f>
-        <v>950</v>
+        <v>920</v>
       </c>
       <c r="M7" s="17">
         <f ca="1">L7/B7</f>
-        <v>96.879461554150524</v>
+        <v>93.820110136651039</v>
       </c>
       <c r="N7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!c"&amp;$C7&amp;":c"&amp;$D7))</f>
@@ -3836,11 +3908,11 @@
       </c>
       <c r="O7" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!f"&amp;$C7&amp;":f"&amp;$D7),"fixed",INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),$A7)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),"&lt;&gt;",INDIRECT("Плеть!i"&amp;$C7&amp;":i"&amp;$D7)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!i"&amp;$C7&amp;":i"&amp;$D7)*INDIRECT("Плеть!j"&amp;$C7&amp;":j"&amp;$D7)))</f>
-        <v>11.200000000000001</v>
+        <v>12</v>
       </c>
       <c r="P7" s="17">
         <f ca="1">O7/B7</f>
-        <v>1.1421578625331432</v>
+        <v>1.2237405669997961</v>
       </c>
       <c r="Q7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!b"&amp;$C7&amp;":b"&amp;$D7))</f>
@@ -3848,11 +3920,11 @@
       </c>
       <c r="R7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!i"&amp;$C7&amp;":i"&amp;$D7))</f>
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="S7" s="17">
         <f ca="1">R7/B7</f>
-        <v>14.276973281664288</v>
+        <v>15.296757087497452</v>
       </c>
       <c r="T7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!d"&amp;$C7&amp;":d"&amp;$D7))</f>
@@ -3860,11 +3932,11 @@
       </c>
       <c r="U7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!i"&amp;$C7&amp;":i"&amp;$D7))</f>
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="V7" s="17">
         <f ca="1">U7/B7</f>
-        <v>14.276973281664288</v>
+        <v>15.296757087497452</v>
       </c>
       <c r="W7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!d"&amp;$C7&amp;":d"&amp;$D7))</f>
@@ -3876,11 +3948,11 @@
       </c>
       <c r="Y7" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!l"&amp;$C7&amp;":l"&amp;$D7),"fixed",INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),$A7)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),"&lt;&gt;",INDIRECT("Плеть!n"&amp;$C7&amp;":n"&amp;$D7)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!n"&amp;$C7&amp;":n"&amp;$D7)*INDIRECT("Плеть!p"&amp;$C7&amp;":p"&amp;$D7)))</f>
-        <v>69.600000000000009</v>
+        <v>70.400000000000006</v>
       </c>
       <c r="Z7" s="17">
         <f ca="1">Y7/B7</f>
-        <v>7.0976952885988185</v>
+        <v>7.1792779930654715</v>
       </c>
       <c r="AA7" s="12">
         <f ca="1">H7</f>
@@ -3888,11 +3960,11 @@
       </c>
       <c r="AB7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!n"&amp;$C7&amp;":n"&amp;$D7))</f>
-        <v>870</v>
+        <v>880</v>
       </c>
       <c r="AC7" s="17">
         <f ca="1">AB7/B7</f>
-        <v>88.721191107485225</v>
+        <v>89.740974913318382</v>
       </c>
       <c r="AD7" s="12">
         <f ca="1">K7</f>
@@ -3900,11 +3972,11 @@
       </c>
       <c r="AE7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!n"&amp;$C7&amp;":n"&amp;$D7))</f>
-        <v>870</v>
+        <v>880</v>
       </c>
       <c r="AF7" s="17">
         <f ca="1">AE7/B7</f>
-        <v>88.721191107485225</v>
+        <v>89.740974913318382</v>
       </c>
       <c r="AG7" s="12">
         <f ca="1">N7</f>
@@ -3912,11 +3984,11 @@
       </c>
       <c r="AH7" s="12">
         <f ca="1">IF(COUNTIFS(INDIRECT("Плеть!l"&amp;$C7&amp;":l"&amp;$D7),"fixed",INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),$A7)&gt;0,SUMIF(INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7),"&lt;&gt;",INDIRECT("Плеть!o"&amp;$C7&amp;":o"&amp;$D7)),SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!o"&amp;$C7&amp;":o"&amp;$D7)*INDIRECT("Плеть!p"&amp;$C7&amp;":p"&amp;$D7)))</f>
-        <v>10.4</v>
+        <v>9.6</v>
       </c>
       <c r="AI7" s="17">
         <f ca="1">AH7/B7</f>
-        <v>1.0605751580664899</v>
+        <v>0.97899245359983689</v>
       </c>
       <c r="AJ7" s="12">
         <f ca="1">Q7</f>
@@ -3924,11 +3996,11 @@
       </c>
       <c r="AK7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!o"&amp;$C7&amp;":o"&amp;$D7))</f>
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="AL7" s="17">
         <f ca="1">AK7/B7</f>
-        <v>13.257189475831124</v>
+        <v>12.237405669997962</v>
       </c>
       <c r="AM7" s="12">
         <f ca="1">T7</f>
@@ -3936,11 +4008,11 @@
       </c>
       <c r="AN7" s="12">
         <f ca="1">SUMPRODUCT((INDIRECT("Плеть!A"&amp;$C7&amp;":A"&amp;$D7)=$A7)*INDIRECT("Плеть!o"&amp;$C7&amp;":o"&amp;$D7))</f>
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="AO7" s="17">
         <f ca="1">AN7/B7</f>
-        <v>13.257189475831124</v>
+        <v>12.237405669997962</v>
       </c>
       <c r="AP7" s="12">
         <f ca="1">W7</f>
@@ -3993,27 +4065,27 @@
     </row>
     <row r="9" spans="1:42" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:42" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:42" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:42" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:42" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -4051,7 +4123,7 @@
   <sheetData>
     <row r="1" spans="1:93" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>441</v>
+        <v>428</v>
       </c>
       <c r="B1" s="42" t="s">
         <v>20</v>
@@ -4062,7 +4134,7 @@
       <c r="F1" s="40"/>
       <c r="G1" s="41"/>
       <c r="H1" s="61" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I1" s="62"/>
       <c r="J1" s="62"/>
@@ -4076,7 +4148,7 @@
       <c r="R1" s="62"/>
       <c r="S1" s="63"/>
       <c r="T1" s="43" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U1" s="40"/>
       <c r="V1" s="40"/>
@@ -4088,7 +4160,7 @@
       <c r="AB1" s="40"/>
       <c r="AC1" s="41"/>
       <c r="AD1" s="39" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AE1" s="40"/>
       <c r="AF1" s="40"/>
@@ -4104,7 +4176,7 @@
       <c r="AP1" s="40"/>
       <c r="AQ1" s="41"/>
       <c r="AR1" s="58" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AS1" s="59"/>
       <c r="AT1" s="59"/>
@@ -4124,7 +4196,7 @@
       <c r="BH1" s="59"/>
       <c r="BI1" s="60"/>
       <c r="BJ1" s="43" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="BK1" s="40"/>
       <c r="BL1" s="40"/>
@@ -4140,7 +4212,7 @@
       <c r="BV1" s="40"/>
       <c r="BW1" s="41"/>
       <c r="BX1" s="42" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="BY1" s="40"/>
       <c r="BZ1" s="40"/>
@@ -4156,7 +4228,7 @@
       <c r="CJ1" s="40"/>
       <c r="CK1" s="41"/>
       <c r="CL1" s="56" t="s">
-        <v>449</v>
+        <v>436</v>
       </c>
       <c r="CM1" s="57"/>
       <c r="CN1" s="57"/>
@@ -4164,575 +4236,575 @@
     </row>
     <row r="2" spans="1:93" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>442</v>
+        <v>429</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="T2" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="R2" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="T2" s="3" t="s">
+      <c r="U2" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="V2" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="V2" s="3" t="s">
+      <c r="W2" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="W2" s="3" t="s">
+      <c r="X2" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="Y2" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="Y2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="Z2" s="3" t="s">
+      <c r="AA2" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="AA2" s="3" t="s">
+      <c r="AB2" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="AB2" s="3" t="s">
+      <c r="AC2" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AD2" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="AD2" s="3" t="s">
+      <c r="AE2" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="AE2" s="3" t="s">
+      <c r="AF2" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="AF2" s="3" t="s">
+      <c r="AG2" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="AG2" s="3" t="s">
+      <c r="AH2" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="AH2" s="3" t="s">
+      <c r="AI2" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="AI2" s="3" t="s">
+      <c r="AJ2" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="AJ2" s="3" t="s">
+      <c r="AK2" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="AK2" s="3" t="s">
+      <c r="AL2" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="AL2" s="3" t="s">
+      <c r="AM2" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="AM2" s="3" t="s">
+      <c r="AN2" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="AN2" s="3" t="s">
+      <c r="AO2" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="AO2" s="3" t="s">
+      <c r="AP2" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="AP2" s="3" t="s">
+      <c r="AQ2" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="AQ2" s="3" t="s">
+      <c r="AR2" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="AR2" s="3" t="s">
+      <c r="AS2" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="AS2" s="3" t="s">
+      <c r="AT2" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="AT2" s="3" t="s">
+      <c r="AU2" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="AU2" s="3" t="s">
+      <c r="AV2" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="AV2" s="3" t="s">
+      <c r="AW2" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="AW2" s="3" t="s">
+      <c r="AX2" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="AX2" s="3" t="s">
+      <c r="AY2" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="AY2" s="3" t="s">
+      <c r="AZ2" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="AZ2" s="3" t="s">
+      <c r="BA2" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="BA2" s="3" t="s">
+      <c r="BB2" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="BB2" s="3" t="s">
+      <c r="BC2" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="BC2" s="3" t="s">
+      <c r="BD2" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="BD2" s="3" t="s">
+      <c r="BE2" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="BE2" s="3" t="s">
+      <c r="BF2" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="BF2" s="3" t="s">
+      <c r="BG2" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="BG2" s="3" t="s">
+      <c r="BH2" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="BH2" s="3" t="s">
+      <c r="BI2" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="BI2" s="3" t="s">
+      <c r="BJ2" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="BJ2" s="3" t="s">
+      <c r="BK2" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="BL2" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="BM2" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="BK2" s="3" t="s">
-        <v>476</v>
-      </c>
-      <c r="BL2" s="3" t="s">
-        <v>477</v>
-      </c>
-      <c r="BM2" s="3" t="s">
+      <c r="BN2" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="BN2" s="3" t="s">
+      <c r="BO2" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="BO2" s="3" t="s">
+      <c r="BP2" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="BP2" s="3" t="s">
+      <c r="BQ2" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="BQ2" s="3" t="s">
+      <c r="BR2" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="BR2" s="3" t="s">
+      <c r="BS2" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="BS2" s="3" t="s">
+      <c r="BT2" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="BT2" s="3" t="s">
+      <c r="BU2" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="BU2" s="3" t="s">
+      <c r="BV2" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="BV2" s="3" t="s">
+      <c r="BW2" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="BW2" s="3" t="s">
+      <c r="BX2" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="BX2" s="3" t="s">
+      <c r="BY2" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="BZ2" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="CA2" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="BY2" s="3" t="s">
-        <v>480</v>
-      </c>
-      <c r="BZ2" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="CA2" s="3" t="s">
+      <c r="CB2" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="CB2" s="3" t="s">
+      <c r="CC2" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="CC2" s="3" t="s">
+      <c r="CD2" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="CD2" s="3" t="s">
+      <c r="CE2" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="CE2" s="3" t="s">
+      <c r="CF2" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="CF2" s="3" t="s">
+      <c r="CG2" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="CG2" s="3" t="s">
+      <c r="CH2" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="CH2" s="3" t="s">
+      <c r="CI2" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="CI2" s="3" t="s">
+      <c r="CJ2" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="CJ2" s="3" t="s">
+      <c r="CK2" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="CK2" s="3" t="s">
-        <v>212</v>
-      </c>
       <c r="CL2" s="3" t="s">
-        <v>450</v>
+        <v>437</v>
       </c>
       <c r="CM2" s="3" t="s">
-        <v>451</v>
+        <v>438</v>
       </c>
       <c r="CN2" s="3" t="s">
-        <v>452</v>
+        <v>439</v>
       </c>
       <c r="CO2" s="3" t="s">
-        <v>453</v>
+        <v>440</v>
       </c>
     </row>
     <row r="3" spans="1:93" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>443</v>
+        <v>430</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>37</v>
       </c>
       <c r="C3" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="F3" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="D3" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="J3" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="N3" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="P3" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="Q3" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="R3" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>446</v>
+      </c>
+      <c r="T3" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="R3" s="9" t="s">
-        <v>458</v>
-      </c>
-      <c r="S3" s="9" t="s">
-        <v>459</v>
-      </c>
-      <c r="T3" s="9" t="s">
+      <c r="U3" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="U3" s="9" t="s">
+      <c r="V3" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="V3" s="9" t="s">
+      <c r="W3" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="W3" s="9" t="s">
+      <c r="X3" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="X3" s="9" t="s">
+      <c r="Y3" s="9" t="s">
+        <v>484</v>
+      </c>
+      <c r="Z3" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="Y3" s="9" t="s">
+      <c r="AA3" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="Z3" s="9" t="s">
+      <c r="AB3" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="AA3" s="9" t="s">
+      <c r="AC3" s="9" t="s">
+        <v>485</v>
+      </c>
+      <c r="AD3" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="AB3" s="9" t="s">
+      <c r="AE3" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="AF3" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="AG3" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="AH3" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="AI3" s="9" t="s">
+        <v>484</v>
+      </c>
+      <c r="AJ3" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="AK3" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="AL3" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="AM3" s="9" t="s">
+        <v>485</v>
+      </c>
+      <c r="AN3" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="AC3" s="9" t="s">
+      <c r="AO3" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="AD3" s="9" t="s">
+      <c r="AP3" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="AE3" s="9" t="s">
+      <c r="AQ3" s="9" t="s">
+        <v>486</v>
+      </c>
+      <c r="AR3" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="AS3" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="AT3" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="AF3" s="9" t="s">
+      <c r="AU3" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="AG3" s="9" t="s">
+      <c r="AV3" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="AH3" s="9" t="s">
+      <c r="AW3" s="9" t="s">
+        <v>484</v>
+      </c>
+      <c r="AX3" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="AI3" s="9" t="s">
+      <c r="AY3" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="AJ3" s="9" t="s">
+      <c r="AZ3" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="AK3" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="AL3" s="9" t="s">
+      <c r="BA3" s="9" t="s">
+        <v>485</v>
+      </c>
+      <c r="BB3" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="AM3" s="9" t="s">
+      <c r="BC3" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="AN3" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="AO3" s="9" t="s">
+      <c r="BD3" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="BE3" s="9" t="s">
+        <v>486</v>
+      </c>
+      <c r="BF3" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="AP3" s="9" t="s">
+      <c r="BG3" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="AQ3" s="9" t="s">
+      <c r="BH3" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="AR3" s="9" t="s">
+      <c r="BI3" s="9" t="s">
+        <v>487</v>
+      </c>
+      <c r="BJ3" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="AS3" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="AT3" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="AU3" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="AV3" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="AW3" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="AX3" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="AY3" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="AZ3" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="BA3" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="BB3" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="BC3" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="BD3" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="BE3" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="BF3" s="9" t="s">
+      <c r="BK3" s="9" t="s">
+        <v>462</v>
+      </c>
+      <c r="BL3" s="9" t="s">
+        <v>461</v>
+      </c>
+      <c r="BM3" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="BG3" s="9" t="s">
+      <c r="BN3" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="BH3" s="9" t="s">
+      <c r="BO3" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="BI3" s="9" t="s">
+      <c r="BP3" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="BJ3" s="9" t="s">
+      <c r="BQ3" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="BK3" s="9" t="s">
-        <v>479</v>
-      </c>
-      <c r="BL3" s="9" t="s">
-        <v>478</v>
-      </c>
-      <c r="BM3" s="9" t="s">
+      <c r="BR3" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="BN3" s="9" t="s">
+      <c r="BS3" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="BO3" s="9" t="s">
+      <c r="BT3" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="BP3" s="9" t="s">
+      <c r="BU3" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="BQ3" s="9" t="s">
+      <c r="BV3" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="BR3" s="9" t="s">
+      <c r="BW3" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="BS3" s="9" t="s">
+      <c r="BX3" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="BT3" s="9" t="s">
+      <c r="BY3" s="9" t="s">
+        <v>462</v>
+      </c>
+      <c r="BZ3" s="9" t="s">
+        <v>461</v>
+      </c>
+      <c r="CA3" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="BU3" s="9" t="s">
+      <c r="CB3" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="BV3" s="9" t="s">
+      <c r="CC3" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="CD3" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="CE3" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="BW3" s="9" t="s">
+      <c r="CF3" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="CG3" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="CH3" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="CI3" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="CJ3" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="CK3" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="BX3" s="9" t="s">
-        <v>258</v>
-      </c>
-      <c r="BY3" s="9" t="s">
-        <v>479</v>
-      </c>
-      <c r="BZ3" s="9" t="s">
-        <v>478</v>
-      </c>
-      <c r="CA3" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="CB3" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="CC3" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="CD3" s="9" t="s">
-        <v>250</v>
-      </c>
-      <c r="CE3" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="CF3" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="CG3" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="CH3" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="CI3" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="CJ3" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="CK3" s="9" t="s">
-        <v>262</v>
-      </c>
       <c r="CL3" s="9" t="s">
-        <v>454</v>
+        <v>441</v>
       </c>
       <c r="CM3" s="9" t="s">
-        <v>455</v>
+        <v>442</v>
       </c>
       <c r="CN3" s="9" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="CO3" s="9" t="s">
-        <v>457</v>
+        <v>444</v>
       </c>
     </row>
     <row r="4" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>444</v>
+        <v>431</v>
       </c>
       <c r="D4" s="21">
         <v>10</v>
@@ -4741,10 +4813,10 @@
         <v>12</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>446</v>
+        <v>433</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>447</v>
+        <v>434</v>
       </c>
       <c r="H4" s="21">
         <v>1</v>
@@ -4791,7 +4863,7 @@
         <v>6</v>
       </c>
       <c r="X4" s="24" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="Y4" s="24">
         <v>1</v>
@@ -4799,7 +4871,7 @@
       <c r="Z4" s="24"/>
       <c r="AA4" s="24"/>
       <c r="AB4" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AC4" s="24"/>
       <c r="AD4" s="21">
@@ -4815,19 +4887,19 @@
         <v>1</v>
       </c>
       <c r="AH4" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AI4" s="24"/>
       <c r="AJ4" s="24"/>
       <c r="AK4" s="24"/>
       <c r="AL4" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AM4" s="24"/>
       <c r="AN4" s="24"/>
       <c r="AO4" s="24"/>
       <c r="AP4" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AQ4" s="24"/>
       <c r="AR4" s="21">
@@ -4843,7 +4915,7 @@
         <v>4</v>
       </c>
       <c r="AV4" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AW4" s="24"/>
       <c r="AX4" s="24">
@@ -4853,7 +4925,7 @@
         <v>3</v>
       </c>
       <c r="AZ4" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="BA4" s="24"/>
       <c r="BB4" s="24">
@@ -4863,13 +4935,13 @@
         <v>5</v>
       </c>
       <c r="BD4" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="BE4" s="24"/>
       <c r="BF4" s="24"/>
       <c r="BG4" s="24"/>
       <c r="BH4" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="BI4" s="24"/>
       <c r="BJ4" s="21">
@@ -4914,7 +4986,7 @@
         <v>1</v>
       </c>
       <c r="BW4" s="21" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="BX4" s="10"/>
       <c r="BY4" s="21">
@@ -4935,27 +5007,27 @@
       <c r="CJ4" s="10"/>
       <c r="CK4" s="10"/>
       <c r="CL4" s="21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="CM4" s="21">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="CN4" s="21">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CO4" s="21">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="D5" s="21">
         <v>10</v>
@@ -4965,7 +5037,7 @@
       </c>
       <c r="F5" s="10"/>
       <c r="G5" s="10" t="s">
-        <v>447</v>
+        <v>434</v>
       </c>
       <c r="H5" s="21">
         <v>1</v>
@@ -5016,7 +5088,7 @@
         <v>6</v>
       </c>
       <c r="X5" s="24" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="Y5" s="24">
         <v>1</v>
@@ -5024,7 +5096,7 @@
       <c r="Z5" s="24"/>
       <c r="AA5" s="24"/>
       <c r="AB5" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AC5" s="24"/>
       <c r="AD5" s="21">
@@ -5040,19 +5112,19 @@
         <v>1</v>
       </c>
       <c r="AH5" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AI5" s="24"/>
       <c r="AJ5" s="24"/>
       <c r="AK5" s="24"/>
       <c r="AL5" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AM5" s="24"/>
       <c r="AN5" s="24"/>
       <c r="AO5" s="24"/>
       <c r="AP5" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AQ5" s="24"/>
       <c r="AR5" s="21">
@@ -5068,7 +5140,7 @@
         <v>4</v>
       </c>
       <c r="AV5" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AW5" s="24"/>
       <c r="AX5" s="24">
@@ -5078,7 +5150,7 @@
         <v>3</v>
       </c>
       <c r="AZ5" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="BA5" s="24"/>
       <c r="BB5" s="24">
@@ -5088,13 +5160,13 @@
         <v>5</v>
       </c>
       <c r="BD5" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="BE5" s="24"/>
       <c r="BF5" s="24"/>
       <c r="BG5" s="24"/>
       <c r="BH5" s="24" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="BI5" s="24"/>
       <c r="BJ5" s="21">
@@ -5139,7 +5211,7 @@
         <v>1</v>
       </c>
       <c r="BW5" s="21" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="BX5" s="21">
         <v>-1</v>
@@ -5183,7 +5255,7 @@
         <v>1</v>
       </c>
       <c r="CK5" s="21" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="CL5" s="21">
         <v>1</v>
@@ -5200,62 +5272,62 @@
     </row>
     <row r="6" spans="1:93" x14ac:dyDescent="0.25">
       <c r="F6" t="s">
-        <v>445</v>
+        <v>432</v>
       </c>
       <c r="AE6" s="19"/>
       <c r="AS6" s="19"/>
       <c r="BX6" s="19" t="s">
-        <v>331</v>
+        <v>318</v>
       </c>
       <c r="BY6" s="33" t="s">
-        <v>475</v>
+        <v>458</v>
       </c>
       <c r="BZ6" s="33"/>
     </row>
     <row r="7" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="F7" t="s">
-        <v>448</v>
+        <v>435</v>
       </c>
       <c r="BX7" s="19" t="s">
-        <v>437</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8" spans="1:93" ht="112.5" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
     </row>
     <row r="9" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:93" ht="90" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" spans="1:93" ht="123.75" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
     </row>
     <row r="12" spans="1:93" ht="90" x14ac:dyDescent="0.25">
       <c r="B12" s="6" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
     </row>
     <row r="13" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
     </row>
     <row r="14" spans="1:93" ht="90" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -5276,243 +5348,306 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:AB10"/>
+  <dimension ref="A1:AK10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="14" customWidth="1"/>
-    <col min="6" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="13" width="14" customWidth="1"/>
-    <col min="14" max="15" width="12" customWidth="1"/>
-    <col min="16" max="17" width="14" customWidth="1"/>
-    <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="22" width="10" customWidth="1"/>
-    <col min="23" max="23" width="12.5703125" customWidth="1"/>
-    <col min="24" max="25" width="14" customWidth="1"/>
-    <col min="26" max="26" width="16" customWidth="1"/>
+    <col min="1" max="11" width="14" customWidth="1"/>
+    <col min="12" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="12" customWidth="1"/>
+    <col min="21" max="22" width="14" customWidth="1"/>
+    <col min="23" max="24" width="12" customWidth="1"/>
+    <col min="25" max="26" width="14" customWidth="1"/>
     <col min="27" max="27" width="12" customWidth="1"/>
-    <col min="28" max="28" width="14" customWidth="1"/>
+    <col min="28" max="31" width="10" customWidth="1"/>
+    <col min="32" max="32" width="12.5703125" customWidth="1"/>
+    <col min="33" max="34" width="14" customWidth="1"/>
+    <col min="35" max="35" width="16" customWidth="1"/>
+    <col min="36" max="36" width="12" customWidth="1"/>
+    <col min="37" max="37" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="67" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="C1" s="40"/>
       <c r="D1" s="40"/>
       <c r="E1" s="40"/>
       <c r="F1" s="40"/>
       <c r="G1" s="40"/>
-      <c r="H1" s="53" t="s">
-        <v>468</v>
-      </c>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="43" t="s">
-        <v>275</v>
-      </c>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
       <c r="L1" s="40"/>
       <c r="M1" s="40"/>
-      <c r="N1" s="41"/>
-      <c r="O1" s="70" t="s">
-        <v>276</v>
-      </c>
-      <c r="P1" s="71"/>
-      <c r="Q1" s="71"/>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71"/>
-      <c r="T1" s="71"/>
-      <c r="U1" s="71"/>
-      <c r="V1" s="72"/>
-      <c r="W1" s="64" t="s">
-        <v>277</v>
-      </c>
-      <c r="X1" s="65"/>
-      <c r="Y1" s="66"/>
-      <c r="Z1" s="68" t="s">
-        <v>278</v>
-      </c>
-      <c r="AA1" s="69"/>
-      <c r="AB1" s="69"/>
-    </row>
-    <row r="2" spans="1:28" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N1" s="53" t="s">
+        <v>455</v>
+      </c>
+      <c r="O1" s="73"/>
+      <c r="P1" s="54"/>
+      <c r="Q1" s="54"/>
+      <c r="R1" s="54"/>
+      <c r="S1" s="54"/>
+      <c r="T1" s="43" t="s">
+        <v>270</v>
+      </c>
+      <c r="U1" s="40"/>
+      <c r="V1" s="40"/>
+      <c r="W1" s="41"/>
+      <c r="X1" s="70" t="s">
+        <v>271</v>
+      </c>
+      <c r="Y1" s="71"/>
+      <c r="Z1" s="71"/>
+      <c r="AA1" s="71"/>
+      <c r="AB1" s="71"/>
+      <c r="AC1" s="71"/>
+      <c r="AD1" s="71"/>
+      <c r="AE1" s="72"/>
+      <c r="AF1" s="64" t="s">
+        <v>272</v>
+      </c>
+      <c r="AG1" s="65"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="68" t="s">
+        <v>273</v>
+      </c>
+      <c r="AJ1" s="69"/>
+      <c r="AK1" s="69"/>
+    </row>
+    <row r="2" spans="1:37" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>24</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="W2" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="X2" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="AB2" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="AC2" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="AD2" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="AE2" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="AF2" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="AG2" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="AH2" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>470</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>471</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>473</v>
-      </c>
-      <c r="K2" s="3" t="s">
+      <c r="AI2" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="AJ2" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="AK2" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="N2" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>462</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>463</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>464</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="W2" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="X2" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="Y2" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="Z2" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="AB2" s="3" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:37" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>37</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>470</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>471</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>475</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>466</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>467</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>481</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>482</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>483</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>492</v>
+      </c>
+      <c r="O3" s="9" t="s">
+        <v>493</v>
+      </c>
+      <c r="P3" s="9" t="s">
+        <v>494</v>
+      </c>
+      <c r="Q3" s="9" t="s">
+        <v>495</v>
+      </c>
+      <c r="R3" s="9" t="s">
+        <v>496</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>457</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="U3" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="V3" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="W3" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="X3" s="9" t="s">
+        <v>453</v>
+      </c>
+      <c r="Y3" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="Z3" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="AA3" s="9" t="s">
+        <v>454</v>
+      </c>
+      <c r="AB3" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="AC3" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="AD3" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="AE3" s="9" t="s">
         <v>297</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="AF3" s="9" t="s">
         <v>298</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="AG3" s="9" t="s">
         <v>299</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="AH3" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="AI3" s="25" t="s">
+        <v>319</v>
+      </c>
+      <c r="AJ3" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="AK3" s="9" t="s">
         <v>301</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>302</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>469</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>472</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>474</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>303</v>
-      </c>
-      <c r="L3" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="M3" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="N3" s="9" t="s">
-        <v>306</v>
-      </c>
-      <c r="O3" s="9" t="s">
-        <v>466</v>
-      </c>
-      <c r="P3" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="Q3" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="R3" s="9" t="s">
-        <v>467</v>
-      </c>
-      <c r="S3" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="T3" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="U3" s="9" t="s">
-        <v>309</v>
-      </c>
-      <c r="V3" s="9" t="s">
-        <v>310</v>
-      </c>
-      <c r="W3" s="9" t="s">
-        <v>311</v>
-      </c>
-      <c r="X3" s="9" t="s">
-        <v>312</v>
-      </c>
-      <c r="Y3" s="9" t="s">
-        <v>313</v>
-      </c>
-      <c r="Z3" s="25" t="s">
-        <v>332</v>
-      </c>
-      <c r="AA3" s="9" t="s">
-        <v>309</v>
-      </c>
-      <c r="AB3" s="9" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:37" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B4" s="32">
         <v>1</v>
@@ -5541,62 +5676,89 @@
       <c r="J4" s="32">
         <v>1</v>
       </c>
-      <c r="K4" s="32" t="s">
-        <v>264</v>
-      </c>
-      <c r="L4" s="32"/>
-      <c r="M4" s="32"/>
-      <c r="N4" s="32"/>
-      <c r="O4" s="32" t="s">
-        <v>264</v>
+      <c r="K4" s="32">
+        <v>1</v>
+      </c>
+      <c r="L4" s="32">
+        <v>1</v>
+      </c>
+      <c r="M4" s="32">
+        <v>1</v>
+      </c>
+      <c r="N4" s="32">
+        <v>1</v>
+      </c>
+      <c r="O4" s="32">
+        <v>1</v>
       </c>
       <c r="P4" s="32">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="32">
+        <v>1</v>
+      </c>
+      <c r="R4" s="32">
+        <v>1</v>
+      </c>
+      <c r="S4" s="32">
+        <v>1</v>
+      </c>
+      <c r="T4" s="32" t="s">
+        <v>259</v>
+      </c>
+      <c r="U4" s="32"/>
+      <c r="V4" s="32"/>
+      <c r="W4" s="32"/>
+      <c r="X4" s="32" t="s">
+        <v>259</v>
+      </c>
+      <c r="Y4" s="32">
         <v>5</v>
       </c>
-      <c r="Q4" s="32">
+      <c r="Z4" s="32">
         <v>0</v>
       </c>
-      <c r="R4" s="32" t="s">
-        <v>264</v>
-      </c>
-      <c r="S4" s="32">
+      <c r="AA4" s="32" t="s">
+        <v>259</v>
+      </c>
+      <c r="AB4" s="32">
         <v>5</v>
       </c>
-      <c r="T4" s="32">
+      <c r="AC4" s="32">
         <v>0</v>
       </c>
-      <c r="U4" s="32">
+      <c r="AD4" s="32">
         <v>1.8</v>
       </c>
-      <c r="V4" s="32">
+      <c r="AE4" s="32">
         <v>30</v>
       </c>
-      <c r="W4" s="32" t="s">
-        <v>264</v>
-      </c>
-      <c r="X4" s="32"/>
-      <c r="Y4" s="32"/>
-      <c r="Z4" s="32" t="s">
-        <v>264</v>
-      </c>
-      <c r="AA4" s="32"/>
-      <c r="AB4" s="32"/>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AF4" s="32" t="s">
+        <v>259</v>
+      </c>
+      <c r="AG4" s="32"/>
+      <c r="AH4" s="32"/>
+      <c r="AI4" s="32" t="s">
+        <v>259</v>
+      </c>
+      <c r="AJ4" s="32"/>
+      <c r="AK4" s="32"/>
+    </row>
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B5" s="32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="32">
         <v>1</v>
@@ -5613,94 +5775,121 @@
       <c r="J5" s="32">
         <v>1</v>
       </c>
-      <c r="K5" s="32" t="s">
-        <v>265</v>
+      <c r="K5" s="32">
+        <v>1</v>
       </c>
       <c r="L5" s="32">
+        <v>1</v>
+      </c>
+      <c r="M5" s="32">
+        <v>1</v>
+      </c>
+      <c r="N5" s="32">
+        <v>1</v>
+      </c>
+      <c r="O5" s="32">
+        <v>1</v>
+      </c>
+      <c r="P5" s="32">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="32">
+        <v>1</v>
+      </c>
+      <c r="R5" s="32">
+        <v>1</v>
+      </c>
+      <c r="S5" s="32">
+        <v>1</v>
+      </c>
+      <c r="T5" s="32" t="s">
+        <v>260</v>
+      </c>
+      <c r="U5" s="32">
         <v>4</v>
       </c>
-      <c r="M5" s="32">
+      <c r="V5" s="32">
         <v>0</v>
       </c>
-      <c r="N5" s="32">
+      <c r="W5" s="32">
         <v>2</v>
       </c>
-      <c r="O5" s="32" t="s">
-        <v>265</v>
-      </c>
-      <c r="P5" s="32">
+      <c r="X5" s="32" t="s">
+        <v>260</v>
+      </c>
+      <c r="Y5" s="32">
         <v>5</v>
       </c>
-      <c r="Q5" s="32">
+      <c r="Z5" s="32">
         <v>0</v>
       </c>
-      <c r="R5" s="32" t="s">
-        <v>265</v>
-      </c>
-      <c r="S5" s="32">
+      <c r="AA5" s="32" t="s">
+        <v>260</v>
+      </c>
+      <c r="AB5" s="32">
         <v>5</v>
       </c>
-      <c r="T5" s="32">
+      <c r="AC5" s="32">
         <v>0</v>
       </c>
-      <c r="U5" s="32">
+      <c r="AD5" s="32">
         <v>1.8</v>
       </c>
-      <c r="V5" s="32">
+      <c r="AE5" s="32">
         <v>30</v>
       </c>
-      <c r="W5" s="32" t="s">
-        <v>265</v>
-      </c>
-      <c r="X5" s="32">
+      <c r="AF5" s="32" t="s">
+        <v>260</v>
+      </c>
+      <c r="AG5" s="32">
         <v>5</v>
       </c>
-      <c r="Y5" s="32">
+      <c r="AH5" s="32">
         <v>4</v>
       </c>
-      <c r="Z5" s="32" t="s">
-        <v>265</v>
-      </c>
-      <c r="AA5" s="32">
+      <c r="AI5" s="32" t="s">
+        <v>260</v>
+      </c>
+      <c r="AJ5" s="32">
         <v>2</v>
       </c>
-      <c r="AB5" s="32">
+      <c r="AK5" s="32">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="112.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" ht="112.5" x14ac:dyDescent="0.25">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="7" spans="1:37" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" ht="123.75" x14ac:dyDescent="0.25">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="8" spans="1:37" ht="123.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="9" spans="1:37" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" ht="112.5" x14ac:dyDescent="0.25">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="10" spans="1:37" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>319</v>
+        <v>306</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="W1:Y1"/>
-    <mergeCell ref="B1:G1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="Z1:AB1"/>
-    <mergeCell ref="O1:V1"/>
-    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="AF1:AH1"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="T1:W1"/>
+    <mergeCell ref="AI1:AK1"/>
+    <mergeCell ref="X1:AE1"/>
+    <mergeCell ref="N1:S1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5716,7 +5905,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>320</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5724,32 +5913,32 @@
     </row>
     <row r="3" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>321</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>333</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>334</v>
+        <v>321</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>336</v>
+        <v>323</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>337</v>
+        <v>324</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5757,22 +5946,22 @@
     </row>
     <row r="10" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>339</v>
+        <v>326</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>341</v>
+        <v>328</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5780,27 +5969,27 @@
     </row>
     <row r="15" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>342</v>
+        <v>329</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>344</v>
+        <v>331</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>345</v>
+        <v>332</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>346</v>
+        <v>333</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5808,52 +5997,52 @@
     </row>
     <row r="21" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>348</v>
+        <v>335</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>349</v>
+        <v>336</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>350</v>
+        <v>337</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
-        <v>352</v>
+        <v>339</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>353</v>
+        <v>340</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>354</v>
+        <v>341</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>355</v>
+        <v>342</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>356</v>
+        <v>343</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
@@ -5861,92 +6050,92 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>357</v>
+        <v>344</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>358</v>
+        <v>345</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>359</v>
+        <v>346</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>360</v>
+        <v>347</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>361</v>
+        <v>348</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>362</v>
+        <v>349</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>363</v>
+        <v>350</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>364</v>
+        <v>351</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>365</v>
+        <v>352</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>367</v>
+        <v>354</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>368</v>
+        <v>355</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>369</v>
+        <v>356</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>370</v>
+        <v>357</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>372</v>
+        <v>359</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>373</v>
+        <v>360</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>374</v>
+        <v>361</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
@@ -5954,92 +6143,92 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
-        <v>375</v>
+        <v>362</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>376</v>
+        <v>363</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>377</v>
+        <v>364</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>378</v>
+        <v>365</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>379</v>
+        <v>366</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>380</v>
+        <v>367</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>381</v>
+        <v>368</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>382</v>
+        <v>369</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>383</v>
+        <v>370</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
-        <v>384</v>
+        <v>371</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>385</v>
+        <v>372</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>386</v>
+        <v>373</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
@@ -6047,112 +6236,112 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
-        <v>393</v>
+        <v>380</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
-        <v>394</v>
+        <v>381</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
-        <v>395</v>
+        <v>382</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
-        <v>396</v>
+        <v>383</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
-        <v>397</v>
+        <v>384</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
-        <v>398</v>
+        <v>385</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
-        <v>399</v>
+        <v>386</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
-        <v>400</v>
+        <v>387</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="14" t="s">
-        <v>401</v>
+        <v>388</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="14" t="s">
-        <v>402</v>
+        <v>389</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="14" t="s">
-        <v>403</v>
+        <v>390</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="14" t="s">
-        <v>404</v>
+        <v>391</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="14" t="s">
-        <v>405</v>
+        <v>392</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="14" t="s">
-        <v>406</v>
+        <v>393</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="14" t="s">
-        <v>407</v>
+        <v>394</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
-        <v>408</v>
+        <v>395</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="14" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="14" t="s">
-        <v>410</v>
+        <v>397</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="14" t="s">
-        <v>411</v>
+        <v>398</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="14" t="s">
-        <v>412</v>
+        <v>399</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="14" t="s">
-        <v>413</v>
+        <v>400</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="14" t="s">
-        <v>414</v>
+        <v>401</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
@@ -6160,87 +6349,87 @@
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
-        <v>415</v>
+        <v>402</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="14" t="s">
-        <v>416</v>
+        <v>403</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="14" t="s">
-        <v>417</v>
+        <v>404</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="14" t="s">
-        <v>418</v>
+        <v>405</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="14" t="s">
-        <v>419</v>
+        <v>406</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="14" t="s">
-        <v>420</v>
+        <v>407</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="14" t="s">
-        <v>421</v>
+        <v>408</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="14" t="s">
-        <v>422</v>
+        <v>409</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="14" t="s">
-        <v>423</v>
+        <v>410</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="14" t="s">
-        <v>424</v>
+        <v>411</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
-        <v>425</v>
+        <v>412</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="14" t="s">
-        <v>426</v>
+        <v>413</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
-        <v>427</v>
+        <v>414</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="14" t="s">
-        <v>428</v>
+        <v>415</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
-        <v>429</v>
+        <v>416</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
-        <v>430</v>
+        <v>417</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
-        <v>431</v>
+        <v>418</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
@@ -6248,27 +6437,27 @@
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="15" t="s">
-        <v>432</v>
+        <v>419</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
-        <v>433</v>
+        <v>420</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
-        <v>434</v>
+        <v>421</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
-        <v>435</v>
+        <v>422</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
-        <v>436</v>
+        <v>423</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
It's ready to be loaded
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{303B6709-5801-45C4-920D-474DA76B2707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC3D1932-672D-4CEC-8E10-9B070BB2C5A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Проект" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="494">
   <si>
     <t>Параметр</t>
   </si>
@@ -1036,9 +1036,6 @@
     <t>Не учтено, что может быть две неподвижные оч вдоль</t>
   </si>
   <si>
-    <t>Не учтено, что на одной опоре может быть одна из двух неподвижная ОЧ. В таком случае со всей плети нагрузка должна собираться на одну ОЧ</t>
-  </si>
-  <si>
     <t>node_offset_piles</t>
   </si>
   <si>
@@ -1049,9 +1046,6 @@
   </si>
   <si>
     <t>Цвет ячеек для заполнения</t>
-  </si>
-  <si>
-    <t>Как-то учесть, что 2 рамки, когда опора относится к двум плетям</t>
   </si>
   <si>
     <t>Нагрузка от грунта
@@ -1370,9 +1364,6 @@
     <t xml:space="preserve">    movable Y → дополнительно Fy (бит 1) на верхнем конце (конец j).</t>
   </si>
   <si>
-    <t>Можно, чтобы он встречал первую рамку, шел на лист массы и брал первое упоминание опоры 3. Потом доходил до 2 рамки и искал второе упоминание</t>
-  </si>
-  <si>
     <t>z_hinge</t>
   </si>
   <si>
@@ -1475,9 +1466,6 @@
   </si>
   <si>
     <t>Ширина сваи, м</t>
-  </si>
-  <si>
-    <t>Может быть не симметрично</t>
   </si>
   <si>
     <t>f1_r_pad_y</t>
@@ -2056,11 +2044,6 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2076,6 +2059,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2469,7 +2457,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2505,7 +2493,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D6" s="22"/>
     </row>
@@ -2609,13 +2597,13 @@
         <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>25</v>
@@ -2665,7 +2653,7 @@
         <v>39</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>40</v>
@@ -3064,12 +3052,9 @@
         <v>312</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="132" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="56.25" x14ac:dyDescent="0.25">
@@ -3153,17 +3138,17 @@
       <c r="L1" s="40"/>
       <c r="M1" s="40"/>
       <c r="N1" s="41"/>
-      <c r="O1" s="53" t="s">
+      <c r="O1" s="50" t="s">
         <v>56</v>
       </c>
-      <c r="P1" s="54"/>
-      <c r="Q1" s="54"/>
-      <c r="R1" s="54"/>
-      <c r="S1" s="54"/>
-      <c r="T1" s="54"/>
-      <c r="U1" s="54"/>
-      <c r="V1" s="54"/>
-      <c r="W1" s="55"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
+      <c r="T1" s="51"/>
+      <c r="U1" s="51"/>
+      <c r="V1" s="51"/>
+      <c r="W1" s="52"/>
       <c r="X1" s="39" t="s">
         <v>57</v>
       </c>
@@ -3176,17 +3161,17 @@
       <c r="AE1" s="40"/>
       <c r="AF1" s="40"/>
       <c r="AG1" s="41"/>
-      <c r="AH1" s="50" t="s">
+      <c r="AH1" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="AI1" s="51"/>
-      <c r="AJ1" s="51"/>
-      <c r="AK1" s="51"/>
-      <c r="AL1" s="51"/>
-      <c r="AM1" s="51"/>
-      <c r="AN1" s="51"/>
-      <c r="AO1" s="51"/>
-      <c r="AP1" s="52"/>
+      <c r="AI1" s="48"/>
+      <c r="AJ1" s="48"/>
+      <c r="AK1" s="48"/>
+      <c r="AL1" s="48"/>
+      <c r="AM1" s="48"/>
+      <c r="AN1" s="48"/>
+      <c r="AO1" s="48"/>
+      <c r="AP1" s="49"/>
     </row>
     <row r="2" spans="1:42" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
@@ -3198,69 +3183,69 @@
       <c r="E2" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="44" t="s">
+      <c r="F2" s="53" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="45"/>
-      <c r="H2" s="46"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="55"/>
       <c r="I2" s="43" t="s">
         <v>62</v>
       </c>
       <c r="J2" s="40"/>
       <c r="K2" s="41"/>
-      <c r="L2" s="47" t="s">
+      <c r="L2" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="M2" s="48"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="44" t="s">
+      <c r="M2" s="45"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="46"/>
+      <c r="P2" s="54"/>
+      <c r="Q2" s="55"/>
       <c r="R2" s="43" t="s">
         <v>65</v>
       </c>
       <c r="S2" s="40"/>
       <c r="T2" s="41"/>
-      <c r="U2" s="47" t="s">
+      <c r="U2" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="V2" s="48"/>
-      <c r="W2" s="49"/>
+      <c r="V2" s="45"/>
+      <c r="W2" s="46"/>
       <c r="X2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="Y2" s="44" t="s">
+      <c r="Y2" s="53" t="s">
         <v>61</v>
       </c>
-      <c r="Z2" s="45"/>
-      <c r="AA2" s="46"/>
+      <c r="Z2" s="54"/>
+      <c r="AA2" s="55"/>
       <c r="AB2" s="43" t="s">
         <v>62</v>
       </c>
       <c r="AC2" s="40"/>
       <c r="AD2" s="41"/>
-      <c r="AE2" s="47" t="s">
+      <c r="AE2" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="AF2" s="48"/>
-      <c r="AG2" s="49"/>
-      <c r="AH2" s="44" t="s">
+      <c r="AF2" s="45"/>
+      <c r="AG2" s="46"/>
+      <c r="AH2" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="AI2" s="45"/>
-      <c r="AJ2" s="46"/>
+      <c r="AI2" s="54"/>
+      <c r="AJ2" s="55"/>
       <c r="AK2" s="43" t="s">
         <v>65</v>
       </c>
       <c r="AL2" s="40"/>
       <c r="AM2" s="41"/>
-      <c r="AN2" s="47" t="s">
+      <c r="AN2" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="AO2" s="48"/>
-      <c r="AP2" s="49"/>
+      <c r="AO2" s="45"/>
+      <c r="AP2" s="46"/>
     </row>
     <row r="3" spans="1:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -4090,6 +4075,14 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="AB2:AD2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="Y2:AA2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="E1:N1"/>
     <mergeCell ref="AE2:AG2"/>
     <mergeCell ref="AH1:AP1"/>
     <mergeCell ref="R2:T2"/>
@@ -4100,14 +4093,6 @@
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="AH2:AJ2"/>
     <mergeCell ref="U2:W2"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="AB2:AD2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="Y2:AA2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="E1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4123,7 +4108,7 @@
   <sheetData>
     <row r="1" spans="1:93" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="B1" s="42" t="s">
         <v>20</v>
@@ -4228,7 +4213,7 @@
       <c r="CJ1" s="40"/>
       <c r="CK1" s="41"/>
       <c r="CL1" s="56" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="CM1" s="57"/>
       <c r="CN1" s="57"/>
@@ -4236,7 +4221,7 @@
     </row>
     <row r="2" spans="1:93" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>24</v>
@@ -4287,10 +4272,10 @@
         <v>145</v>
       </c>
       <c r="R2" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="S2" s="3" t="s">
         <v>314</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>315</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>146</v>
@@ -4422,10 +4407,10 @@
         <v>188</v>
       </c>
       <c r="BK2" s="3" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="BL2" s="3" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="BM2" s="3" t="s">
         <v>189</v>
@@ -4464,10 +4449,10 @@
         <v>200</v>
       </c>
       <c r="BY2" s="3" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="BZ2" s="3" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="CA2" s="3" t="s">
         <v>201</v>
@@ -4503,21 +4488,21 @@
         <v>211</v>
       </c>
       <c r="CL2" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="CM2" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="CN2" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="CO2" s="3" t="s">
         <v>437</v>
-      </c>
-      <c r="CM2" s="3" t="s">
-        <v>438</v>
-      </c>
-      <c r="CN2" s="3" t="s">
-        <v>439</v>
-      </c>
-      <c r="CO2" s="3" t="s">
-        <v>440</v>
       </c>
     </row>
     <row r="3" spans="1:93" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>37</v>
@@ -4568,10 +4553,10 @@
         <v>224</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="T3" s="9" t="s">
         <v>225</v>
@@ -4589,7 +4574,7 @@
         <v>229</v>
       </c>
       <c r="Y3" s="9" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="Z3" s="9" t="s">
         <v>230</v>
@@ -4601,7 +4586,7 @@
         <v>232</v>
       </c>
       <c r="AC3" s="9" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="AD3" s="9" t="s">
         <v>233</v>
@@ -4619,7 +4604,7 @@
         <v>229</v>
       </c>
       <c r="AI3" s="9" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="AJ3" s="9" t="s">
         <v>230</v>
@@ -4631,7 +4616,7 @@
         <v>232</v>
       </c>
       <c r="AM3" s="9" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="AN3" s="9" t="s">
         <v>234</v>
@@ -4643,7 +4628,7 @@
         <v>236</v>
       </c>
       <c r="AQ3" s="9" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="AR3" s="9" t="s">
         <v>237</v>
@@ -4661,7 +4646,7 @@
         <v>229</v>
       </c>
       <c r="AW3" s="9" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="AX3" s="9" t="s">
         <v>230</v>
@@ -4673,7 +4658,7 @@
         <v>232</v>
       </c>
       <c r="BA3" s="9" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="BB3" s="9" t="s">
         <v>234</v>
@@ -4685,7 +4670,7 @@
         <v>236</v>
       </c>
       <c r="BE3" s="9" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="BF3" s="9" t="s">
         <v>238</v>
@@ -4697,16 +4682,16 @@
         <v>240</v>
       </c>
       <c r="BI3" s="9" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="BJ3" s="9" t="s">
         <v>241</v>
       </c>
       <c r="BK3" s="9" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="BL3" s="9" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="BM3" s="9" t="s">
         <v>242</v>
@@ -4745,10 +4730,10 @@
         <v>253</v>
       </c>
       <c r="BY3" s="9" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="BZ3" s="9" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="CA3" s="9" t="s">
         <v>254</v>
@@ -4784,16 +4769,16 @@
         <v>257</v>
       </c>
       <c r="CL3" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="CM3" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="CN3" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="CO3" s="9" t="s">
         <v>441</v>
-      </c>
-      <c r="CM3" s="9" t="s">
-        <v>442</v>
-      </c>
-      <c r="CN3" s="9" t="s">
-        <v>443</v>
-      </c>
-      <c r="CO3" s="9" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="4" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -4804,7 +4789,7 @@
         <v>121</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D4" s="21">
         <v>10</v>
@@ -4813,10 +4798,10 @@
         <v>12</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="H4" s="21">
         <v>1</v>
@@ -5037,7 +5022,7 @@
       </c>
       <c r="F5" s="10"/>
       <c r="G5" s="10" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="H5" s="21">
         <v>1</v>
@@ -5272,16 +5257,12 @@
     </row>
     <row r="6" spans="1:93" x14ac:dyDescent="0.25">
       <c r="F6" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="AE6" s="19"/>
       <c r="AS6" s="19"/>
-      <c r="BX6" s="19" t="s">
-        <v>318</v>
-      </c>
-      <c r="BY6" s="33" t="s">
-        <v>458</v>
-      </c>
+      <c r="BX6" s="19"/>
+      <c r="BY6" s="33"/>
       <c r="BZ6" s="33"/>
     </row>
     <row r="7" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
@@ -5289,11 +5270,9 @@
         <v>261</v>
       </c>
       <c r="F7" t="s">
-        <v>435</v>
-      </c>
-      <c r="BX7" s="19" t="s">
-        <v>424</v>
-      </c>
+        <v>432</v>
+      </c>
+      <c r="BX7" s="19"/>
     </row>
     <row r="8" spans="1:93" ht="112.5" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
@@ -5384,14 +5363,14 @@
       <c r="K1" s="40"/>
       <c r="L1" s="40"/>
       <c r="M1" s="40"/>
-      <c r="N1" s="53" t="s">
-        <v>455</v>
+      <c r="N1" s="50" t="s">
+        <v>452</v>
       </c>
       <c r="O1" s="73"/>
-      <c r="P1" s="54"/>
-      <c r="Q1" s="54"/>
-      <c r="R1" s="54"/>
-      <c r="S1" s="54"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
       <c r="T1" s="43" t="s">
         <v>270</v>
       </c>
@@ -5424,34 +5403,34 @@
         <v>24</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>468</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>472</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>473</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>477</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>274</v>
@@ -5460,22 +5439,22 @@
         <v>275</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>276</v>
@@ -5490,22 +5469,22 @@
         <v>279</v>
       </c>
       <c r="X2" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="AA2" s="3" t="s">
         <v>447</v>
       </c>
-      <c r="Y2" s="3" t="s">
+      <c r="AB2" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="Z2" s="3" t="s">
+      <c r="AC2" s="3" t="s">
         <v>449</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>450</v>
-      </c>
-      <c r="AB2" s="3" t="s">
-        <v>451</v>
-      </c>
-      <c r="AC2" s="3" t="s">
-        <v>452</v>
       </c>
       <c r="AD2" s="3" t="s">
         <v>280</v>
@@ -5537,34 +5516,34 @@
         <v>37</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>466</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>467</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>471</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>470</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>471</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>475</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>474</v>
-      </c>
       <c r="F3" s="9" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="L3" s="9" t="s">
         <v>288</v>
@@ -5573,22 +5552,22 @@
         <v>289</v>
       </c>
       <c r="N3" s="9" t="s">
+        <v>488</v>
+      </c>
+      <c r="O3" s="9" t="s">
+        <v>489</v>
+      </c>
+      <c r="P3" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="Q3" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="R3" s="9" t="s">
         <v>492</v>
       </c>
-      <c r="O3" s="9" t="s">
-        <v>493</v>
-      </c>
-      <c r="P3" s="9" t="s">
-        <v>494</v>
-      </c>
-      <c r="Q3" s="9" t="s">
-        <v>495</v>
-      </c>
-      <c r="R3" s="9" t="s">
-        <v>496</v>
-      </c>
       <c r="S3" s="9" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="T3" s="9" t="s">
         <v>290</v>
@@ -5603,7 +5582,7 @@
         <v>293</v>
       </c>
       <c r="X3" s="9" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="Y3" s="9" t="s">
         <v>294</v>
@@ -5612,7 +5591,7 @@
         <v>295</v>
       </c>
       <c r="AA3" s="9" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="AB3" s="9" t="s">
         <v>294</v>
@@ -5636,7 +5615,7 @@
         <v>300</v>
       </c>
       <c r="AI3" s="25" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="AJ3" s="9" t="s">
         <v>296</v>
@@ -5918,27 +5897,27 @@
     </row>
     <row r="4" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5946,22 +5925,22 @@
     </row>
     <row r="10" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5969,27 +5948,27 @@
     </row>
     <row r="15" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5997,52 +5976,52 @@
     </row>
     <row r="21" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
@@ -6050,92 +6029,92 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
@@ -6143,92 +6122,92 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
@@ -6236,112 +6215,112 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="14" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="14" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="14" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="14" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="14" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="14" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="14" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="14" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="14" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="14" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="14" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="14" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
@@ -6349,87 +6328,87 @@
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="14" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="14" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="14" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="14" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="14" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="14" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="14" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="14" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="14" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="14" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="14" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
@@ -6437,27 +6416,27 @@
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="15" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Module 1 fixed to read soil data in excel properly
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC3D1932-672D-4CEC-8E10-9B070BB2C5A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0590DD7F-C571-44A2-A12D-A2232026DB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Проект" sheetId="1" r:id="rId1"/>
@@ -2044,6 +2044,11 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2059,11 +2064,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3138,17 +3138,17 @@
       <c r="L1" s="40"/>
       <c r="M1" s="40"/>
       <c r="N1" s="41"/>
-      <c r="O1" s="50" t="s">
+      <c r="O1" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="P1" s="51"/>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="51"/>
-      <c r="S1" s="51"/>
-      <c r="T1" s="51"/>
-      <c r="U1" s="51"/>
-      <c r="V1" s="51"/>
-      <c r="W1" s="52"/>
+      <c r="P1" s="54"/>
+      <c r="Q1" s="54"/>
+      <c r="R1" s="54"/>
+      <c r="S1" s="54"/>
+      <c r="T1" s="54"/>
+      <c r="U1" s="54"/>
+      <c r="V1" s="54"/>
+      <c r="W1" s="55"/>
       <c r="X1" s="39" t="s">
         <v>57</v>
       </c>
@@ -3161,17 +3161,17 @@
       <c r="AE1" s="40"/>
       <c r="AF1" s="40"/>
       <c r="AG1" s="41"/>
-      <c r="AH1" s="47" t="s">
+      <c r="AH1" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="AI1" s="48"/>
-      <c r="AJ1" s="48"/>
-      <c r="AK1" s="48"/>
-      <c r="AL1" s="48"/>
-      <c r="AM1" s="48"/>
-      <c r="AN1" s="48"/>
-      <c r="AO1" s="48"/>
-      <c r="AP1" s="49"/>
+      <c r="AI1" s="51"/>
+      <c r="AJ1" s="51"/>
+      <c r="AK1" s="51"/>
+      <c r="AL1" s="51"/>
+      <c r="AM1" s="51"/>
+      <c r="AN1" s="51"/>
+      <c r="AO1" s="51"/>
+      <c r="AP1" s="52"/>
     </row>
     <row r="2" spans="1:42" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
@@ -3183,69 +3183,69 @@
       <c r="E2" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="53" t="s">
+      <c r="F2" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="54"/>
-      <c r="H2" s="55"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="46"/>
       <c r="I2" s="43" t="s">
         <v>62</v>
       </c>
       <c r="J2" s="40"/>
       <c r="K2" s="41"/>
-      <c r="L2" s="44" t="s">
+      <c r="L2" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="M2" s="45"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="53" t="s">
+      <c r="M2" s="48"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="44" t="s">
         <v>64</v>
       </c>
-      <c r="P2" s="54"/>
-      <c r="Q2" s="55"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="46"/>
       <c r="R2" s="43" t="s">
         <v>65</v>
       </c>
       <c r="S2" s="40"/>
       <c r="T2" s="41"/>
-      <c r="U2" s="44" t="s">
+      <c r="U2" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="V2" s="45"/>
-      <c r="W2" s="46"/>
+      <c r="V2" s="48"/>
+      <c r="W2" s="49"/>
       <c r="X2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="Y2" s="53" t="s">
+      <c r="Y2" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="Z2" s="54"/>
-      <c r="AA2" s="55"/>
+      <c r="Z2" s="45"/>
+      <c r="AA2" s="46"/>
       <c r="AB2" s="43" t="s">
         <v>62</v>
       </c>
       <c r="AC2" s="40"/>
       <c r="AD2" s="41"/>
-      <c r="AE2" s="44" t="s">
+      <c r="AE2" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="AF2" s="45"/>
-      <c r="AG2" s="46"/>
-      <c r="AH2" s="53" t="s">
+      <c r="AF2" s="48"/>
+      <c r="AG2" s="49"/>
+      <c r="AH2" s="44" t="s">
         <v>64</v>
       </c>
-      <c r="AI2" s="54"/>
-      <c r="AJ2" s="55"/>
+      <c r="AI2" s="45"/>
+      <c r="AJ2" s="46"/>
       <c r="AK2" s="43" t="s">
         <v>65</v>
       </c>
       <c r="AL2" s="40"/>
       <c r="AM2" s="41"/>
-      <c r="AN2" s="44" t="s">
+      <c r="AN2" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="AO2" s="45"/>
-      <c r="AP2" s="46"/>
+      <c r="AO2" s="48"/>
+      <c r="AP2" s="49"/>
     </row>
     <row r="3" spans="1:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -4075,14 +4075,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="AB2:AD2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="Y2:AA2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="E1:N1"/>
     <mergeCell ref="AE2:AG2"/>
     <mergeCell ref="AH1:AP1"/>
     <mergeCell ref="R2:T2"/>
@@ -4093,6 +4085,14 @@
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="AH2:AJ2"/>
     <mergeCell ref="U2:W2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="AB2:AD2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="Y2:AA2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="E1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4783,7 +4783,7 @@
     </row>
     <row r="4" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>121</v>
@@ -5006,7 +5006,7 @@
     </row>
     <row r="5" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B5" s="21" t="s">
         <v>51</v>
@@ -5363,14 +5363,14 @@
       <c r="K1" s="40"/>
       <c r="L1" s="40"/>
       <c r="M1" s="40"/>
-      <c r="N1" s="50" t="s">
+      <c r="N1" s="53" t="s">
         <v>452</v>
       </c>
       <c r="O1" s="73"/>
-      <c r="P1" s="51"/>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="51"/>
-      <c r="S1" s="51"/>
+      <c r="P1" s="54"/>
+      <c r="Q1" s="54"/>
+      <c r="R1" s="54"/>
+      <c r="S1" s="54"/>
       <c r="T1" s="43" t="s">
         <v>270</v>
       </c>

</xml_diff>

<commit_message>
Module 3 part 1 doesn't work properly
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0590DD7F-C571-44A2-A12D-A2232026DB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F8C20A2-FDFB-4489-8D2E-585D446FFEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Проект" sheetId="1" r:id="rId1"/>
@@ -4783,7 +4783,7 @@
     </row>
     <row r="4" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>121</v>
@@ -5006,7 +5006,7 @@
     </row>
     <row r="5" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B5" s="21" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
Module 3 part 1 still doesn't work properly. It seems to me that the problem is in module 2 part 2, frames nodes have wrong coordinates. And pod 2 has wrong nodes
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F8C20A2-FDFB-4489-8D2E-585D446FFEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B5CE8E-F159-401C-A32B-C1E7C6C5A4A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="494">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="496">
   <si>
     <t>Параметр</t>
   </si>
@@ -70,9 +70,6 @@
   </si>
   <si>
     <t>* Все отметки Z — от низа ростверка (Z = 0 = подошва ростверка)</t>
-  </si>
-  <si>
-    <t>* Сейсмическое воздействие (*SFUNCTION и др.) задаётся в Midas Civil вручную</t>
   </si>
   <si>
     <t>* Формулы на листе "Массы" должны быть пересчитаны в Excel перед запуском скрипта</t>
@@ -195,9 +192,6 @@
     <t>* Строку-разделитель "Плеть N" вставляйте перед первой опорой каждой плети.</t>
   </si>
   <si>
-    <t>* bearing_X / bearing_Y: "fixed" или "movable". μ задаётся только для movable.</t>
-  </si>
-  <si>
     <t>ОЧ СПРАВА — Постоянная нагрузка</t>
   </si>
   <si>
@@ -405,18 +399,6 @@
   </si>
   <si>
     <t>O4</t>
-  </si>
-  <si>
-    <t>* C/D = строки начала и конца плети на листе "Плеть". Одна строка на опору -&gt; C = D.</t>
-  </si>
-  <si>
-    <t>* Z-отметки общие для обеих ОЧ — берутся из столбцов B/C/D листа "Плеть".</t>
-  </si>
-  <si>
-    <t>* mX: bearing_X="fixed" -&gt; ΣR_пост всей плети/g;  "movable" -&gt; ΣR_пост×μX/g.</t>
-  </si>
-  <si>
-    <t>* mY=R_пост×μY/g (z_cg). mZ=R_пост/g (z_cg). Временные — к z_road.</t>
   </si>
   <si>
     <t>* Зелёные ячейки считаются автоматически. Копируйте строку 5 для каждой новой опоры.</t>
@@ -1609,6 +1591,46 @@
   </si>
   <si>
     <t>cap_sec_2_width</t>
+  </si>
+  <si>
+    <t>Пока алгоритм работает только для обычных опорных частей (не сейсмических)</t>
+  </si>
+  <si>
+    <t>В базовом файле .mcb должно быть задано следующее:
+- Сейсмическое воздействие.
+- Материалы и сечения. Рекомендуется в файле шаблона для проекта задать все материалы и сечения для всего проекта. Собственный вес материалов должен быть с коэф. надежности
+- Параметры eigenvalues.
+- В Structure Type должен быть включен учет собственного веса
+- Group damping, если есть.
+- Должны быть заданы лоадкейсы: 
+     SW (задать в него собственный вес схемы)
+     Permanent (для постоянных нагрузок)
+    Temporary (для временных нагрузок)
+- Сочетания нагрузок</t>
+  </si>
+  <si>
+    <t>Вдоль (X)
+fixed/movable</t>
+  </si>
+  <si>
+    <t>Поперёк (Y)
+fixed/movable</t>
+  </si>
+  <si>
+    <t>Строка
+начала плети
+на листе "Плеть"</t>
+  </si>
+  <si>
+    <t>Строка
+конца плети
+на листе "Плеть"</t>
+  </si>
+  <si>
+    <t>Массы чвычисляются в соответствии с п. 8.3.23 и 8.3.24 СП 268.1325800.2016</t>
+  </si>
+  <si>
+    <t>это не работает</t>
   </si>
 </sst>
 </file>
@@ -1925,7 +1947,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2001,13 +2023,17 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2016,10 +2042,9 @@
     <xf numFmtId="164" fontId="7" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2044,11 +2069,6 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2064,6 +2084,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2136,6 +2161,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>496737</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>48327</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Рисунок 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0BAE4AB-0BCA-E19A-7D0D-D4DEA5A419E7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="3324225"/>
+          <a:ext cx="10297962" cy="5029902"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2423,7 +2497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -2457,7 +2531,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2488,38 +2562,67 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C6" s="23" t="s">
+        <v>310</v>
+      </c>
+      <c r="D6" s="22"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="34" t="s">
+        <v>488</v>
+      </c>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+    </row>
+    <row r="8" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="23" t="s">
-        <v>316</v>
-      </c>
-      <c r="D6" s="22"/>
-    </row>
-    <row r="7" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+    </row>
+    <row r="9" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="34" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+    </row>
+    <row r="10" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="34" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="33.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>16</v>
-      </c>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+    </row>
+    <row r="11" spans="1:4" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="34" t="s">
+        <v>489</v>
+      </c>
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A7:D7"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2535,186 +2638,186 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="42" t="s">
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="40"/>
-      <c r="P1" s="40"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="41"/>
+      <c r="P1" s="41"/>
     </row>
     <row r="2" spans="1:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="40" t="s">
+        <v>305</v>
+      </c>
+      <c r="C2" s="41"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="39" t="s">
-        <v>311</v>
-      </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="42" t="s">
+      <c r="F2" s="41"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="40"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="43" t="s">
+      <c r="I2" s="42"/>
+      <c r="J2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="41"/>
-      <c r="J2" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" s="39" t="s">
+      <c r="K2" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="41"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="L2" s="40"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="43" t="s">
+      <c r="O2" s="42"/>
+      <c r="P2" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="O2" s="41"/>
-      <c r="P2" s="8" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>422</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>423</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>424</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="P3" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
+        <v>455</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>461</v>
-      </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="L4" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="M4" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="N4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="O4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="P4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="9" t="s">
+    </row>
+    <row r="5" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="K4" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="L4" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="O4" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="34" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="38"/>
-      <c r="I5" s="38"/>
-      <c r="J5" s="38"/>
-      <c r="K5" s="38"/>
-      <c r="L5" s="38"/>
-      <c r="M5" s="38"/>
-      <c r="N5" s="38"/>
-      <c r="O5" s="38"/>
-      <c r="P5" s="38"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="39"/>
+      <c r="I5" s="39"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="39"/>
+      <c r="L5" s="39"/>
+      <c r="M5" s="39"/>
+      <c r="N5" s="39"/>
+      <c r="O5" s="39"/>
+      <c r="P5" s="39"/>
     </row>
     <row r="6" spans="1:16" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" s="21">
         <v>49.19</v>
@@ -2729,10 +2832,10 @@
         <v>1</v>
       </c>
       <c r="F6" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="21" t="s">
         <v>48</v>
-      </c>
-      <c r="G6" s="21" t="s">
-        <v>49</v>
       </c>
       <c r="H6" s="21">
         <v>950</v>
@@ -2748,10 +2851,10 @@
         <v>2</v>
       </c>
       <c r="L6" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M6" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N6" s="21">
         <v>870</v>
@@ -2766,7 +2869,7 @@
     </row>
     <row r="7" spans="1:16" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" s="21">
         <v>12.18</v>
@@ -2781,10 +2884,10 @@
         <v>1</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H7" s="21">
         <v>820</v>
@@ -2800,10 +2903,10 @@
         <v>2</v>
       </c>
       <c r="L7" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M7" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N7" s="21">
         <v>647</v>
@@ -2818,7 +2921,7 @@
     </row>
     <row r="8" spans="1:16" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" s="21">
         <v>49.19</v>
@@ -2833,10 +2936,10 @@
         <v>1</v>
       </c>
       <c r="F8" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="21" t="s">
         <v>48</v>
-      </c>
-      <c r="G8" s="21" t="s">
-        <v>49</v>
       </c>
       <c r="H8" s="21">
         <v>950</v>
@@ -2852,10 +2955,10 @@
         <v>2</v>
       </c>
       <c r="L8" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M8" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N8" s="21">
         <v>870</v>
@@ -2869,28 +2972,28 @@
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
-        <v>309</v>
-      </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="35"/>
-      <c r="L9" s="35"/>
-      <c r="M9" s="35"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="35"/>
-      <c r="P9" s="35"/>
+      <c r="A9" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="36"/>
+      <c r="K9" s="36"/>
+      <c r="L9" s="36"/>
+      <c r="M9" s="36"/>
+      <c r="N9" s="36"/>
+      <c r="O9" s="36"/>
+      <c r="P9" s="36"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B10" s="21">
         <v>12.18</v>
@@ -2905,10 +3008,10 @@
         <v>3</v>
       </c>
       <c r="F10" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="21" t="s">
         <v>48</v>
-      </c>
-      <c r="G10" s="21" t="s">
-        <v>49</v>
       </c>
       <c r="H10" s="21">
         <v>920</v>
@@ -2924,10 +3027,10 @@
         <v>4</v>
       </c>
       <c r="L10" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M10" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N10" s="21">
         <v>880</v>
@@ -2942,7 +3045,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B11" s="21">
         <v>12.18</v>
@@ -2957,10 +3060,10 @@
         <v>1</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H11" s="21">
         <v>820</v>
@@ -2976,10 +3079,10 @@
         <v>2</v>
       </c>
       <c r="L11" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M11" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N11" s="21">
         <v>647</v>
@@ -2994,7 +3097,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="B12" s="21">
         <v>49.19</v>
@@ -3009,10 +3112,10 @@
         <v>1</v>
       </c>
       <c r="F12" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="21" t="s">
         <v>48</v>
-      </c>
-      <c r="G12" s="21" t="s">
-        <v>49</v>
       </c>
       <c r="H12" s="21">
         <v>950</v>
@@ -3028,10 +3131,10 @@
         <v>2</v>
       </c>
       <c r="L12" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M12" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N12" s="21">
         <v>870</v>
@@ -3044,26 +3147,33 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+    <row r="14" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="F14" s="18" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="F15" s="18" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="67.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>54</v>
-      </c>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A9:P9"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:P5"/>
@@ -3081,7 +3191,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AP13"/>
+  <dimension ref="A1:AP10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -3120,392 +3230,392 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:42" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="42" t="s">
+      <c r="A1" s="40" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="51" t="s">
+        <v>54</v>
+      </c>
+      <c r="P1" s="52"/>
+      <c r="Q1" s="52"/>
+      <c r="R1" s="52"/>
+      <c r="S1" s="52"/>
+      <c r="T1" s="52"/>
+      <c r="U1" s="52"/>
+      <c r="V1" s="52"/>
+      <c r="W1" s="53"/>
+      <c r="X1" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="41"/>
-      <c r="O1" s="53" t="s">
+      <c r="Y1" s="41"/>
+      <c r="Z1" s="41"/>
+      <c r="AA1" s="41"/>
+      <c r="AB1" s="41"/>
+      <c r="AC1" s="41"/>
+      <c r="AD1" s="41"/>
+      <c r="AE1" s="41"/>
+      <c r="AF1" s="41"/>
+      <c r="AG1" s="42"/>
+      <c r="AH1" s="48" t="s">
         <v>56</v>
       </c>
-      <c r="P1" s="54"/>
-      <c r="Q1" s="54"/>
-      <c r="R1" s="54"/>
-      <c r="S1" s="54"/>
-      <c r="T1" s="54"/>
-      <c r="U1" s="54"/>
-      <c r="V1" s="54"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="39" t="s">
+      <c r="AI1" s="49"/>
+      <c r="AJ1" s="49"/>
+      <c r="AK1" s="49"/>
+      <c r="AL1" s="49"/>
+      <c r="AM1" s="49"/>
+      <c r="AN1" s="49"/>
+      <c r="AO1" s="49"/>
+      <c r="AP1" s="50"/>
+    </row>
+    <row r="2" spans="1:42" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="40" t="s">
         <v>57</v>
       </c>
-      <c r="Y1" s="40"/>
-      <c r="Z1" s="40"/>
-      <c r="AA1" s="40"/>
-      <c r="AB1" s="40"/>
-      <c r="AC1" s="40"/>
-      <c r="AD1" s="40"/>
-      <c r="AE1" s="40"/>
-      <c r="AF1" s="40"/>
-      <c r="AG1" s="41"/>
-      <c r="AH1" s="50" t="s">
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AI1" s="51"/>
-      <c r="AJ1" s="51"/>
-      <c r="AK1" s="51"/>
-      <c r="AL1" s="51"/>
-      <c r="AM1" s="51"/>
-      <c r="AN1" s="51"/>
-      <c r="AO1" s="51"/>
-      <c r="AP1" s="52"/>
-    </row>
-    <row r="2" spans="1:42" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="F2" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="7" t="s">
+      <c r="G2" s="55"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="44" t="s">
+      <c r="J2" s="41"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="45"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="43" t="s">
+      <c r="M2" s="46"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="J2" s="40"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="47" t="s">
+      <c r="P2" s="55"/>
+      <c r="Q2" s="56"/>
+      <c r="R2" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="M2" s="48"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="44" t="s">
+      <c r="S2" s="41"/>
+      <c r="T2" s="42"/>
+      <c r="U2" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="46"/>
-      <c r="R2" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="S2" s="40"/>
-      <c r="T2" s="41"/>
-      <c r="U2" s="47" t="s">
-        <v>66</v>
-      </c>
-      <c r="V2" s="48"/>
-      <c r="W2" s="49"/>
+      <c r="V2" s="46"/>
+      <c r="W2" s="47"/>
       <c r="X2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y2" s="54" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z2" s="55"/>
+      <c r="AA2" s="56"/>
+      <c r="AB2" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="Y2" s="44" t="s">
+      <c r="AC2" s="41"/>
+      <c r="AD2" s="42"/>
+      <c r="AE2" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="Z2" s="45"/>
-      <c r="AA2" s="46"/>
-      <c r="AB2" s="43" t="s">
+      <c r="AF2" s="46"/>
+      <c r="AG2" s="47"/>
+      <c r="AH2" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="AC2" s="40"/>
-      <c r="AD2" s="41"/>
-      <c r="AE2" s="47" t="s">
+      <c r="AI2" s="55"/>
+      <c r="AJ2" s="56"/>
+      <c r="AK2" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="AF2" s="48"/>
-      <c r="AG2" s="49"/>
-      <c r="AH2" s="44" t="s">
+      <c r="AL2" s="41"/>
+      <c r="AM2" s="42"/>
+      <c r="AN2" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="AI2" s="45"/>
-      <c r="AJ2" s="46"/>
-      <c r="AK2" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="AL2" s="40"/>
-      <c r="AM2" s="41"/>
-      <c r="AN2" s="47" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO2" s="48"/>
-      <c r="AP2" s="49"/>
+      <c r="AO2" s="46"/>
+      <c r="AP2" s="47"/>
     </row>
     <row r="3" spans="1:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="P3" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="Q3" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="P3" s="3" t="s">
+      <c r="R3" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="S3" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="T3" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="U3" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="V3" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="W3" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="V3" s="3" t="s">
+      <c r="X3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y3" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="W3" s="3" t="s">
+      <c r="Z3" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="X3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Y3" s="3" t="s">
+      <c r="AA3" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="Z3" s="3" t="s">
+      <c r="AB3" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="AA3" s="3" t="s">
+      <c r="AC3" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="AB3" s="3" t="s">
+      <c r="AD3" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="AC3" s="3" t="s">
+      <c r="AE3" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="AD3" s="3" t="s">
+      <c r="AF3" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="AE3" s="3" t="s">
+      <c r="AG3" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="AF3" s="3" t="s">
+      <c r="AH3" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="AG3" s="3" t="s">
+      <c r="AI3" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AH3" s="3" t="s">
+      <c r="AJ3" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="AI3" s="3" t="s">
+      <c r="AK3" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="AJ3" s="3" t="s">
+      <c r="AL3" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="AK3" s="3" t="s">
+      <c r="AM3" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="AL3" s="3" t="s">
+      <c r="AN3" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="AM3" s="3" t="s">
+      <c r="AO3" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="AN3" s="3" t="s">
+      <c r="AP3" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="AO3" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="AP3" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:42" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:42" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>492</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>493</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="J4" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="K4" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="L4" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="M4" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="N4" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="O4" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="P4" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q4" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="R4" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="N4" s="9" t="s">
+      <c r="S4" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="T4" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="U4" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="V4" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="W4" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="X4" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="Y4" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z4" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="AA4" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB4" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="AC4" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD4" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="AE4" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="AF4" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="AG4" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="AH4" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI4" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="AJ4" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="AK4" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="AL4" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="AM4" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="P4" s="9" t="s">
+      <c r="AN4" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="AO4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="Q4" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="R4" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="S4" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="T4" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="U4" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="V4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="W4" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="X4" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="Y4" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="Z4" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA4" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AB4" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="AC4" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="AD4" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AE4" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="AF4" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="AG4" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AH4" s="9" t="s">
+      <c r="AP4" s="9" t="s">
         <v>117</v>
-      </c>
-      <c r="AI4" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="AJ4" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AK4" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="AL4" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="AM4" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="AN4" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="AO4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="AP4" s="9" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:42" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B5" s="11">
         <f>Проект!$D$3</f>
@@ -3672,7 +3782,7 @@
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="11">
         <f>Проект!$D$3</f>
@@ -3839,7 +3949,7 @@
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B7" s="11">
         <f>Проект!$D$3</f>
@@ -4005,76 +4115,73 @@
       </c>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="A8" s="27"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-      <c r="M8" s="31"/>
-      <c r="N8" s="30"/>
-      <c r="O8" s="30"/>
-      <c r="P8" s="31"/>
-      <c r="Q8" s="30"/>
-      <c r="R8" s="30"/>
-      <c r="S8" s="31"/>
-      <c r="T8" s="30"/>
-      <c r="U8" s="30"/>
-      <c r="V8" s="31"/>
-      <c r="W8" s="30"/>
-      <c r="X8" s="28"/>
-      <c r="Y8" s="30"/>
-      <c r="Z8" s="31"/>
-      <c r="AA8" s="30"/>
-      <c r="AB8" s="30"/>
-      <c r="AC8" s="31"/>
-      <c r="AD8" s="30"/>
-      <c r="AE8" s="30"/>
-      <c r="AF8" s="31"/>
-      <c r="AG8" s="30"/>
-      <c r="AH8" s="30"/>
-      <c r="AI8" s="31"/>
-      <c r="AJ8" s="30"/>
-      <c r="AK8" s="30"/>
-      <c r="AL8" s="31"/>
-      <c r="AM8" s="30"/>
-      <c r="AN8" s="30"/>
-      <c r="AO8" s="31"/>
-      <c r="AP8" s="30"/>
-    </row>
-    <row r="9" spans="1:42" ht="67.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="10" spans="1:42" ht="67.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="11" spans="1:42" ht="67.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="12" spans="1:42" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="13" spans="1:42" ht="90" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>126</v>
-      </c>
+      <c r="A8" s="29"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="32"/>
+      <c r="L8" s="32"/>
+      <c r="M8" s="33"/>
+      <c r="N8" s="32"/>
+      <c r="O8" s="32"/>
+      <c r="P8" s="33"/>
+      <c r="Q8" s="32"/>
+      <c r="R8" s="32"/>
+      <c r="S8" s="33"/>
+      <c r="T8" s="32"/>
+      <c r="U8" s="32"/>
+      <c r="V8" s="33"/>
+      <c r="W8" s="32"/>
+      <c r="X8" s="31"/>
+      <c r="Y8" s="32"/>
+      <c r="Z8" s="33"/>
+      <c r="AA8" s="32"/>
+      <c r="AB8" s="32"/>
+      <c r="AC8" s="33"/>
+      <c r="AD8" s="32"/>
+      <c r="AE8" s="32"/>
+      <c r="AF8" s="33"/>
+      <c r="AG8" s="32"/>
+      <c r="AH8" s="32"/>
+      <c r="AI8" s="33"/>
+      <c r="AJ8" s="32"/>
+      <c r="AK8" s="32"/>
+      <c r="AL8" s="33"/>
+      <c r="AM8" s="32"/>
+      <c r="AN8" s="32"/>
+      <c r="AO8" s="33"/>
+      <c r="AP8" s="32"/>
+    </row>
+    <row r="9" spans="1:42" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+    </row>
+    <row r="10" spans="1:42" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="34" t="s">
+        <v>494</v>
+      </c>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="20">
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="E1:N1"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="AE2:AG2"/>
     <mergeCell ref="AH1:AP1"/>
     <mergeCell ref="R2:T2"/>
@@ -4089,12 +4196,9 @@
     <mergeCell ref="AB2:AD2"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="Y2:AA2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="E1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4108,688 +4212,688 @@
   <sheetData>
     <row r="1" spans="1:93" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>425</v>
-      </c>
-      <c r="B1" s="42" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="61" t="s">
-        <v>128</v>
-      </c>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="63"/>
-      <c r="T1" s="43" t="s">
-        <v>129</v>
-      </c>
-      <c r="U1" s="40"/>
-      <c r="V1" s="40"/>
-      <c r="W1" s="40"/>
-      <c r="X1" s="40"/>
-      <c r="Y1" s="40"/>
-      <c r="Z1" s="40"/>
-      <c r="AA1" s="40"/>
-      <c r="AB1" s="40"/>
-      <c r="AC1" s="41"/>
-      <c r="AD1" s="39" t="s">
-        <v>130</v>
-      </c>
-      <c r="AE1" s="40"/>
-      <c r="AF1" s="40"/>
-      <c r="AG1" s="40"/>
-      <c r="AH1" s="40"/>
-      <c r="AI1" s="40"/>
-      <c r="AJ1" s="40"/>
-      <c r="AK1" s="40"/>
-      <c r="AL1" s="40"/>
-      <c r="AM1" s="40"/>
-      <c r="AN1" s="40"/>
-      <c r="AO1" s="40"/>
-      <c r="AP1" s="40"/>
-      <c r="AQ1" s="41"/>
-      <c r="AR1" s="58" t="s">
-        <v>131</v>
-      </c>
-      <c r="AS1" s="59"/>
-      <c r="AT1" s="59"/>
-      <c r="AU1" s="59"/>
-      <c r="AV1" s="59"/>
-      <c r="AW1" s="59"/>
-      <c r="AX1" s="59"/>
-      <c r="AY1" s="59"/>
-      <c r="AZ1" s="59"/>
-      <c r="BA1" s="59"/>
-      <c r="BB1" s="59"/>
-      <c r="BC1" s="59"/>
-      <c r="BD1" s="59"/>
-      <c r="BE1" s="59"/>
-      <c r="BF1" s="59"/>
-      <c r="BG1" s="59"/>
-      <c r="BH1" s="59"/>
-      <c r="BI1" s="60"/>
-      <c r="BJ1" s="43" t="s">
-        <v>132</v>
-      </c>
-      <c r="BK1" s="40"/>
-      <c r="BL1" s="40"/>
-      <c r="BM1" s="40"/>
-      <c r="BN1" s="40"/>
-      <c r="BO1" s="40"/>
-      <c r="BP1" s="40"/>
-      <c r="BQ1" s="40"/>
-      <c r="BR1" s="40"/>
-      <c r="BS1" s="40"/>
-      <c r="BT1" s="40"/>
-      <c r="BU1" s="40"/>
-      <c r="BV1" s="40"/>
-      <c r="BW1" s="41"/>
-      <c r="BX1" s="42" t="s">
-        <v>127</v>
-      </c>
-      <c r="BY1" s="40"/>
-      <c r="BZ1" s="40"/>
-      <c r="CA1" s="40"/>
-      <c r="CB1" s="40"/>
-      <c r="CC1" s="40"/>
-      <c r="CD1" s="40"/>
-      <c r="CE1" s="40"/>
-      <c r="CF1" s="40"/>
-      <c r="CG1" s="40"/>
-      <c r="CH1" s="40"/>
-      <c r="CI1" s="40"/>
-      <c r="CJ1" s="40"/>
-      <c r="CK1" s="41"/>
-      <c r="CL1" s="56" t="s">
-        <v>433</v>
-      </c>
-      <c r="CM1" s="57"/>
-      <c r="CN1" s="57"/>
-      <c r="CO1" s="57"/>
+        <v>419</v>
+      </c>
+      <c r="B1" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="62" t="s">
+        <v>122</v>
+      </c>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="63"/>
+      <c r="R1" s="63"/>
+      <c r="S1" s="64"/>
+      <c r="T1" s="44" t="s">
+        <v>123</v>
+      </c>
+      <c r="U1" s="41"/>
+      <c r="V1" s="41"/>
+      <c r="W1" s="41"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="41"/>
+      <c r="Z1" s="41"/>
+      <c r="AA1" s="41"/>
+      <c r="AB1" s="41"/>
+      <c r="AC1" s="42"/>
+      <c r="AD1" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="AE1" s="41"/>
+      <c r="AF1" s="41"/>
+      <c r="AG1" s="41"/>
+      <c r="AH1" s="41"/>
+      <c r="AI1" s="41"/>
+      <c r="AJ1" s="41"/>
+      <c r="AK1" s="41"/>
+      <c r="AL1" s="41"/>
+      <c r="AM1" s="41"/>
+      <c r="AN1" s="41"/>
+      <c r="AO1" s="41"/>
+      <c r="AP1" s="41"/>
+      <c r="AQ1" s="42"/>
+      <c r="AR1" s="59" t="s">
+        <v>125</v>
+      </c>
+      <c r="AS1" s="60"/>
+      <c r="AT1" s="60"/>
+      <c r="AU1" s="60"/>
+      <c r="AV1" s="60"/>
+      <c r="AW1" s="60"/>
+      <c r="AX1" s="60"/>
+      <c r="AY1" s="60"/>
+      <c r="AZ1" s="60"/>
+      <c r="BA1" s="60"/>
+      <c r="BB1" s="60"/>
+      <c r="BC1" s="60"/>
+      <c r="BD1" s="60"/>
+      <c r="BE1" s="60"/>
+      <c r="BF1" s="60"/>
+      <c r="BG1" s="60"/>
+      <c r="BH1" s="60"/>
+      <c r="BI1" s="61"/>
+      <c r="BJ1" s="44" t="s">
+        <v>126</v>
+      </c>
+      <c r="BK1" s="41"/>
+      <c r="BL1" s="41"/>
+      <c r="BM1" s="41"/>
+      <c r="BN1" s="41"/>
+      <c r="BO1" s="41"/>
+      <c r="BP1" s="41"/>
+      <c r="BQ1" s="41"/>
+      <c r="BR1" s="41"/>
+      <c r="BS1" s="41"/>
+      <c r="BT1" s="41"/>
+      <c r="BU1" s="41"/>
+      <c r="BV1" s="41"/>
+      <c r="BW1" s="42"/>
+      <c r="BX1" s="43" t="s">
+        <v>121</v>
+      </c>
+      <c r="BY1" s="41"/>
+      <c r="BZ1" s="41"/>
+      <c r="CA1" s="41"/>
+      <c r="CB1" s="41"/>
+      <c r="CC1" s="41"/>
+      <c r="CD1" s="41"/>
+      <c r="CE1" s="41"/>
+      <c r="CF1" s="41"/>
+      <c r="CG1" s="41"/>
+      <c r="CH1" s="41"/>
+      <c r="CI1" s="41"/>
+      <c r="CJ1" s="41"/>
+      <c r="CK1" s="42"/>
+      <c r="CL1" s="57" t="s">
+        <v>427</v>
+      </c>
+      <c r="CM1" s="58"/>
+      <c r="CN1" s="58"/>
+      <c r="CO1" s="58"/>
     </row>
     <row r="2" spans="1:93" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="R2" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="T2" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="U2" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="V2" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="W2" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="X2" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Y2" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="R2" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="T2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="AA2" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="V2" s="3" t="s">
+      <c r="AB2" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="W2" s="3" t="s">
+      <c r="AC2" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="AD2" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="Y2" s="3" t="s">
+      <c r="AE2" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="Z2" s="3" t="s">
+      <c r="AF2" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="AA2" s="3" t="s">
+      <c r="AG2" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="AB2" s="3" t="s">
+      <c r="AH2" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AI2" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="AD2" s="3" t="s">
+      <c r="AJ2" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="AE2" s="3" t="s">
+      <c r="AK2" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="AF2" s="3" t="s">
+      <c r="AL2" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="AG2" s="3" t="s">
+      <c r="AM2" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="AH2" s="3" t="s">
+      <c r="AN2" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="AI2" s="3" t="s">
+      <c r="AO2" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="AJ2" s="3" t="s">
+      <c r="AP2" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="AK2" s="3" t="s">
+      <c r="AQ2" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="AL2" s="3" t="s">
+      <c r="AR2" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="AM2" s="3" t="s">
+      <c r="AS2" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="AN2" s="3" t="s">
+      <c r="AT2" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="AO2" s="3" t="s">
+      <c r="AU2" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="AP2" s="3" t="s">
+      <c r="AV2" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="AQ2" s="3" t="s">
+      <c r="AW2" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="AR2" s="3" t="s">
+      <c r="AX2" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="AS2" s="3" t="s">
+      <c r="AY2" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="AT2" s="3" t="s">
+      <c r="AZ2" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="AU2" s="3" t="s">
+      <c r="BA2" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="AV2" s="3" t="s">
+      <c r="BB2" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="AW2" s="3" t="s">
+      <c r="BC2" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="AX2" s="3" t="s">
+      <c r="BD2" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="AY2" s="3" t="s">
+      <c r="BE2" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="AZ2" s="3" t="s">
+      <c r="BF2" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="BA2" s="3" t="s">
+      <c r="BG2" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="BB2" s="3" t="s">
+      <c r="BH2" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="BC2" s="3" t="s">
+      <c r="BI2" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="BD2" s="3" t="s">
+      <c r="BJ2" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="BE2" s="3" t="s">
+      <c r="BK2" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="BL2" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="BM2" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="BF2" s="3" t="s">
+      <c r="BN2" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="BG2" s="3" t="s">
+      <c r="BO2" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="BH2" s="3" t="s">
+      <c r="BP2" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="BI2" s="3" t="s">
+      <c r="BQ2" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="BJ2" s="3" t="s">
+      <c r="BR2" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="BK2" s="3" t="s">
-        <v>455</v>
-      </c>
-      <c r="BL2" s="3" t="s">
-        <v>456</v>
-      </c>
-      <c r="BM2" s="3" t="s">
+      <c r="BS2" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="BN2" s="3" t="s">
+      <c r="BT2" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="BO2" s="3" t="s">
+      <c r="BU2" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="BP2" s="3" t="s">
+      <c r="BV2" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="BQ2" s="3" t="s">
+      <c r="BW2" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="BR2" s="3" t="s">
+      <c r="BX2" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="BS2" s="3" t="s">
+      <c r="BY2" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="BZ2" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="CA2" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="BT2" s="3" t="s">
+      <c r="CB2" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="BU2" s="3" t="s">
+      <c r="CC2" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="BV2" s="3" t="s">
+      <c r="CD2" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="BW2" s="3" t="s">
+      <c r="CE2" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="BX2" s="3" t="s">
+      <c r="CF2" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="BY2" s="3" t="s">
-        <v>459</v>
-      </c>
-      <c r="BZ2" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="CA2" s="3" t="s">
+      <c r="CG2" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="CB2" s="3" t="s">
+      <c r="CH2" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="CC2" s="3" t="s">
+      <c r="CI2" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="CD2" s="3" t="s">
+      <c r="CJ2" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="CE2" s="3" t="s">
+      <c r="CK2" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="CF2" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="CG2" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="CH2" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="CI2" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="CJ2" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="CK2" s="3" t="s">
-        <v>211</v>
-      </c>
       <c r="CL2" s="3" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="CM2" s="3" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="CN2" s="3" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="CO2" s="3" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
     </row>
     <row r="3" spans="1:93" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="K3" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="D3" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="F3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="N3" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="P3" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="Q3" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="R3" s="9" t="s">
+        <v>436</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="T3" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="U3" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="V3" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="W3" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="X3" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="Y3" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="Z3" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="R3" s="9" t="s">
-        <v>442</v>
-      </c>
-      <c r="S3" s="9" t="s">
-        <v>443</v>
-      </c>
-      <c r="T3" s="9" t="s">
+      <c r="AA3" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="U3" s="9" t="s">
+      <c r="AB3" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="V3" s="9" t="s">
+      <c r="AC3" s="9" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD3" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="W3" s="9" t="s">
+      <c r="AE3" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="AF3" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="AG3" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="AH3" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="AI3" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="AJ3" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="AK3" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="AL3" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="AM3" s="9" t="s">
+        <v>475</v>
+      </c>
+      <c r="AN3" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="X3" s="9" t="s">
+      <c r="AO3" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="Y3" s="9" t="s">
-        <v>480</v>
-      </c>
-      <c r="Z3" s="9" t="s">
+      <c r="AP3" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="AA3" s="9" t="s">
+      <c r="AQ3" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="AR3" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="AB3" s="9" t="s">
+      <c r="AS3" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="AT3" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="AU3" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="AV3" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="AW3" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="AX3" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="AY3" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="AZ3" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="BA3" s="9" t="s">
+        <v>475</v>
+      </c>
+      <c r="BB3" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="BC3" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="BD3" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="BE3" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="BF3" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="AC3" s="9" t="s">
-        <v>481</v>
-      </c>
-      <c r="AD3" s="9" t="s">
+      <c r="BG3" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="AE3" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="AF3" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="AG3" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="AH3" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="AI3" s="9" t="s">
-        <v>480</v>
-      </c>
-      <c r="AJ3" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="AK3" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="AL3" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="AM3" s="9" t="s">
-        <v>481</v>
-      </c>
-      <c r="AN3" s="9" t="s">
+      <c r="BH3" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="AO3" s="9" t="s">
+      <c r="BI3" s="9" t="s">
+        <v>477</v>
+      </c>
+      <c r="BJ3" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="AP3" s="9" t="s">
+      <c r="BK3" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="BL3" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="BM3" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="AQ3" s="9" t="s">
-        <v>482</v>
-      </c>
-      <c r="AR3" s="9" t="s">
+      <c r="BN3" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="AS3" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="AT3" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="AU3" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="AV3" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="AW3" s="9" t="s">
-        <v>480</v>
-      </c>
-      <c r="AX3" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="AY3" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="AZ3" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="BA3" s="9" t="s">
-        <v>481</v>
-      </c>
-      <c r="BB3" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="BC3" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="BD3" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="BE3" s="9" t="s">
-        <v>482</v>
-      </c>
-      <c r="BF3" s="9" t="s">
+      <c r="BO3" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="BG3" s="9" t="s">
+      <c r="BP3" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="BH3" s="9" t="s">
+      <c r="BQ3" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="BI3" s="9" t="s">
-        <v>483</v>
-      </c>
-      <c r="BJ3" s="9" t="s">
+      <c r="BR3" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="BK3" s="9" t="s">
-        <v>458</v>
-      </c>
-      <c r="BL3" s="9" t="s">
-        <v>457</v>
-      </c>
-      <c r="BM3" s="9" t="s">
+      <c r="BS3" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="BN3" s="9" t="s">
+      <c r="BT3" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="BO3" s="9" t="s">
+      <c r="BU3" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="BP3" s="9" t="s">
+      <c r="BV3" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="BQ3" s="9" t="s">
+      <c r="BW3" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="BR3" s="9" t="s">
+      <c r="BX3" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="BS3" s="9" t="s">
+      <c r="BY3" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="BZ3" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="CA3" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="BT3" s="9" t="s">
+      <c r="CB3" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="BU3" s="9" t="s">
+      <c r="CC3" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="CD3" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="CE3" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="BV3" s="9" t="s">
+      <c r="CF3" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="CG3" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="CH3" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="CI3" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="CJ3" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="CK3" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="BW3" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="BX3" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="BY3" s="9" t="s">
-        <v>458</v>
-      </c>
-      <c r="BZ3" s="9" t="s">
-        <v>457</v>
-      </c>
-      <c r="CA3" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="CB3" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="CC3" s="9" t="s">
-        <v>244</v>
-      </c>
-      <c r="CD3" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="CE3" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="CF3" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="CG3" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="CH3" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="CI3" s="9" t="s">
-        <v>250</v>
-      </c>
-      <c r="CJ3" s="9" t="s">
-        <v>251</v>
-      </c>
-      <c r="CK3" s="9" t="s">
-        <v>257</v>
-      </c>
       <c r="CL3" s="9" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="CM3" s="9" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="CN3" s="9" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="CO3" s="9" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
     </row>
     <row r="4" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="D4" s="21">
         <v>10</v>
@@ -4798,10 +4902,10 @@
         <v>12</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="H4" s="21">
         <v>1</v>
@@ -4848,7 +4952,7 @@
         <v>6</v>
       </c>
       <c r="X4" s="24" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="Y4" s="24">
         <v>1</v>
@@ -4856,7 +4960,7 @@
       <c r="Z4" s="24"/>
       <c r="AA4" s="24"/>
       <c r="AB4" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AC4" s="24"/>
       <c r="AD4" s="21">
@@ -4872,19 +4976,19 @@
         <v>1</v>
       </c>
       <c r="AH4" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AI4" s="24"/>
       <c r="AJ4" s="24"/>
       <c r="AK4" s="24"/>
       <c r="AL4" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AM4" s="24"/>
       <c r="AN4" s="24"/>
       <c r="AO4" s="24"/>
       <c r="AP4" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AQ4" s="24"/>
       <c r="AR4" s="21">
@@ -4900,7 +5004,7 @@
         <v>4</v>
       </c>
       <c r="AV4" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AW4" s="24"/>
       <c r="AX4" s="24">
@@ -4910,7 +5014,7 @@
         <v>3</v>
       </c>
       <c r="AZ4" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="BA4" s="24"/>
       <c r="BB4" s="24">
@@ -4920,13 +5024,13 @@
         <v>5</v>
       </c>
       <c r="BD4" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="BE4" s="24"/>
       <c r="BF4" s="24"/>
       <c r="BG4" s="24"/>
       <c r="BH4" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="BI4" s="24"/>
       <c r="BJ4" s="21">
@@ -4971,7 +5075,7 @@
         <v>1</v>
       </c>
       <c r="BW4" s="21" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="BX4" s="10"/>
       <c r="BY4" s="21">
@@ -5006,13 +5110,13 @@
     </row>
     <row r="5" spans="1:93" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="D5" s="21">
         <v>10</v>
@@ -5022,7 +5126,7 @@
       </c>
       <c r="F5" s="10"/>
       <c r="G5" s="10" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="H5" s="21">
         <v>1</v>
@@ -5073,7 +5177,7 @@
         <v>6</v>
       </c>
       <c r="X5" s="24" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="Y5" s="24">
         <v>1</v>
@@ -5081,7 +5185,7 @@
       <c r="Z5" s="24"/>
       <c r="AA5" s="24"/>
       <c r="AB5" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AC5" s="24"/>
       <c r="AD5" s="21">
@@ -5097,19 +5201,19 @@
         <v>1</v>
       </c>
       <c r="AH5" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AI5" s="24"/>
       <c r="AJ5" s="24"/>
       <c r="AK5" s="24"/>
       <c r="AL5" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AM5" s="24"/>
       <c r="AN5" s="24"/>
       <c r="AO5" s="24"/>
       <c r="AP5" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AQ5" s="24"/>
       <c r="AR5" s="21">
@@ -5125,7 +5229,7 @@
         <v>4</v>
       </c>
       <c r="AV5" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AW5" s="24"/>
       <c r="AX5" s="24">
@@ -5135,7 +5239,7 @@
         <v>3</v>
       </c>
       <c r="AZ5" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="BA5" s="24"/>
       <c r="BB5" s="24">
@@ -5145,13 +5249,13 @@
         <v>5</v>
       </c>
       <c r="BD5" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="BE5" s="24"/>
       <c r="BF5" s="24"/>
       <c r="BG5" s="24"/>
       <c r="BH5" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="BI5" s="24"/>
       <c r="BJ5" s="21">
@@ -5196,16 +5300,16 @@
         <v>1</v>
       </c>
       <c r="BW5" s="21" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="BX5" s="21">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="BY5" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BZ5" s="21">
-        <v>-2.5</v>
+        <v>-1.5</v>
       </c>
       <c r="CA5" s="5">
         <f>AR5</f>
@@ -5215,12 +5319,12 @@
         <v>11.88</v>
       </c>
       <c r="CC5" s="21">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="CD5" s="21">
-        <v>2</v>
-      </c>
-      <c r="CE5" s="21">
+        <v>1</v>
+      </c>
+      <c r="CE5" s="5">
         <f>CB5</f>
         <v>11.88</v>
       </c>
@@ -5240,73 +5344,68 @@
         <v>1</v>
       </c>
       <c r="CK5" s="21" t="s">
-        <v>259</v>
-      </c>
-      <c r="CL5" s="21">
-        <v>1</v>
-      </c>
-      <c r="CM5" s="21">
-        <v>2</v>
-      </c>
-      <c r="CN5" s="21">
-        <v>0</v>
-      </c>
-      <c r="CO5" s="21">
-        <v>15</v>
-      </c>
+        <v>253</v>
+      </c>
+      <c r="CL5" s="21"/>
+      <c r="CM5" s="21"/>
+      <c r="CN5" s="21"/>
+      <c r="CO5" s="21"/>
     </row>
     <row r="6" spans="1:93" x14ac:dyDescent="0.25">
       <c r="F6" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="AE6" s="19"/>
       <c r="AS6" s="19"/>
+      <c r="BW6" t="s">
+        <v>495</v>
+      </c>
       <c r="BX6" s="19"/>
-      <c r="BY6" s="33"/>
-      <c r="BZ6" s="33"/>
+      <c r="BY6" s="28"/>
+      <c r="BZ6" s="28"/>
     </row>
     <row r="7" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="F7" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="BX7" s="19"/>
     </row>
     <row r="8" spans="1:93" ht="112.5" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:93" ht="90" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:93" ht="123.75" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:93" ht="90" x14ac:dyDescent="0.25">
       <c r="B12" s="6" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" spans="1:93" ht="101.25" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" spans="1:93" ht="90" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -5347,518 +5446,518 @@
   <sheetData>
     <row r="1" spans="1:37" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="67" t="s">
-        <v>269</v>
-      </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="53" t="s">
-        <v>452</v>
-      </c>
-      <c r="O1" s="73"/>
-      <c r="P1" s="54"/>
-      <c r="Q1" s="54"/>
-      <c r="R1" s="54"/>
-      <c r="S1" s="54"/>
-      <c r="T1" s="43" t="s">
-        <v>270</v>
-      </c>
-      <c r="U1" s="40"/>
-      <c r="V1" s="40"/>
-      <c r="W1" s="41"/>
-      <c r="X1" s="70" t="s">
-        <v>271</v>
-      </c>
-      <c r="Y1" s="71"/>
-      <c r="Z1" s="71"/>
-      <c r="AA1" s="71"/>
-      <c r="AB1" s="71"/>
-      <c r="AC1" s="71"/>
-      <c r="AD1" s="71"/>
-      <c r="AE1" s="72"/>
-      <c r="AF1" s="64" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG1" s="65"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="68" t="s">
-        <v>273</v>
-      </c>
-      <c r="AJ1" s="69"/>
-      <c r="AK1" s="69"/>
+        <v>19</v>
+      </c>
+      <c r="B1" s="68" t="s">
+        <v>263</v>
+      </c>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="51" t="s">
+        <v>446</v>
+      </c>
+      <c r="O1" s="74"/>
+      <c r="P1" s="52"/>
+      <c r="Q1" s="52"/>
+      <c r="R1" s="52"/>
+      <c r="S1" s="52"/>
+      <c r="T1" s="44" t="s">
+        <v>264</v>
+      </c>
+      <c r="U1" s="41"/>
+      <c r="V1" s="41"/>
+      <c r="W1" s="42"/>
+      <c r="X1" s="71" t="s">
+        <v>265</v>
+      </c>
+      <c r="Y1" s="72"/>
+      <c r="Z1" s="72"/>
+      <c r="AA1" s="72"/>
+      <c r="AB1" s="72"/>
+      <c r="AC1" s="72"/>
+      <c r="AD1" s="72"/>
+      <c r="AE1" s="73"/>
+      <c r="AF1" s="65" t="s">
+        <v>266</v>
+      </c>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="67"/>
+      <c r="AI1" s="69" t="s">
+        <v>267</v>
+      </c>
+      <c r="AJ1" s="70"/>
+      <c r="AK1" s="70"/>
     </row>
     <row r="2" spans="1:37" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>468</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>473</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>474</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>475</v>
-      </c>
       <c r="I2" s="3" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="L2" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="AB2" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="AC2" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="AD2" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="AE2" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="N2" s="3" t="s">
-        <v>484</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>493</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>485</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>487</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>453</v>
-      </c>
-      <c r="T2" s="3" t="s">
+      <c r="AF2" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="AG2" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="V2" s="3" t="s">
+      <c r="AH2" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="W2" s="3" t="s">
+      <c r="AI2" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="X2" s="3" t="s">
-        <v>444</v>
-      </c>
-      <c r="Y2" s="3" t="s">
-        <v>445</v>
-      </c>
-      <c r="Z2" s="3" t="s">
-        <v>446</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>447</v>
-      </c>
-      <c r="AB2" s="3" t="s">
-        <v>448</v>
-      </c>
-      <c r="AC2" s="3" t="s">
-        <v>449</v>
-      </c>
-      <c r="AD2" s="3" t="s">
+      <c r="AJ2" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="AE2" s="3" t="s">
+      <c r="AK2" s="3" t="s">
         <v>281</v>
-      </c>
-      <c r="AF2" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="AG2" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="AH2" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="AI2" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="AJ2" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="AK2" s="3" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="3" spans="1:37" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>460</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>461</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>465</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>464</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>456</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>457</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>471</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>472</v>
+      </c>
+      <c r="J3" s="9" t="s">
         <v>466</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>467</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>471</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>470</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>462</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>463</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>477</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>478</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>472</v>
-      </c>
       <c r="K3" s="9" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="L3" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>482</v>
+      </c>
+      <c r="O3" s="9" t="s">
+        <v>483</v>
+      </c>
+      <c r="P3" s="9" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q3" s="9" t="s">
+        <v>485</v>
+      </c>
+      <c r="R3" s="9" t="s">
+        <v>486</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>448</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="U3" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="V3" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="W3" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="X3" s="9" t="s">
+        <v>444</v>
+      </c>
+      <c r="Y3" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="Z3" s="9" t="s">
         <v>289</v>
       </c>
-      <c r="N3" s="9" t="s">
-        <v>488</v>
-      </c>
-      <c r="O3" s="9" t="s">
-        <v>489</v>
-      </c>
-      <c r="P3" s="9" t="s">
-        <v>490</v>
-      </c>
-      <c r="Q3" s="9" t="s">
-        <v>491</v>
-      </c>
-      <c r="R3" s="9" t="s">
-        <v>492</v>
-      </c>
-      <c r="S3" s="9" t="s">
-        <v>454</v>
-      </c>
-      <c r="T3" s="9" t="s">
+      <c r="AA3" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="AB3" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="AC3" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="AD3" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="U3" s="9" t="s">
+      <c r="AE3" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="V3" s="9" t="s">
+      <c r="AF3" s="9" t="s">
         <v>292</v>
       </c>
-      <c r="W3" s="9" t="s">
+      <c r="AG3" s="9" t="s">
         <v>293</v>
       </c>
-      <c r="X3" s="9" t="s">
-        <v>450</v>
-      </c>
-      <c r="Y3" s="9" t="s">
+      <c r="AH3" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="Z3" s="9" t="s">
+      <c r="AI3" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="AJ3" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="AK3" s="9" t="s">
         <v>295</v>
-      </c>
-      <c r="AA3" s="9" t="s">
-        <v>451</v>
-      </c>
-      <c r="AB3" s="9" t="s">
-        <v>294</v>
-      </c>
-      <c r="AC3" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="AD3" s="9" t="s">
-        <v>296</v>
-      </c>
-      <c r="AE3" s="9" t="s">
-        <v>297</v>
-      </c>
-      <c r="AF3" s="9" t="s">
-        <v>298</v>
-      </c>
-      <c r="AG3" s="9" t="s">
-        <v>299</v>
-      </c>
-      <c r="AH3" s="9" t="s">
-        <v>300</v>
-      </c>
-      <c r="AI3" s="25" t="s">
-        <v>317</v>
-      </c>
-      <c r="AJ3" s="9" t="s">
-        <v>296</v>
-      </c>
-      <c r="AK3" s="9" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:37" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="B4" s="32">
+        <v>119</v>
+      </c>
+      <c r="B4" s="27">
         <v>1</v>
       </c>
-      <c r="C4" s="32">
+      <c r="C4" s="27">
         <v>1</v>
       </c>
-      <c r="D4" s="32">
+      <c r="D4" s="27">
         <v>1</v>
       </c>
-      <c r="E4" s="32">
+      <c r="E4" s="27">
         <v>1</v>
       </c>
-      <c r="F4" s="32">
+      <c r="F4" s="27">
         <v>1</v>
       </c>
-      <c r="G4" s="32">
+      <c r="G4" s="27">
         <v>1</v>
       </c>
-      <c r="H4" s="32">
+      <c r="H4" s="27">
         <v>1</v>
       </c>
-      <c r="I4" s="32">
+      <c r="I4" s="27">
         <v>1</v>
       </c>
-      <c r="J4" s="32">
+      <c r="J4" s="27">
         <v>1</v>
       </c>
-      <c r="K4" s="32">
+      <c r="K4" s="27">
         <v>1</v>
       </c>
-      <c r="L4" s="32">
+      <c r="L4" s="27">
         <v>1</v>
       </c>
-      <c r="M4" s="32">
+      <c r="M4" s="27">
         <v>1</v>
       </c>
-      <c r="N4" s="32">
+      <c r="N4" s="27">
         <v>1</v>
       </c>
-      <c r="O4" s="32">
+      <c r="O4" s="27">
         <v>1</v>
       </c>
-      <c r="P4" s="32">
+      <c r="P4" s="27">
         <v>1</v>
       </c>
-      <c r="Q4" s="32">
+      <c r="Q4" s="27">
         <v>1</v>
       </c>
-      <c r="R4" s="32">
+      <c r="R4" s="27">
         <v>1</v>
       </c>
-      <c r="S4" s="32">
+      <c r="S4" s="27">
         <v>1</v>
       </c>
-      <c r="T4" s="32" t="s">
-        <v>259</v>
-      </c>
-      <c r="U4" s="32"/>
-      <c r="V4" s="32"/>
-      <c r="W4" s="32"/>
-      <c r="X4" s="32" t="s">
-        <v>259</v>
-      </c>
-      <c r="Y4" s="32">
+      <c r="T4" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="U4" s="27"/>
+      <c r="V4" s="27"/>
+      <c r="W4" s="27"/>
+      <c r="X4" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y4" s="27">
         <v>5</v>
       </c>
-      <c r="Z4" s="32">
+      <c r="Z4" s="27">
         <v>0</v>
       </c>
-      <c r="AA4" s="32" t="s">
-        <v>259</v>
-      </c>
-      <c r="AB4" s="32">
+      <c r="AA4" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="AB4" s="27">
         <v>5</v>
       </c>
-      <c r="AC4" s="32">
+      <c r="AC4" s="27">
         <v>0</v>
       </c>
-      <c r="AD4" s="32">
+      <c r="AD4" s="27">
         <v>1.8</v>
       </c>
-      <c r="AE4" s="32">
+      <c r="AE4" s="27">
         <v>30</v>
       </c>
-      <c r="AF4" s="32" t="s">
-        <v>259</v>
-      </c>
-      <c r="AG4" s="32"/>
-      <c r="AH4" s="32"/>
-      <c r="AI4" s="32" t="s">
-        <v>259</v>
-      </c>
-      <c r="AJ4" s="32"/>
-      <c r="AK4" s="32"/>
+      <c r="AF4" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG4" s="27"/>
+      <c r="AH4" s="27"/>
+      <c r="AI4" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ4" s="27"/>
+      <c r="AK4" s="27"/>
     </row>
     <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="32">
+        <v>50</v>
+      </c>
+      <c r="B5" s="27">
         <v>2</v>
       </c>
-      <c r="C5" s="32">
+      <c r="C5" s="27">
         <v>2</v>
       </c>
-      <c r="D5" s="32">
+      <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" s="32">
+      <c r="E5" s="27">
         <v>2</v>
       </c>
-      <c r="F5" s="32">
+      <c r="F5" s="27">
         <v>1</v>
       </c>
-      <c r="G5" s="32">
+      <c r="G5" s="27">
         <v>1</v>
       </c>
-      <c r="H5" s="32">
+      <c r="H5" s="27">
         <v>1</v>
       </c>
-      <c r="I5" s="32">
+      <c r="I5" s="27">
         <v>1</v>
       </c>
-      <c r="J5" s="32">
+      <c r="J5" s="27">
         <v>1</v>
       </c>
-      <c r="K5" s="32">
+      <c r="K5" s="27">
         <v>1</v>
       </c>
-      <c r="L5" s="32">
+      <c r="L5" s="27">
         <v>1</v>
       </c>
-      <c r="M5" s="32">
+      <c r="M5" s="27">
         <v>1</v>
       </c>
-      <c r="N5" s="32">
+      <c r="N5" s="27">
         <v>1</v>
       </c>
-      <c r="O5" s="32">
+      <c r="O5" s="27">
         <v>1</v>
       </c>
-      <c r="P5" s="32">
+      <c r="P5" s="27">
         <v>1</v>
       </c>
-      <c r="Q5" s="32">
+      <c r="Q5" s="27">
         <v>1</v>
       </c>
-      <c r="R5" s="32">
+      <c r="R5" s="27">
         <v>1</v>
       </c>
-      <c r="S5" s="32">
+      <c r="S5" s="27">
         <v>1</v>
       </c>
-      <c r="T5" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="U5" s="32">
+      <c r="T5" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="U5" s="27">
         <v>4</v>
       </c>
-      <c r="V5" s="32">
+      <c r="V5" s="27">
         <v>0</v>
       </c>
-      <c r="W5" s="32">
+      <c r="W5" s="27">
         <v>2</v>
       </c>
-      <c r="X5" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="Y5" s="32">
+      <c r="X5" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="Y5" s="27">
         <v>5</v>
       </c>
-      <c r="Z5" s="32">
+      <c r="Z5" s="27">
         <v>0</v>
       </c>
-      <c r="AA5" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="AB5" s="32">
+      <c r="AA5" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="AB5" s="27">
         <v>5</v>
       </c>
-      <c r="AC5" s="32">
+      <c r="AC5" s="27">
         <v>0</v>
       </c>
-      <c r="AD5" s="32">
+      <c r="AD5" s="27">
         <v>1.8</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="27">
         <v>30</v>
       </c>
-      <c r="AF5" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="AG5" s="32">
+      <c r="AF5" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="AG5" s="27">
         <v>5</v>
       </c>
-      <c r="AH5" s="32">
+      <c r="AH5" s="27">
         <v>4</v>
       </c>
-      <c r="AI5" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="AJ5" s="32">
+      <c r="AI5" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="AJ5" s="27">
         <v>2</v>
       </c>
-      <c r="AK5" s="32">
+      <c r="AK5" s="27">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:37" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:37" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8" spans="1:37" ht="123.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" spans="1:37" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
     </row>
     <row r="10" spans="1:37" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -5884,7 +5983,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5892,32 +5991,32 @@
     </row>
     <row r="3" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5925,22 +6024,22 @@
     </row>
     <row r="10" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5948,27 +6047,27 @@
     </row>
     <row r="15" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5976,52 +6075,52 @@
     </row>
     <row r="21" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
@@ -6029,92 +6128,92 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
@@ -6122,92 +6221,92 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>365</v>
+        <v>359</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
@@ -6215,112 +6314,112 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="14" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="14" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="14" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="14" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="14" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="14" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="14" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="14" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="14" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="14" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="14" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="14" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="14" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
@@ -6328,87 +6427,87 @@
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="14" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="14" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="14" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="14" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="14" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="14" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="14" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="14" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="14" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="14" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="14" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
@@ -6416,27 +6515,27 @@
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="15" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Module 3 part 1 seems to work properly. Pads need to be separated
</commit_message>
<xml_diff>
--- a/seismic_input.xlsx
+++ b/seismic_input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Create_mct_bear_seismo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B5CE8E-F159-401C-A32B-C1E7C6C5A4A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A0A206-9E39-43B3-8AA7-1A1C3F960913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2069,6 +2069,11 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2084,11 +2089,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3248,17 +3248,17 @@
       <c r="L1" s="41"/>
       <c r="M1" s="41"/>
       <c r="N1" s="42"/>
-      <c r="O1" s="51" t="s">
+      <c r="O1" s="54" t="s">
         <v>54</v>
       </c>
-      <c r="P1" s="52"/>
-      <c r="Q1" s="52"/>
-      <c r="R1" s="52"/>
-      <c r="S1" s="52"/>
-      <c r="T1" s="52"/>
-      <c r="U1" s="52"/>
-      <c r="V1" s="52"/>
-      <c r="W1" s="53"/>
+      <c r="P1" s="55"/>
+      <c r="Q1" s="55"/>
+      <c r="R1" s="55"/>
+      <c r="S1" s="55"/>
+      <c r="T1" s="55"/>
+      <c r="U1" s="55"/>
+      <c r="V1" s="55"/>
+      <c r="W1" s="56"/>
       <c r="X1" s="40" t="s">
         <v>55</v>
       </c>
@@ -3271,17 +3271,17 @@
       <c r="AE1" s="41"/>
       <c r="AF1" s="41"/>
       <c r="AG1" s="42"/>
-      <c r="AH1" s="48" t="s">
+      <c r="AH1" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="AI1" s="49"/>
-      <c r="AJ1" s="49"/>
-      <c r="AK1" s="49"/>
-      <c r="AL1" s="49"/>
-      <c r="AM1" s="49"/>
-      <c r="AN1" s="49"/>
-      <c r="AO1" s="49"/>
-      <c r="AP1" s="50"/>
+      <c r="AI1" s="52"/>
+      <c r="AJ1" s="52"/>
+      <c r="AK1" s="52"/>
+      <c r="AL1" s="52"/>
+      <c r="AM1" s="52"/>
+      <c r="AN1" s="52"/>
+      <c r="AO1" s="52"/>
+      <c r="AP1" s="53"/>
     </row>
     <row r="2" spans="1:42" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
@@ -3293,69 +3293,69 @@
       <c r="E2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F2" s="54" t="s">
+      <c r="F2" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="G2" s="55"/>
-      <c r="H2" s="56"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="47"/>
       <c r="I2" s="44" t="s">
         <v>60</v>
       </c>
       <c r="J2" s="41"/>
       <c r="K2" s="42"/>
-      <c r="L2" s="45" t="s">
+      <c r="L2" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="M2" s="46"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="54" t="s">
+      <c r="M2" s="49"/>
+      <c r="N2" s="50"/>
+      <c r="O2" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="P2" s="55"/>
-      <c r="Q2" s="56"/>
+      <c r="P2" s="46"/>
+      <c r="Q2" s="47"/>
       <c r="R2" s="44" t="s">
         <v>63</v>
       </c>
       <c r="S2" s="41"/>
       <c r="T2" s="42"/>
-      <c r="U2" s="45" t="s">
+      <c r="U2" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="V2" s="46"/>
-      <c r="W2" s="47"/>
+      <c r="V2" s="49"/>
+      <c r="W2" s="50"/>
       <c r="X2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="Y2" s="54" t="s">
+      <c r="Y2" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="Z2" s="55"/>
-      <c r="AA2" s="56"/>
+      <c r="Z2" s="46"/>
+      <c r="AA2" s="47"/>
       <c r="AB2" s="44" t="s">
         <v>60</v>
       </c>
       <c r="AC2" s="41"/>
       <c r="AD2" s="42"/>
-      <c r="AE2" s="45" t="s">
+      <c r="AE2" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="AF2" s="46"/>
-      <c r="AG2" s="47"/>
-      <c r="AH2" s="54" t="s">
+      <c r="AF2" s="49"/>
+      <c r="AG2" s="50"/>
+      <c r="AH2" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="AI2" s="55"/>
-      <c r="AJ2" s="56"/>
+      <c r="AI2" s="46"/>
+      <c r="AJ2" s="47"/>
       <c r="AK2" s="44" t="s">
         <v>63</v>
       </c>
       <c r="AL2" s="41"/>
       <c r="AM2" s="42"/>
-      <c r="AN2" s="45" t="s">
+      <c r="AN2" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="AO2" s="46"/>
-      <c r="AP2" s="47"/>
+      <c r="AO2" s="49"/>
+      <c r="AP2" s="50"/>
     </row>
     <row r="3" spans="1:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -4176,11 +4176,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="E1:N1"/>
-    <mergeCell ref="A9:D9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="AE2:AG2"/>
     <mergeCell ref="AH1:AP1"/>
@@ -4196,6 +4191,11 @@
     <mergeCell ref="AB2:AD2"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="Y2:AA2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="E1:N1"/>
+    <mergeCell ref="A9:D9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -5306,10 +5306,10 @@
         <v>1</v>
       </c>
       <c r="BY5" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BZ5" s="21">
-        <v>-1.5</v>
+        <v>-2.5</v>
       </c>
       <c r="CA5" s="5">
         <f>AR5</f>
@@ -5462,14 +5462,14 @@
       <c r="K1" s="41"/>
       <c r="L1" s="41"/>
       <c r="M1" s="41"/>
-      <c r="N1" s="51" t="s">
+      <c r="N1" s="54" t="s">
         <v>446</v>
       </c>
       <c r="O1" s="74"/>
-      <c r="P1" s="52"/>
-      <c r="Q1" s="52"/>
-      <c r="R1" s="52"/>
-      <c r="S1" s="52"/>
+      <c r="P1" s="55"/>
+      <c r="Q1" s="55"/>
+      <c r="R1" s="55"/>
+      <c r="S1" s="55"/>
       <c r="T1" s="44" t="s">
         <v>264</v>
       </c>

</xml_diff>